<commit_message>
Fix: supprimer drapeau header, lier groupes→partis, exclure Marcel Dobler et Baume-Schneider (CF)
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -590,12 +590,51 @@
     <t xml:space="preserve">Finanze</t>
   </si>
   <si>
+    <t xml:space="preserve">25.4794</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-12-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGOV und E-ID. Die Authentifizierung bei Bundes-Applikationen soll vereinheitlicht werden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agov et e-ID. L'authentification pour les applications fédérales doit être uniformisée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGOV ed Id-e. L'autenticazione nelle applicazioni federali deve essere uniformata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;AGOV est un service d’authentification standardisé pour les services numériques de la Confédération, des cantons et des communes. La loi sur l’e-ID ayant été adoptée, une nouvelle possibilité de vérifier l’identité existera pour accéder à une application administrative.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Les départements ont actuellement des opinions divergentes quant à l’utilisation de ces possibilités d’authentification. En effet, les coûts liés à la vérification d’identité (p.&amp;nbsp;ex.&amp;nbsp;pour AGOV&amp;nbsp;400) sont à la charge du gestionnaire de l’application administrative, tandis que l’e-ID pourra être utilisée sans coûts supplémentaires. Si ces coûts ne sont pas pris en charge, il y aura de facto une obligation d’utiliser l’e-ID, ce qu’il convient d’éviter en uniformisant l’authentification pour les applications fédérales.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Le Conseil fédéral doit déterminer comment AGOV et l’e-ID devront être utilisés de manière uniforme dans tous les départements s’agissant de l’authentification dans les applications fédérales.&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Il doit décider que l’utilisation de l’e-ID restera facultative et que toutes les applications fédérales offriront également la possibilité d’une authentification au moyen d’AGOV.&amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Les coûts liés à la vérification d’identité sont à la charge des gestionnaires des applications fédérales.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;AGOV ist ein standardisierter Authentifizierungsdienst für digitale Angebote von Bund, Kantonen und Gemeinden. Wenn für den Zugriff auf eine Behörden-Applikation eine Identitätsprüfung erforderlich ist, steht seit der Annahme des e-ID Gesetzes eine neue Möglichkeit zur Identitätsüberprüfung zur Verfügung.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Die verschiedenen Departemente haben aktuell unterschiedliche Auffassungen über die Verwendung dieser Authentifizierungsmöglichkeiten. Dies weil die Kosten der Identitätsüberprüfung&amp;nbsp;(z.B. für AGOV 400) vom Betreiber der Behörden-Applikation übernommen werden müssen, während die e-ID nach deren Einführung ohne Kostenfolge eingesetzt werden kann. Wenn diese Kosten der Identitätsüberprüfung nicht übernommen werden, führt dies zu einem faktischen e-ID-Zwang, den es zu verhindern gilt mit einer Vereinheitlichung der Authentifizierung bei Bundes-Applikationen:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Der Bundesrat hat festzulegen, wie AGOV und die e-ID einheitlich über alle Departemente hinweg bei den Bundes-Applikationen zur Authentifizierung genutzt werden sollen.&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Der Bundesrat hat festzulegen, dass die Verwendung der e-ID freiwillig bleibt und in allen Bundes-Applikationen auch die Möglichkeit der AGOV Authentifizierung angeboten werden muss.&amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Die Kosten der Identitätsüberprüfung sind von den Betreibern der Bundes-Applikationen zu übernehmen.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stellungnahme zum Vorstoss liegt vor / L’avis relatif à l’intervention est disponible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254794</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254794</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staatspolitik|Finanzwesen|Medien und Kommunikation|Menschenrechte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique d'Etat|Finances|Médias et communication|Droits de l'homme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica nazionale|Finanze|Media e comunicazione|Diritti umani</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.4774</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-12-19</t>
-  </si>
-  <si>
     <t xml:space="preserve">Gewalttätiger Extremismus bei Demonstrationen. Veranstalter sollen die Kosten übernehmen</t>
   </si>
   <si>
@@ -629,45 +668,6 @@
     <t xml:space="preserve">Politica nazionale|Politica di sicurezza|Questioni sociali</t>
   </si>
   <si>
-    <t xml:space="preserve">25.4794</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AGOV und E-ID. Die Authentifizierung bei Bundes-Applikationen soll vereinheitlicht werden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agov et e-ID. L'authentification pour les applications fédérales doit être uniformisée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AGOV ed Id-e. L'autenticazione nelle applicazioni federali deve essere uniformata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;AGOV est un service d’authentification standardisé pour les services numériques de la Confédération, des cantons et des communes. La loi sur l’e-ID ayant été adoptée, une nouvelle possibilité de vérifier l’identité existera pour accéder à une application administrative.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Les départements ont actuellement des opinions divergentes quant à l’utilisation de ces possibilités d’authentification. En effet, les coûts liés à la vérification d’identité (p.&amp;nbsp;ex.&amp;nbsp;pour AGOV&amp;nbsp;400) sont à la charge du gestionnaire de l’application administrative, tandis que l’e-ID pourra être utilisée sans coûts supplémentaires. Si ces coûts ne sont pas pris en charge, il y aura de facto une obligation d’utiliser l’e-ID, ce qu’il convient d’éviter en uniformisant l’authentification pour les applications fédérales.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Le Conseil fédéral doit déterminer comment AGOV et l’e-ID devront être utilisés de manière uniforme dans tous les départements s’agissant de l’authentification dans les applications fédérales.&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Il doit décider que l’utilisation de l’e-ID restera facultative et que toutes les applications fédérales offriront également la possibilité d’une authentification au moyen d’AGOV.&amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Les coûts liés à la vérification d’identité sont à la charge des gestionnaires des applications fédérales.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;AGOV ist ein standardisierter Authentifizierungsdienst für digitale Angebote von Bund, Kantonen und Gemeinden. Wenn für den Zugriff auf eine Behörden-Applikation eine Identitätsprüfung erforderlich ist, steht seit der Annahme des e-ID Gesetzes eine neue Möglichkeit zur Identitätsüberprüfung zur Verfügung.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Die verschiedenen Departemente haben aktuell unterschiedliche Auffassungen über die Verwendung dieser Authentifizierungsmöglichkeiten. Dies weil die Kosten der Identitätsüberprüfung&amp;nbsp;(z.B. für AGOV 400) vom Betreiber der Behörden-Applikation übernommen werden müssen, während die e-ID nach deren Einführung ohne Kostenfolge eingesetzt werden kann. Wenn diese Kosten der Identitätsüberprüfung nicht übernommen werden, führt dies zu einem faktischen e-ID-Zwang, den es zu verhindern gilt mit einer Vereinheitlichung der Authentifizierung bei Bundes-Applikationen:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Der Bundesrat hat festzulegen, wie AGOV und die e-ID einheitlich über alle Departemente hinweg bei den Bundes-Applikationen zur Authentifizierung genutzt werden sollen.&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Der Bundesrat hat festzulegen, dass die Verwendung der e-ID freiwillig bleibt und in allen Bundes-Applikationen auch die Möglichkeit der AGOV Authentifizierung angeboten werden muss.&amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Die Kosten der Identitätsüberprüfung sind von den Betreibern der Bundes-Applikationen zu übernehmen.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stellungnahme zum Vorstoss liegt vor / L’avis relatif à l’intervention est disponible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254794</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254794</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik|Finanzwesen|Medien und Kommunikation|Menschenrechte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat|Finances|Médias et communication|Droits de l'homme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale|Finanze|Media e comunicazione|Diritti umani</t>
-  </si>
-  <si>
     <t xml:space="preserve">25.4836</t>
   </si>
   <si>
@@ -890,15 +890,45 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254517</t>
   </si>
   <si>
+    <t xml:space="preserve">25.8270</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-12-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SRG-Sparprogramm November 2025. Ist Gebühren-Zuwachs berücksichtigt?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programme d’économies de la SSR en novembre 2025. La croissance en volume de la redevance a-t-elle été prise en compte ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;En novembre 2025, la SSR a annoncé son intention de réaliser 270 millions de francs d'économies. L’immigration engendre une hausse de 57&amp;nbsp;000 ménages en moyenne par an.&lt;br&gt;- Le Conseil fédéral peut-il confirmer que la hausse du volume de la redevance qui en découle pour la SSR, soit 170 millions de francs (sur dix ans) n’a pas été intégré au plan d’économies de 270&amp;nbsp;millions de francs&amp;nbsp;?&lt;br&gt;- &amp;nbsp;Dans la négative, à combien s’élèvent les économies potentielles, selon lui&amp;nbsp;?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Die SRG hat im November 2025 angekündet, dass sie 270 Mio. Franken einsparen will. Durch Zuwanderung wächst die Schweiz im Durchschnitt um 57'000 Haushalte pro Jahr.&lt;br&gt;- Kann der Bundesrat bestätigen, dass der dadurch entstehende Gebühren-Zuwachs der SRG von 170 Mio. Franken (in zehn Jahren) in diesem Sparbetrag von 270 Mio. Franken nicht enthalten ist?&lt;br&gt;- &amp;nbsp;Falls nein, wie hoch ist der einzusparende Betrag nach Ansicht des Bundesrats?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20258270</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20258270</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanzwesen|Medien und Kommunikation|Steuer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finances|Médias et communication|Fiscalité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanze|Media e comunicazione|Imposte</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.8254</t>
   </si>
   <si>
     <t xml:space="preserve">Alijaj Islam</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-12-10</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nationalen Finanzausgleich (NFA) im Bezug auf Sportschulen</t>
   </si>
   <si>
@@ -926,36 +956,6 @@
     <t xml:space="preserve">Finanze|Questioni sociali|Formazione</t>
   </si>
   <si>
-    <t xml:space="preserve">25.8270</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRG-Sparprogramm November 2025. Ist Gebühren-Zuwachs berücksichtigt?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Programme d’économies de la SSR en novembre 2025. La croissance en volume de la redevance a-t-elle été prise en compte ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;En novembre 2025, la SSR a annoncé son intention de réaliser 270 millions de francs d'économies. L’immigration engendre une hausse de 57&amp;nbsp;000 ménages en moyenne par an.&lt;br&gt;- Le Conseil fédéral peut-il confirmer que la hausse du volume de la redevance qui en découle pour la SSR, soit 170 millions de francs (sur dix ans) n’a pas été intégré au plan d’économies de 270&amp;nbsp;millions de francs&amp;nbsp;?&lt;br&gt;- &amp;nbsp;Dans la négative, à combien s’élèvent les économies potentielles, selon lui&amp;nbsp;?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Die SRG hat im November 2025 angekündet, dass sie 270 Mio. Franken einsparen will. Durch Zuwanderung wächst die Schweiz im Durchschnitt um 57'000 Haushalte pro Jahr.&lt;br&gt;- Kann der Bundesrat bestätigen, dass der dadurch entstehende Gebühren-Zuwachs der SRG von 170 Mio. Franken (in zehn Jahren) in diesem Sparbetrag von 270 Mio. Franken nicht enthalten ist?&lt;br&gt;- &amp;nbsp;Falls nein, wie hoch ist der einzusparende Betrag nach Ansicht des Bundesrats?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20258270</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20258270</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanzwesen|Medien und Kommunikation|Steuer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finances|Médias et communication|Fiscalité</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanze|Media e comunicazione|Imposte</t>
-  </si>
-  <si>
     <t xml:space="preserve">25.8286</t>
   </si>
   <si>
@@ -1019,15 +1019,48 @@
     <t xml:space="preserve">Politica nazionale|Cultura|Pianificazione territoriale e alloggi</t>
   </si>
   <si>
+    <t xml:space="preserve">25.4317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stärkung der Aufsicht über die SRG unter Wahrung der Programmautonomie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renforcer la surveillance de la SSR tout en préservant l'autonomie des programmes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rafforzare la vigilanza sulla SSR nel rispetto dell'autonomia in materia di programmi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de présenter une modification de la loi fédérale sur la radio et la télévision (LRTV) afin de soumettre la SSR à la haute surveillance financière du Contrôle fédéral des finances (CDF) sans porter atteinte à l’autonomie des programmes.&lt;/p&gt;&lt;p&gt;Il respectera les principes suivants :&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Garantir l’autonomie dans la conception des programmes visée à l’art. 93, al. 3, Cst.&lt;/p&gt;&lt;p&gt;L’indépendance de la SSR dans la conception des programmes et dans ses activités rédactionnelles restera entièrement garantie.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Éviter les doublons&lt;/p&gt;&lt;p&gt;La répartition des tâches entre l’OFCOM, le DETEC, l’organe de révision interne de la SSR et le CDF doit être clairement harmonisée et coordonnée, comme c’est le cas pour des entreprises comparables qui sont soumises à la surveillance du CDF (par ex. la Poste, Swisscom et les CFF). Il conviendra d’éviter les doublons lors des contrôles afin de maintenir l’efficacité du processus de contrôle. L’indépendance du CDF, telle qu’elle est définie dans la loi sur le Contrôle des finances, sera garantie en permanence.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Assurer une surveillance complémentaire par le CDF&lt;/p&gt;&lt;p&gt;La surveillance actuelle par le DETEC et l’OFCOM et le contrôle des états financiers selon le droit de la société anonyme seront maintenus sans être remplacés. Lors du contrôle, le CDF agira de manière complémentaire et ciblée et interviendra de manière autonome et indépendante là où sa position particulière et sa spécialisation (par ex. contrôles de l’économicité) lui permettent de créer une plus-value, comme c’est le cas par rapport aux révisions internes, quand il définit lui-même l’accent qu’il va mettre.&amp;nbsp;&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, eine Änderung des Bundesgesetzes über Radio und Fernsehen (RTVG) vorzulegen, damit die SRG der finanziellen Oberaufsicht der eidgenössischen Finanzkontrolle (EFK) ohne Beeinträchtigung der Programmautonomie, unterstellt wird.&lt;/p&gt;&lt;p&gt;Folgende Bedingungen sollen dabei berücksichtigt werden:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Programmautonomie gemäss Bundesverfassung (Art. 93 Abs. 3 BV):&lt;/p&gt;&lt;p&gt;Die Unabhängigkeit der SRG in der Programmgestaltung und redaktionellen Tätigkeit bleibt vollständig gewährleistet.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Vermeidung von Doppelspurigkeiten:&lt;/p&gt;&lt;p&gt;Die Aufgabenverteilung zwischen BAKOM, UVEK, interner Revision SRG und EFK ist klar abzustimmen und zu koordinieren, wie das bei vergleichbaren Unternehmen, welche der Aufsicht der EFK unterstehen (z.B. Post, Swisscom, SBB der Fall ist. Doppelspurigkeiten bei der Prüfung sollen vermieden werden, um den Prüfungsprozess effizient zu halten. Die Unabhängigkeit der EFK gemäss Finanzkontrollgesetz bleibt hierbei jederzeit gewahrt.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Ergänzende Aufsicht durch die EFK:&lt;/p&gt;&lt;p&gt;Die bestehende Aufsicht durch UVEK/BAKOM und die aktienrechtliche Abschlussprüfung bleiben erhalten und werden nicht ersetzt. Die EFK wirkt bei der Prüfung gezielt ergänzend und wird selbständig und unabhängig dort eingesetzt, wo sie durch ihre Sonderstellung und Spezialisierung (z.B. Wirtschaftlichkeitsprüfungen) einen Mehrwert schaffen kann, wie zum Beispiel gegenüber internen Revisionen wo der Fokus selbst definiert wird.&amp;nbsp;&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanzwesen|Medien und Kommunikation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finances|Médias et communication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanze|Media e comunicazione</t>
+  </si>
+  <si>
     <t xml:space="preserve">25.4263</t>
   </si>
   <si>
     <t xml:space="preserve">Germann Hannes</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-09-26</t>
-  </si>
-  <si>
     <t xml:space="preserve">Vollumfänglicher Abzug der Krankenversicherungsprämien von der direkten Bundessteuer</t>
   </si>
   <si>
@@ -1056,39 +1089,6 @@
   </si>
   <si>
     <t xml:space="preserve">Imposte|Salute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.4317</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stärkung der Aufsicht über die SRG unter Wahrung der Programmautonomie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renforcer la surveillance de la SSR tout en préservant l'autonomie des programmes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rafforzare la vigilanza sulla SSR nel rispetto dell'autonomia in materia di programmi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de présenter une modification de la loi fédérale sur la radio et la télévision (LRTV) afin de soumettre la SSR à la haute surveillance financière du Contrôle fédéral des finances (CDF) sans porter atteinte à l’autonomie des programmes.&lt;/p&gt;&lt;p&gt;Il respectera les principes suivants :&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Garantir l’autonomie dans la conception des programmes visée à l’art. 93, al. 3, Cst.&lt;/p&gt;&lt;p&gt;L’indépendance de la SSR dans la conception des programmes et dans ses activités rédactionnelles restera entièrement garantie.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Éviter les doublons&lt;/p&gt;&lt;p&gt;La répartition des tâches entre l’OFCOM, le DETEC, l’organe de révision interne de la SSR et le CDF doit être clairement harmonisée et coordonnée, comme c’est le cas pour des entreprises comparables qui sont soumises à la surveillance du CDF (par ex. la Poste, Swisscom et les CFF). Il conviendra d’éviter les doublons lors des contrôles afin de maintenir l’efficacité du processus de contrôle. L’indépendance du CDF, telle qu’elle est définie dans la loi sur le Contrôle des finances, sera garantie en permanence.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Assurer une surveillance complémentaire par le CDF&lt;/p&gt;&lt;p&gt;La surveillance actuelle par le DETEC et l’OFCOM et le contrôle des états financiers selon le droit de la société anonyme seront maintenus sans être remplacés. Lors du contrôle, le CDF agira de manière complémentaire et ciblée et interviendra de manière autonome et indépendante là où sa position particulière et sa spécialisation (par ex. contrôles de l’économicité) lui permettent de créer une plus-value, comme c’est le cas par rapport aux révisions internes, quand il définit lui-même l’accent qu’il va mettre.&amp;nbsp;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, eine Änderung des Bundesgesetzes über Radio und Fernsehen (RTVG) vorzulegen, damit die SRG der finanziellen Oberaufsicht der eidgenössischen Finanzkontrolle (EFK) ohne Beeinträchtigung der Programmautonomie, unterstellt wird.&lt;/p&gt;&lt;p&gt;Folgende Bedingungen sollen dabei berücksichtigt werden:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Programmautonomie gemäss Bundesverfassung (Art. 93 Abs. 3 BV):&lt;/p&gt;&lt;p&gt;Die Unabhängigkeit der SRG in der Programmgestaltung und redaktionellen Tätigkeit bleibt vollständig gewährleistet.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Vermeidung von Doppelspurigkeiten:&lt;/p&gt;&lt;p&gt;Die Aufgabenverteilung zwischen BAKOM, UVEK, interner Revision SRG und EFK ist klar abzustimmen und zu koordinieren, wie das bei vergleichbaren Unternehmen, welche der Aufsicht der EFK unterstehen (z.B. Post, Swisscom, SBB der Fall ist. Doppelspurigkeiten bei der Prüfung sollen vermieden werden, um den Prüfungsprozess effizient zu halten. Die Unabhängigkeit der EFK gemäss Finanzkontrollgesetz bleibt hierbei jederzeit gewahrt.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Ergänzende Aufsicht durch die EFK:&lt;/p&gt;&lt;p&gt;Die bestehende Aufsicht durch UVEK/BAKOM und die aktienrechtliche Abschlussprüfung bleiben erhalten und werden nicht ersetzt. Die EFK wirkt bei der Prüfung gezielt ergänzend und wird selbständig und unabhängig dort eingesetzt, wo sie durch ihre Sonderstellung und Spezialisierung (z.B. Wirtschaftlichkeitsprüfungen) einen Mehrwert schaffen kann, wie zum Beispiel gegenüber internen Revisionen wo der Fokus selbst definiert wird.&amp;nbsp;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254317</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254317</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanzwesen|Medien und Kommunikation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finances|Médias et communication</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanze|Media e comunicazione</t>
   </si>
   <si>
     <t xml:space="preserve">25.4320</t>
@@ -5975,7 +5975,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>20254774</v>
+        <v>20254794</v>
       </c>
       <c r="B17" t="s">
         <v>192</v>
@@ -5984,55 +5984,55 @@
         <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>93</v>
+        <v>121</v>
       </c>
       <c r="E17" t="s">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="F17" t="s">
         <v>193</v>
       </c>
       <c r="G17" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="H17" t="s">
-        <v>146</v>
+        <v>194</v>
       </c>
       <c r="I17" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="J17" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="K17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="L17" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="M17" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="N17" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="O17" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="P17" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="Q17" t="s">
         <v>47</v>
       </c>
       <c r="R17" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S17" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="T17" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="U17" t="s">
         <v>37</v>
@@ -6040,28 +6040,28 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>20254794</v>
+        <v>20254774</v>
       </c>
       <c r="B18" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C18" t="s">
         <v>22</v>
       </c>
       <c r="D18" t="s">
-        <v>121</v>
+        <v>93</v>
       </c>
       <c r="E18" t="s">
-        <v>122</v>
+        <v>94</v>
       </c>
       <c r="F18" t="s">
         <v>193</v>
       </c>
       <c r="G18" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H18" t="s">
-        <v>206</v>
+        <v>146</v>
       </c>
       <c r="I18" t="s">
         <v>207</v>
@@ -6144,7 +6144,7 @@
         <v>225</v>
       </c>
       <c r="N19" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O19" t="s">
         <v>226</v>
@@ -6209,7 +6209,7 @@
         <v>239</v>
       </c>
       <c r="N20" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O20" t="s">
         <v>240</v>
@@ -6274,7 +6274,7 @@
         <v>252</v>
       </c>
       <c r="N21" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="O21" t="s">
         <v>253</v>
@@ -6469,7 +6469,7 @@
         <v>289</v>
       </c>
       <c r="N24" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O24" t="s">
         <v>290</v>
@@ -6495,7 +6495,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>20258254</v>
+        <v>20258270</v>
       </c>
       <c r="B25" t="s">
         <v>292</v>
@@ -6504,53 +6504,53 @@
         <v>120</v>
       </c>
       <c r="D25" t="s">
+        <v>121</v>
+      </c>
+      <c r="E25" t="s">
+        <v>122</v>
+      </c>
+      <c r="F25" t="s">
         <v>293</v>
-      </c>
-      <c r="E25" t="s">
-        <v>40</v>
-      </c>
-      <c r="F25" t="s">
-        <v>294</v>
       </c>
       <c r="G25" t="s">
         <v>25</v>
       </c>
       <c r="H25" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="I25" t="s">
+        <v>294</v>
+      </c>
+      <c r="J25" t="s">
         <v>295</v>
-      </c>
-      <c r="J25" t="s">
-        <v>296</v>
       </c>
       <c r="K25"/>
       <c r="L25" t="s">
+        <v>296</v>
+      </c>
+      <c r="M25" t="s">
         <v>297</v>
-      </c>
-      <c r="M25" t="s">
-        <v>298</v>
       </c>
       <c r="N25" t="s">
         <v>129</v>
       </c>
       <c r="O25" t="s">
+        <v>298</v>
+      </c>
+      <c r="P25" t="s">
         <v>299</v>
       </c>
-      <c r="P25" t="s">
+      <c r="Q25" t="s">
+        <v>47</v>
+      </c>
+      <c r="R25" t="s">
         <v>300</v>
       </c>
-      <c r="Q25" t="s">
-        <v>33</v>
-      </c>
-      <c r="R25" t="s">
+      <c r="S25" t="s">
         <v>301</v>
       </c>
-      <c r="S25" t="s">
+      <c r="T25" t="s">
         <v>302</v>
-      </c>
-      <c r="T25" t="s">
-        <v>303</v>
       </c>
       <c r="U25" t="s">
         <v>37</v>
@@ -6558,28 +6558,28 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>20258270</v>
+        <v>20258254</v>
       </c>
       <c r="B26" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C26" t="s">
         <v>120</v>
       </c>
       <c r="D26" t="s">
-        <v>121</v>
+        <v>304</v>
       </c>
       <c r="E26" t="s">
-        <v>122</v>
+        <v>40</v>
       </c>
       <c r="F26" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G26" t="s">
         <v>25</v>
       </c>
       <c r="H26" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="I26" t="s">
         <v>305</v>
@@ -6604,7 +6604,7 @@
         <v>310</v>
       </c>
       <c r="Q26" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="R26" t="s">
         <v>311</v>
@@ -6636,7 +6636,7 @@
         <v>54</v>
       </c>
       <c r="F27" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G27" t="s">
         <v>25</v>
@@ -6747,7 +6747,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>20254263</v>
+        <v>20254317</v>
       </c>
       <c r="B29" t="s">
         <v>335</v>
@@ -6756,55 +6756,55 @@
         <v>22</v>
       </c>
       <c r="D29" t="s">
+        <v>121</v>
+      </c>
+      <c r="E29" t="s">
+        <v>122</v>
+      </c>
+      <c r="F29" t="s">
         <v>336</v>
       </c>
-      <c r="E29" t="s">
-        <v>54</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
+        <v>25</v>
+      </c>
+      <c r="H29" t="s">
+        <v>234</v>
+      </c>
+      <c r="I29" t="s">
         <v>337</v>
       </c>
-      <c r="G29" t="s">
-        <v>41</v>
-      </c>
-      <c r="H29" t="s">
-        <v>124</v>
-      </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>338</v>
       </c>
-      <c r="J29" t="s">
+      <c r="K29" t="s">
         <v>339</v>
       </c>
-      <c r="K29" t="s">
+      <c r="L29" t="s">
         <v>340</v>
       </c>
-      <c r="L29" t="s">
+      <c r="M29" t="s">
         <v>341</v>
       </c>
-      <c r="M29" t="s">
+      <c r="N29" t="s">
+        <v>200</v>
+      </c>
+      <c r="O29" t="s">
         <v>342</v>
       </c>
-      <c r="N29" t="s">
-        <v>129</v>
-      </c>
-      <c r="O29" t="s">
+      <c r="P29" t="s">
         <v>343</v>
       </c>
-      <c r="P29" t="s">
+      <c r="Q29" t="s">
+        <v>47</v>
+      </c>
+      <c r="R29" t="s">
         <v>344</v>
       </c>
-      <c r="Q29" t="s">
-        <v>33</v>
-      </c>
-      <c r="R29" t="s">
+      <c r="S29" t="s">
         <v>345</v>
       </c>
-      <c r="S29" t="s">
+      <c r="T29" t="s">
         <v>346</v>
-      </c>
-      <c r="T29" t="s">
-        <v>347</v>
       </c>
       <c r="U29" t="s">
         <v>37</v>
@@ -6812,28 +6812,28 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>20254317</v>
+        <v>20254263</v>
       </c>
       <c r="B30" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C30" t="s">
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>121</v>
+        <v>348</v>
       </c>
       <c r="E30" t="s">
-        <v>122</v>
+        <v>54</v>
       </c>
       <c r="F30" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G30" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H30" t="s">
-        <v>234</v>
+        <v>124</v>
       </c>
       <c r="I30" t="s">
         <v>349</v>
@@ -6851,7 +6851,7 @@
         <v>353</v>
       </c>
       <c r="N30" t="s">
-        <v>212</v>
+        <v>129</v>
       </c>
       <c r="O30" t="s">
         <v>354</v>
@@ -6860,7 +6860,7 @@
         <v>355</v>
       </c>
       <c r="Q30" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="R30" t="s">
         <v>356</v>
@@ -6892,7 +6892,7 @@
         <v>74</v>
       </c>
       <c r="F31" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G31" t="s">
         <v>25</v>
@@ -6916,7 +6916,7 @@
         <v>365</v>
       </c>
       <c r="N31" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O31" t="s">
         <v>366</v>
@@ -6957,7 +6957,7 @@
         <v>40</v>
       </c>
       <c r="F32" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G32" t="s">
         <v>25</v>
@@ -6981,7 +6981,7 @@
         <v>373</v>
       </c>
       <c r="N32" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O32" t="s">
         <v>374</v>
@@ -7022,7 +7022,7 @@
         <v>40</v>
       </c>
       <c r="F33" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G33" t="s">
         <v>41</v>
@@ -7046,7 +7046,7 @@
         <v>381</v>
       </c>
       <c r="N33" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="O33" t="s">
         <v>382</v>
@@ -7241,7 +7241,7 @@
         <v>416</v>
       </c>
       <c r="N36" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O36" t="s">
         <v>417</v>
@@ -7436,7 +7436,7 @@
         <v>456</v>
       </c>
       <c r="N39" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O39" t="s">
         <v>457</v>
@@ -7753,7 +7753,7 @@
         <v>511</v>
       </c>
       <c r="N44" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O44" t="s">
         <v>512</v>
@@ -7877,7 +7877,7 @@
         <v>536</v>
       </c>
       <c r="N46" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="O46" t="s">
         <v>537</v>
@@ -7936,7 +7936,7 @@
         <v>546</v>
       </c>
       <c r="N47" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O47" t="s">
         <v>547</v>
@@ -8001,7 +8001,7 @@
         <v>558</v>
       </c>
       <c r="N48" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O48" t="s">
         <v>559</v>
@@ -8129,7 +8129,7 @@
         <v>583</v>
       </c>
       <c r="N50" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O50" t="s">
         <v>584</v>
@@ -8387,7 +8387,7 @@
         <v>628</v>
       </c>
       <c r="N54" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O54" t="s">
         <v>629</v>
@@ -8517,7 +8517,7 @@
         <v>651</v>
       </c>
       <c r="N56" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O56" t="s">
         <v>652</v>
@@ -8582,7 +8582,7 @@
         <v>662</v>
       </c>
       <c r="N57" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O57" t="s">
         <v>663</v>
@@ -8647,7 +8647,7 @@
         <v>673</v>
       </c>
       <c r="N58" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O58" t="s">
         <v>674</v>
@@ -8840,7 +8840,7 @@
         <v>708</v>
       </c>
       <c r="N61" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O61" t="s">
         <v>709</v>
@@ -8905,7 +8905,7 @@
         <v>720</v>
       </c>
       <c r="N62" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O62" t="s">
         <v>721</v>
@@ -9035,7 +9035,7 @@
         <v>741</v>
       </c>
       <c r="N64" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="O64" t="s">
         <v>742</v>
@@ -9165,7 +9165,7 @@
         <v>762</v>
       </c>
       <c r="N66" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O66" t="s">
         <v>763</v>
@@ -9468,7 +9468,7 @@
         <v>817</v>
       </c>
       <c r="N71" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O71" t="s">
         <v>818</v>
@@ -9515,7 +9515,7 @@
         <v>25</v>
       </c>
       <c r="H72" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="I72" t="s">
         <v>825</v>
@@ -9663,7 +9663,7 @@
         <v>852</v>
       </c>
       <c r="N74" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O74" t="s">
         <v>853</v>
@@ -9728,7 +9728,7 @@
         <v>864</v>
       </c>
       <c r="N75" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O75" t="s">
         <v>865</v>
@@ -9858,7 +9858,7 @@
         <v>888</v>
       </c>
       <c r="N77" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O77" t="s">
         <v>889</v>
@@ -9963,7 +9963,7 @@
         <v>124</v>
       </c>
       <c r="I79" t="s">
-        <v>338</v>
+        <v>349</v>
       </c>
       <c r="J79" t="s">
         <v>905</v>
@@ -9990,13 +9990,13 @@
         <v>33</v>
       </c>
       <c r="R79" t="s">
-        <v>345</v>
+        <v>356</v>
       </c>
       <c r="S79" t="s">
-        <v>346</v>
+        <v>357</v>
       </c>
       <c r="T79" t="s">
-        <v>347</v>
+        <v>358</v>
       </c>
       <c r="U79" t="s">
         <v>37</v>
@@ -10346,7 +10346,7 @@
         <v>971</v>
       </c>
       <c r="N85" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O85" t="s">
         <v>972</v>
@@ -10411,7 +10411,7 @@
         <v>984</v>
       </c>
       <c r="N86" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O86" t="s">
         <v>985</v>
@@ -10606,7 +10606,7 @@
         <v>1017</v>
       </c>
       <c r="N89" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O89" t="s">
         <v>1018</v>
@@ -10671,7 +10671,7 @@
         <v>1027</v>
       </c>
       <c r="N90" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O90" t="s">
         <v>1028</v>
@@ -10683,13 +10683,13 @@
         <v>153</v>
       </c>
       <c r="R90" t="s">
-        <v>301</v>
+        <v>311</v>
       </c>
       <c r="S90" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="T90" t="s">
-        <v>303</v>
+        <v>313</v>
       </c>
       <c r="U90" t="s">
         <v>37</v>
@@ -11116,7 +11116,7 @@
         <v>1078</v>
       </c>
       <c r="N97" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O97" t="s">
         <v>1079</v>
@@ -11246,7 +11246,7 @@
         <v>1099</v>
       </c>
       <c r="N99" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O99" t="s">
         <v>1100</v>
@@ -11258,13 +11258,13 @@
         <v>33</v>
       </c>
       <c r="R99" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="S99" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="T99" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="U99" t="s">
         <v>37</v>
@@ -11311,7 +11311,7 @@
         <v>1108</v>
       </c>
       <c r="N100" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O100" t="s">
         <v>1109</v>
@@ -11437,7 +11437,7 @@
         <v>1131</v>
       </c>
       <c r="N102" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O102" t="s">
         <v>1132</v>
@@ -11502,7 +11502,7 @@
         <v>1143</v>
       </c>
       <c r="N103" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O103" t="s">
         <v>1144</v>
@@ -11632,7 +11632,7 @@
         <v>1163</v>
       </c>
       <c r="N105" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O105" t="s">
         <v>1164</v>
@@ -12018,7 +12018,7 @@
         <v>1224</v>
       </c>
       <c r="N111" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="O111" t="s">
         <v>1225</v>
@@ -12459,7 +12459,7 @@
         <v>1299</v>
       </c>
       <c r="N118" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="O118" t="s">
         <v>1300</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-03-26
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -455,15 +455,39 @@
     <t xml:space="preserve">Politica internazionale|Politica di sicurezza|Energia</t>
   </si>
   <si>
+    <t xml:space="preserve">26.3069</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sollberger Sandra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verkehrssicherheit stärken mit Projekten entlang der N18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projets le long de la N18 pour renforcer la sécurité routière</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Fin janvier 2026, le Conseil fédéral a publié les grandes lignes du programme Transports ’45. Le fait que les projets routiers le long de la N18 entre Bâle et Delémont, à l’exception du désengorgement du centre de Laufon (horizon de réalisation 2055), soient reportés à une date lointaine après 2055 suscite de l’incompréhension. Ce refus d’améliorer dans les faits l’accessibilité de la région et, par conséquent, ses perspectives de développement économique est en contradiction flagrante avec les résultats de la vaste étude menée sur le corridor&amp;nbsp;N1 sous la direction de l’OFROU selon les méthodes les plus récentes.&lt;/p&gt;&lt;p&gt;La N18 est un élément central du réseau routier national entre la région de Bâle et l’arc lémanique. Elle relie Delémont, le chef-lieu du Jura, et la vallée de Laufon, qui présente un bon dynamisme économique, au réseau routier à grand débit. Cependant, en raison de la croissance démographique, ce tronçon devient toujours plus un goulet d’étranglement. Il affiche même l’un des taux d’embouteillage les plus élevés de Suisse. Parallèlement, la gestion actuelle du trafic nuit considérablement à la qualité de vie dans le cœur des localités et compromet la sécurité des automobilistes et des cyclistes. Les accidents sont notamment fréquents à Grellingen Ouest et au carrefour d’Angenstein. Avec dix blessés légers et un blessé grave entre 2022 et 2024, ce carrefour est même le deuxième endroit le plus accidentogène du canton de Bâle-Campagne. Le nombre d’accidents est aussi élevé dans toutes les localités traversées, ce qui rend la situation intenable. Il est donc primordial de poursuivre rapidement le développement du corridor.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Quel est l’avis du Conseil fédéral sur le besoin d’agir rapidement pour améliorer la sécurité routière le long de la N18, en particulier aux points noirs suivants&amp;nbsp;: carrefour d’Angenstein et Grellingen Ouest (portail sud d’Eggflue)&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Idem en ce qui concerne les traversées de localités, en particulier à Zwingen, Laufon et Delémont&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Considère-t-il le tunnel de Muggenberg comme une mesure qui permettrait d’améliorer durablement la sécurité routière au niveau d’Angenstein&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Du point de vue du Conseil fédéral, un contournement de Laufon et Zwingen contribuerait-il à la sécurité routière le long de la N18&amp;nbsp;?&lt;/li&gt;&lt;/ul&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Ende Januar 2026 wurden vom Bundesrat die Eckwerte zu Verkehr ’45 veröffentlicht. Dass die Strassenprojekte entlang der Nationalstrasse 18 zwischen Basel und Delémont mit Ausnahme der Zentrumsentlastung Laufen (Realisierungshorizont 2055) in einen fernen Zeitraum nach 2055 verschoben werden sollen, stösst in der Region auf Unverständnis. Diese faktische Absage an eine bessere Erreichbarkeit und damit ernsthafte wirtschaftliche Entwicklungsperspektiven steht in direktem Widerspruch zu den Ergebnissen der breit abgestützten Korridorstudie N18, welche unter Federführung des ASTRA nach neuesten Methoden durchgeführt wurde.&lt;/p&gt;&lt;p&gt;Die N18 ist ein zentraler Bestandteil des nationalen Strassennetzes, der den Grossraum Basel mit dem Arc lémanique verbindet. Sie schliesst das wirtschaftlich dynamische Laufental und den Kantonshauptort Delémont an das Hochleistungsstrassennetz an. Aufgrund des Bevölkerungswachstums entwickelt sich dieser Abschnitt jedoch zunehmend zu einem Engpass – mit einer der schweizweit höchsten Staudichten. Gleichzeitig beeinträchtigt die aktuelle Verkehrsführung die Lebensqualität in den Ortszentren erheblich und gefährdet die Sicherheit des Auto- und Veloverkehrs. So kommt es in Grellingen West sowie beim Knoten Angenstein immer wieder zu Unfällen. Bei Letzterem handelt es sich mit zehn Leichtverletzten und einem Schwerverletzten in den Jahren 2022-2024 gar um den zweitgrössten Unfallhotspot des Kantons Baselland. Erhöhte Unfallraten sind zudem auf allen Ortsdurchfahrten zu beobachten – eine unhaltbare Situation. Eine zeitnahe Weiterentwicklung des Korridors ist daher von höchster Priorität.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Wie beurteilt der Bundesrat den Handlungsbedarf zur Verbesserung der Verkehrssicherheit entlang der N18, insbesondere an den Unfallschwerpunkten am Knoten Angenstein sowie am Eggflue-Südportal bzw. Grellingen West?&lt;/li&gt;&lt;li&gt;Wie beurteilt der Bundesrat den Handlungsbedarf zur Verbesserung der Verkehrssicherheit bei den Ortsdurchfahrten entlang der N18, insbesondere in Zwingen, Laufen und Delémont?&lt;/li&gt;&lt;li&gt;Sieht der Bundesrat den Muggenbergtunnel als Massnahme zur nachhaltigen Verbesserung der Verkehrssicherheit am Unfallschwerpunkt Angenstein?&lt;/li&gt;&lt;li&gt;Würde aus Sicht des Bundesrates eine Umfahrung Laufen-Zwingen zur Verkehrssicherheit entlang der N18 beitragen?&lt;/li&gt;&lt;/ul&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263069</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263069</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.7151</t>
   </si>
   <si>
     <t xml:space="preserve">Feller Olivier</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-09</t>
-  </si>
-  <si>
     <t xml:space="preserve">EJPD</t>
   </si>
   <si>
@@ -495,30 +519,6 @@
   </si>
   <si>
     <t xml:space="preserve">Economia|Diritto penale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.3069</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sollberger Sandra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verkehrssicherheit stärken mit Projekten entlang der N18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projets le long de la N18 pour renforcer la sécurité routière</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Fin janvier 2026, le Conseil fédéral a publié les grandes lignes du programme Transports ’45. Le fait que les projets routiers le long de la N18 entre Bâle et Delémont, à l’exception du désengorgement du centre de Laufon (horizon de réalisation 2055), soient reportés à une date lointaine après 2055 suscite de l’incompréhension. Ce refus d’améliorer dans les faits l’accessibilité de la région et, par conséquent, ses perspectives de développement économique est en contradiction flagrante avec les résultats de la vaste étude menée sur le corridor&amp;nbsp;N1 sous la direction de l’OFROU selon les méthodes les plus récentes.&lt;/p&gt;&lt;p&gt;La N18 est un élément central du réseau routier national entre la région de Bâle et l’arc lémanique. Elle relie Delémont, le chef-lieu du Jura, et la vallée de Laufon, qui présente un bon dynamisme économique, au réseau routier à grand débit. Cependant, en raison de la croissance démographique, ce tronçon devient toujours plus un goulet d’étranglement. Il affiche même l’un des taux d’embouteillage les plus élevés de Suisse. Parallèlement, la gestion actuelle du trafic nuit considérablement à la qualité de vie dans le cœur des localités et compromet la sécurité des automobilistes et des cyclistes. Les accidents sont notamment fréquents à Grellingen Ouest et au carrefour d’Angenstein. Avec dix blessés légers et un blessé grave entre 2022 et 2024, ce carrefour est même le deuxième endroit le plus accidentogène du canton de Bâle-Campagne. Le nombre d’accidents est aussi élevé dans toutes les localités traversées, ce qui rend la situation intenable. Il est donc primordial de poursuivre rapidement le développement du corridor.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Quel est l’avis du Conseil fédéral sur le besoin d’agir rapidement pour améliorer la sécurité routière le long de la N18, en particulier aux points noirs suivants&amp;nbsp;: carrefour d’Angenstein et Grellingen Ouest (portail sud d’Eggflue)&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Idem en ce qui concerne les traversées de localités, en particulier à Zwingen, Laufon et Delémont&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Considère-t-il le tunnel de Muggenberg comme une mesure qui permettrait d’améliorer durablement la sécurité routière au niveau d’Angenstein&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Du point de vue du Conseil fédéral, un contournement de Laufon et Zwingen contribuerait-il à la sécurité routière le long de la N18&amp;nbsp;?&lt;/li&gt;&lt;/ul&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Ende Januar 2026 wurden vom Bundesrat die Eckwerte zu Verkehr ’45 veröffentlicht. Dass die Strassenprojekte entlang der Nationalstrasse 18 zwischen Basel und Delémont mit Ausnahme der Zentrumsentlastung Laufen (Realisierungshorizont 2055) in einen fernen Zeitraum nach 2055 verschoben werden sollen, stösst in der Region auf Unverständnis. Diese faktische Absage an eine bessere Erreichbarkeit und damit ernsthafte wirtschaftliche Entwicklungsperspektiven steht in direktem Widerspruch zu den Ergebnissen der breit abgestützten Korridorstudie N18, welche unter Federführung des ASTRA nach neuesten Methoden durchgeführt wurde.&lt;/p&gt;&lt;p&gt;Die N18 ist ein zentraler Bestandteil des nationalen Strassennetzes, der den Grossraum Basel mit dem Arc lémanique verbindet. Sie schliesst das wirtschaftlich dynamische Laufental und den Kantonshauptort Delémont an das Hochleistungsstrassennetz an. Aufgrund des Bevölkerungswachstums entwickelt sich dieser Abschnitt jedoch zunehmend zu einem Engpass – mit einer der schweizweit höchsten Staudichten. Gleichzeitig beeinträchtigt die aktuelle Verkehrsführung die Lebensqualität in den Ortszentren erheblich und gefährdet die Sicherheit des Auto- und Veloverkehrs. So kommt es in Grellingen West sowie beim Knoten Angenstein immer wieder zu Unfällen. Bei Letzterem handelt es sich mit zehn Leichtverletzten und einem Schwerverletzten in den Jahren 2022-2024 gar um den zweitgrössten Unfallhotspot des Kantons Baselland. Erhöhte Unfallraten sind zudem auf allen Ortsdurchfahrten zu beobachten – eine unhaltbare Situation. Eine zeitnahe Weiterentwicklung des Korridors ist daher von höchster Priorität.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Wie beurteilt der Bundesrat den Handlungsbedarf zur Verbesserung der Verkehrssicherheit entlang der N18, insbesondere an den Unfallschwerpunkten am Knoten Angenstein sowie am Eggflue-Südportal bzw. Grellingen West?&lt;/li&gt;&lt;li&gt;Wie beurteilt der Bundesrat den Handlungsbedarf zur Verbesserung der Verkehrssicherheit bei den Ortsdurchfahrten entlang der N18, insbesondere in Zwingen, Laufen und Delémont?&lt;/li&gt;&lt;li&gt;Sieht der Bundesrat den Muggenbergtunnel als Massnahme zur nachhaltigen Verbesserung der Verkehrssicherheit am Unfallschwerpunkt Angenstein?&lt;/li&gt;&lt;li&gt;Würde aus Sicht des Bundesrates eine Umfahrung Laufen-Zwingen zur Verkehrssicherheit entlang der N18 beitragen?&lt;/li&gt;&lt;/ul&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263069</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263069</t>
   </si>
   <si>
     <t xml:space="preserve">26.030</t>
@@ -5797,19 +5797,19 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>20267151</v>
+        <v>20263069</v>
       </c>
       <c r="B13" t="s">
         <v>147</v>
       </c>
       <c r="C13" t="s">
-        <v>120</v>
+        <v>52</v>
       </c>
       <c r="D13" t="s">
         <v>148</v>
       </c>
       <c r="E13" t="s">
-        <v>122</v>
+        <v>54</v>
       </c>
       <c r="F13" t="s">
         <v>149</v>
@@ -5817,42 +5817,42 @@
       <c r="G13" t="s">
         <v>25</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13"/>
+      <c r="I13" t="s">
         <v>150</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>151</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
+        <v>28</v>
+      </c>
+      <c r="L13" t="s">
         <v>152</v>
       </c>
-      <c r="K13"/>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>153</v>
       </c>
-      <c r="M13" t="s">
+      <c r="N13" t="s">
+        <v>30</v>
+      </c>
+      <c r="O13" t="s">
         <v>154</v>
       </c>
-      <c r="N13" t="s">
-        <v>129</v>
-      </c>
-      <c r="O13" t="s">
+      <c r="P13" t="s">
         <v>155</v>
       </c>
-      <c r="P13" t="s">
-        <v>156</v>
-      </c>
       <c r="Q13" t="s">
-        <v>157</v>
+        <v>33</v>
       </c>
       <c r="R13" t="s">
-        <v>158</v>
+        <v>59</v>
       </c>
       <c r="S13" t="s">
-        <v>159</v>
+        <v>60</v>
       </c>
       <c r="T13" t="s">
-        <v>160</v>
+        <v>61</v>
       </c>
       <c r="U13" t="s">
         <v>37</v>
@@ -5860,19 +5860,19 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>20263069</v>
+        <v>20267151</v>
       </c>
       <c r="B14" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>120</v>
       </c>
       <c r="D14" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E14" t="s">
-        <v>54</v>
+        <v>122</v>
       </c>
       <c r="F14" t="s">
         <v>149</v>
@@ -5880,42 +5880,42 @@
       <c r="G14" t="s">
         <v>25</v>
       </c>
-      <c r="H14"/>
+      <c r="H14" t="s">
+        <v>158</v>
+      </c>
       <c r="I14" t="s">
+        <v>159</v>
+      </c>
+      <c r="J14" t="s">
+        <v>160</v>
+      </c>
+      <c r="K14"/>
+      <c r="L14" t="s">
+        <v>161</v>
+      </c>
+      <c r="M14" t="s">
+        <v>162</v>
+      </c>
+      <c r="N14" t="s">
+        <v>129</v>
+      </c>
+      <c r="O14" t="s">
         <v>163</v>
       </c>
-      <c r="J14" t="s">
+      <c r="P14" t="s">
         <v>164</v>
       </c>
-      <c r="K14" t="s">
-        <v>28</v>
-      </c>
-      <c r="L14" t="s">
+      <c r="Q14" t="s">
         <v>165</v>
       </c>
-      <c r="M14" t="s">
+      <c r="R14" t="s">
         <v>166</v>
       </c>
-      <c r="N14" t="s">
-        <v>30</v>
-      </c>
-      <c r="O14" t="s">
+      <c r="S14" t="s">
         <v>167</v>
       </c>
-      <c r="P14" t="s">
+      <c r="T14" t="s">
         <v>168</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>33</v>
-      </c>
-      <c r="R14" t="s">
-        <v>59</v>
-      </c>
-      <c r="S14" t="s">
-        <v>60</v>
-      </c>
-      <c r="T14" t="s">
-        <v>61</v>
       </c>
       <c r="U14" t="s">
         <v>37</v>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="G15"/>
       <c r="H15" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I15" t="s">
         <v>172</v>
@@ -6190,7 +6190,7 @@
         <v>41</v>
       </c>
       <c r="H19" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I19" t="s">
         <v>219</v>
@@ -6347,7 +6347,7 @@
         <v>253</v>
       </c>
       <c r="Q21" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R21" t="s">
         <v>254</v>
@@ -6450,7 +6450,7 @@
         <v>41</v>
       </c>
       <c r="H23" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I23" t="s">
         <v>271</v>
@@ -6542,7 +6542,7 @@
         <v>291</v>
       </c>
       <c r="Q24" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R24" t="s">
         <v>292</v>
@@ -6607,7 +6607,7 @@
         <v>303</v>
       </c>
       <c r="Q25" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R25" t="s">
         <v>201</v>
@@ -6836,7 +6836,7 @@
         <v>25</v>
       </c>
       <c r="H29" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I29" t="s">
         <v>339</v>
@@ -7444,7 +7444,7 @@
         <v>440</v>
       </c>
       <c r="Q38" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R38" t="s">
         <v>441</v>
@@ -7765,7 +7765,7 @@
         <v>500</v>
       </c>
       <c r="Q43" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R43" t="s">
         <v>501</v>
@@ -7866,7 +7866,7 @@
         <v>25</v>
       </c>
       <c r="H45" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I45" t="s">
         <v>517</v>
@@ -8139,7 +8139,7 @@
         <v>570</v>
       </c>
       <c r="Q49" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R49" t="s">
         <v>571</v>
@@ -8397,7 +8397,7 @@
         <v>619</v>
       </c>
       <c r="Q53" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R53" t="s">
         <v>620</v>
@@ -8785,7 +8785,7 @@
         <v>686</v>
       </c>
       <c r="Q59" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R59" t="s">
         <v>687</v>
@@ -9108,7 +9108,7 @@
         <v>744</v>
       </c>
       <c r="Q64" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R64" t="s">
         <v>481</v>
@@ -9303,7 +9303,7 @@
         <v>774</v>
       </c>
       <c r="Q67" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R67" t="s">
         <v>775</v>
@@ -9457,7 +9457,7 @@
       </c>
       <c r="G70"/>
       <c r="H70" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I70" t="s">
         <v>554</v>
@@ -9514,7 +9514,7 @@
         <v>41</v>
       </c>
       <c r="H71" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I71" t="s">
         <v>812</v>
@@ -9736,7 +9736,7 @@
         <v>853</v>
       </c>
       <c r="Q74" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R74" t="s">
         <v>854</v>
@@ -9839,7 +9839,7 @@
         <v>25</v>
       </c>
       <c r="H76" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I76" t="s">
         <v>870</v>
@@ -9866,7 +9866,7 @@
         <v>876</v>
       </c>
       <c r="Q76" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R76" t="s">
         <v>877</v>
@@ -10061,7 +10061,7 @@
         <v>912</v>
       </c>
       <c r="Q79" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R79" t="s">
         <v>913</v>
@@ -10219,7 +10219,7 @@
         <v>25</v>
       </c>
       <c r="H82" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I82" t="s">
         <v>936</v>
@@ -10339,7 +10339,7 @@
       </c>
       <c r="G84"/>
       <c r="H84" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I84" t="s">
         <v>956</v>
@@ -10549,7 +10549,7 @@
         <v>995</v>
       </c>
       <c r="Q87" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R87" t="s">
         <v>996</v>
@@ -10614,7 +10614,7 @@
         <v>1008</v>
       </c>
       <c r="Q88" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R88" t="s">
         <v>1009</v>
@@ -10874,7 +10874,7 @@
         <v>1051</v>
       </c>
       <c r="Q92" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R92" t="s">
         <v>334</v>
@@ -10912,7 +10912,7 @@
         <v>25</v>
       </c>
       <c r="H93" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I93" t="s">
         <v>1054</v>
@@ -11103,7 +11103,7 @@
         <v>25</v>
       </c>
       <c r="H96" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I96" t="s">
         <v>1078</v>
@@ -11166,7 +11166,7 @@
         <v>25</v>
       </c>
       <c r="H97" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I97" t="s">
         <v>1078</v>
@@ -11229,7 +11229,7 @@
         <v>25</v>
       </c>
       <c r="H98" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I98" t="s">
         <v>1078</v>
@@ -11514,7 +11514,7 @@
         <v>1132</v>
       </c>
       <c r="Q102" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R102" t="s">
         <v>1133</v>
@@ -11640,7 +11640,7 @@
         <v>1155</v>
       </c>
       <c r="Q104" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R104" t="s">
         <v>1156</v>
@@ -11705,7 +11705,7 @@
         <v>1167</v>
       </c>
       <c r="Q105" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R105" t="s">
         <v>1168</v>
@@ -11835,7 +11835,7 @@
         <v>1187</v>
       </c>
       <c r="Q107" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R107" t="s">
         <v>1188</v>
@@ -12253,7 +12253,7 @@
       </c>
       <c r="G114"/>
       <c r="H114" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I114" t="s">
         <v>1251</v>
@@ -12310,7 +12310,7 @@
       </c>
       <c r="G115"/>
       <c r="H115" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="I115" t="s">
         <v>1262</v>
@@ -12597,7 +12597,7 @@
         <v>1314</v>
       </c>
       <c r="Q119" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R119" t="s">
         <v>1145</v>
@@ -12727,7 +12727,7 @@
         <v>1336</v>
       </c>
       <c r="Q121" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R121" t="s">
         <v>1337</v>
@@ -12922,7 +12922,7 @@
         <v>1369</v>
       </c>
       <c r="Q124" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R124" t="s">
         <v>1370</v>
@@ -12987,7 +12987,7 @@
         <v>1382</v>
       </c>
       <c r="Q125" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R125" t="s">
         <v>698</v>
@@ -13436,7 +13436,7 @@
         <v>1448</v>
       </c>
       <c r="Q132" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R132" t="s">
         <v>1449</v>
@@ -13501,7 +13501,7 @@
         <v>1459</v>
       </c>
       <c r="Q133" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R133" t="s">
         <v>1460</v>
@@ -13566,7 +13566,7 @@
         <v>1472</v>
       </c>
       <c r="Q134" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R134" t="s">
         <v>1473</v>
@@ -13631,7 +13631,7 @@
         <v>1478</v>
       </c>
       <c r="Q135" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R135" t="s">
         <v>1479</v>
@@ -13696,7 +13696,7 @@
         <v>1491</v>
       </c>
       <c r="Q136" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R136" t="s">
         <v>481</v>
@@ -13889,7 +13889,7 @@
         <v>1523</v>
       </c>
       <c r="Q139" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R139" t="s">
         <v>1513</v>
@@ -14078,7 +14078,7 @@
         <v>1547</v>
       </c>
       <c r="Q142" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="R142" t="s">
         <v>1548</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-04-17
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -359,13 +359,13 @@
     <t xml:space="preserve">2026-03-16</t>
   </si>
   <si>
-    <t xml:space="preserve">Streichung von Art. 22 des Epidemiengesetzes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abrogation de l’art. 22 de la loi sur les épidémies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stralcio dell’articolo 22 della legge sulle epidemie</t>
+    <t xml:space="preserve">Streichung von Artikel 22 des Epidemiengesetzes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrogation de l'article 22 de la loi sur les épidémies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stralcio dell'articolo 22 della legge sulle epidemie</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de présenter à l’Assemblée fédérale un projet d’acte législatif prévoyant l’abrogation de l’art.&amp;nbsp;22 de la loi du 28&amp;nbsp;septembre&amp;nbsp;2012 sur les épidémies (LEp).&amp;nbsp;&lt;/p&gt;</t>
@@ -455,10 +455,10 @@
     <t xml:space="preserve">Rechtliche Abklärungen und Potenzial von künstlicher Intelligenz in den Bereichen Polizei und innere Sicherheit</t>
   </si>
   <si>
-    <t xml:space="preserve">Clarifications juridiques et potentiel de l’utilisation de l’intelligence artificielle (IA) dans les domaines de la police et de la sécurité intérieure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chiarimenti giuridici e potenzialità dell’impiego dell’intelligenza artificiale (IA) nei settori della polizia e della sicurezza interna</t>
+    <t xml:space="preserve">Clarifications juridiques et potentiel de l'utilisation de l'intelligence artificielle (IA) dans les domaines de la police et de la sécurité intérieure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chiarimenti giuridici e potenzialità dell'impiego dell'intelligenza artificiale (IA) nei settori della polizia e della sicurezza interna</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de présenter un rapport concernant l’utilisation de l’intelligence artificielle (IA) dans les domaines de la police, de la sécurité intérieure et de la poursuite pénale exposant le potentiel, les bases légales et les limites constitutionnelles, notamment pour la protection de la vie privée. Sur la base de ces conclusions, il devra soumettre au Parlement des lignes directrices pour une utilisation cohérente et conforme aux droits fondamentaux de l’IA dans les domaines de la police, de la sécurité intérieure et de la poursuite pénale, tout en respectant la souveraineté numérique de la Suisse. Le rapport devra notamment :&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Démontrer le potentiel et les domaines d’application des technologies d’IA pour rendre la lutte contre la criminalité plus efficace et contribuer à la sauvegarde de la sécurité intérieure.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Analyser le cadre juridique existant pour l’utilisation des technologies d’IA dans le domaine de la sécurité et identifier les éventuelles lacunes du cadre juridique.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Expliquer les limites constitutionnelles à l’utilisation des technologies d’IA dans les domaines de la police et de la sécurité et définir des conditions cadre et les lignes directrices pour l’utilisation de ces technologies.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;4. Démontrer comment les exigences en matière de protection de la vie privée peuvent être satisfaites lors de l'utilisation des technologies d'IA dans les domaines de la police et de la sécurité.&amp;nbsp;&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;5. Expliquer comment la souveraineté numérique de la Suisse peut être préservée et la dépendance vis-à-vis des prestataires externes évitée lors de l'acquisition et de l'exploitation des technologies d'IA dans le secteur de la sécurité.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-04-29
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -2354,358 +2354,358 @@
     <t xml:space="preserve">&lt;p&gt;Das Bundesparlament und der Bundesrat werden gebeten, die notwendigen Schritte zu unternehmen, damit unter dem Aspekt des Gebots der bundesstaatlichen und föderalen Rechtsgleichheit die ehemaligen Halbkantone Basel-Stadt und Basel-Landschaft den übrigen Kantonen im Hinblick auf die Vertretung im Ständerat gleichgestellt werden (Aufwertung als Kantone mit Vollem Ständerecht, Änderung von Art. 142 Abs. 4 und Art. 150 Abs. 1 und 2 der Bundesverfassung).&lt;/p&gt;</t>
   </si>
   <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20250301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20250301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.401</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commission de gestion Conseil des États</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-01-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eidgenössische Gerichte. Disziplinarsystem einführen, um das Vertrauen in diese Institutionen zu stärken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tribunaux fédéraux. Introduire un système disciplinaire pour renforcer la confiance à leur égard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tribunali della Confederazione. Introdurre un sistema disciplinare per rafforzare la fiducia in queste istituzioni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Il y a lieu d’élaborer les bases légales permettant d’introduire une surveillance disciplinaire des juges des tribunaux fédéraux. Les principes de l’indépendance des juges, de l’autonomie des tribunaux en matière d’organisation et de la séparation des pouvoirs devront être respectés.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Es seien die gesetzlichen Grundlagen zu erarbeiten, um eine Disziplinaraufsicht über die Richterinnen und Richter an den eidgenössischen Gerichten einzuführen. Dabei ist den Grundsätzen der richterlichen Unabhängigkeit, der Organisationsautonomie und der Gewaltentrennung Rechnung zu tragen.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20250401</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20250401</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staatspolitik|Gerichtswesen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique d'Etat|Justice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica nazionale|Giustizia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.477</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-12-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integrierter Ansatz für Service-Center des Service public</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pour une approche intégrée des centres de services dans le service public</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per un approccio integrato per i centri di servizio del servizio pubblico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;L’Assemblée fédérale est chargée de créer les bases légales permettant de développer et de mettre en œuvre une approche intégrée des centres de services dans le service public. Ce faisant, elle intégrera l’infrastructure existante du réseau postal. L’objectif est de créer une infrastructure moderne et efficace pour la population et de garantir un réseau physique qui assure l’accès des personnes aux produits numériques et aux produits physiques.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Die Bundesversammlung wird beauftragt, die gesetzlichen Grundlagen zu schaffen, um einen integrierten Ansatz für ServiceCenter des Service Public zu entwickeln und umzusetzen. Die bestehende Infrastruktur von PostNetz ist dabei einzubeziehen. Ziel ist es, eine moderne und effiziente Infrastruktur für die Bevölkerung zu schaffen, ein physisches Netz zu sichern, das den Zugang der Menschen zu digitalen und physischen Produkten sichert.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20240477</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20240477</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staatspolitik|Medien und Kommunikation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique d'Etat|Médias et communication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica nazionale|Media e comunicazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.4553</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einführung eines Mechanismus zum interkantonalen Ausgleich des alterungsbedingten Anstiegs der Krankenkassenprämien </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vieillissement de la population. Créer un mécanisme de compensation pour les primes de l’assurance-maladie </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introdurre un meccanismo di compensazione intercantonale per i premi di cassa malati dovuti all’invecchiamento dalla popolazione </t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Dans son avis sur la motion Quadri 24.4209, qui le charge «&amp;nbsp;de proposer un mécanisme de compensation intercantonale de l’augmentation des primes de l’assurance-maladie due au vieillissement de la population&amp;nbsp;», le Conseil fédéral affirme: «&amp;nbsp;Le Conseil fédéral reste d’avis que la péréquation financière nationale assure un équilibre entre les cantons&amp;nbsp;» et souligne notamment que «&amp;nbsp;... la compensation des charges dans le cadre de la péréquation financière nationale comprend une composante sociodémographique, qui tient compte des coûts liés à la structure de la population, notamment à la pyramide des âges. Le Canton du Tessin reçoit déjà des contributions fédérales dans ce cadre.&amp;nbsp;»&lt;/p&gt;&lt;p&gt;Malheureusement, ce n’est pas ce que disent les montants définitifs des paiements compensatoires pour 2025 récemment publiés. Au contraire, le canton du Tessin ne reçoit rien au titre de la compensation sociodémographique, bien qu’il compte le plus grand nombre de personnes de 80 ans ou plus (7,6 % de la population résidante permanente, contre 5,7&amp;nbsp;% pour la moyenne nationale). Le moment est donc venu de reconnaître la situation particulière du Tessin, qui compte une proportion non négligeable de retraités âgés originaires de la Suisse alémanique.&amp;nbsp;&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Je prie donc le Conseil fédéral de répondre aux questions suivantes:&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Confirme-t-il que le Tessin ne reçoit aucune contribution au titre de la compensation sociodémographique, contrairement à ce qu’il affirme dans son avis sur la motion 24.4209?&lt;/li&gt;&lt;li&gt;Au vu de ce qui précède, convient-il que la péréquation financière nationale n’atteint pas son but?&lt;/li&gt;&lt;li&gt;Par conséquent, ne pense-t-il pas que la création d’un mécanisme de compensation intercantonale de l’augmentation des primes de l’assurance-maladie due au vieillissement de la population, demandée par la motion 24.4209, soit à la fois opportune et nécessaire?&amp;nbsp;&lt;/li&gt;&lt;/ul&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;In der Stellungnahme zur Motion Quadri 24.4209, die den Bundesrat beauftragte, einen Mechanismus zum interkantonalen Ausgleich des alterungsbedingten Anstiegs der Krankenkassenprämien einzuführen, hat der Bundesrat festgehalten: «Der Bundesrat ist weiterhin der Meinung, dass der nationale Finanzausgleich für ein Gleichgewicht zwischen den Kantonen sorgt. [...], insbesondere hat er ausgeführt, dass der nationale Finanzausgleich eine soziodemographische Komponente innerhalb des Lastenausgleichs enthält, der die Kosten aufgrund der Bevölkerungsstruktur, u. a. des Alters, berücksichtigt. Der Kanton [...] erhält bereits Beiträge vom Bund im Rahmen des Lastenausgleichs».&lt;/p&gt;&lt;p&gt;Leider decken sich aber die kürzlich veröffentlichten Berechnungen zu den Ausgleichszahlungen 2025 nicht mit diesen Aussagen. So erhält der Kanton Tessin keine Ausgleichszahlungen für den soziodemografischen Lastenausgleich, obwohl er einen besonders hohen Anteil an Personen im Alter von 80 Jahren und mehr im Verhältnis zur ständigen Wohnbevölkerung aufweist (7,6 % gegenüber dem schweizerischen Durchschnitt von 5,7 %). Es ist daher an der Zeit, die besondere Situation des Kantons Tessin anzuerkennen, wo ein nicht unerheblicher Teil der älteren Menschen Rentnerinnen und Rentner aus der Deutschschweiz sind.&amp;nbsp;&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Ich bitte deshalb den Bundesrat, folgende Fragen zu beantworten:&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Bestätigt der Bundesrat, dass der Kanton Tessin – anders als in der Stellungnahme zur Motion 24.4209 behauptet – keine Ausgleichszahlungen für den soziodemografischen Lastenausgleich erhält?&lt;/li&gt;&lt;li&gt;Teilt der Bundesrat in Anbetracht der obigen Ausführungen die Ansicht, dass der nationale Finanzausgleich seinen Zweck nicht erfüllt?&lt;/li&gt;&lt;li&gt;Hält der Bundesrat die Einführung eines Mechanismus zum interkantonalen Ausgleich des alterungsbedingten Anstiegs der Krankenkassenprämien, wie sie mit der Motion 24.4209 verlangt wird, nicht auch für sinnvoll und notwendig?&amp;nbsp;&lt;/li&gt;&lt;/ul&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244553</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244553</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staatspolitik|Finanzwesen|Soziale Fragen|Gesundheit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique d'Etat|Finances|Questions sociales|Santé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica nazionale|Finanze|Questioni sociali|Salute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.4562</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rechsteiner Thomas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Öffentlichkeitsarbeit des Bundes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relations publiques de la Confédération</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attività di pubbliche relazioni della Confederazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Le chancelier de la Confédération a répondu le 16&amp;nbsp;décembre 2024 de manière relativement détaillée à ma question 24.7932 «&amp;nbsp;400 fonctionnaires médias. Y a-t-il un potentiel d’économies&amp;nbsp;?&amp;nbsp;». Certains points restent toutefois flous, et les réponses fournies soulèvent d’autres questions.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Meine Frage 24.7932 «400 Medienbeamte – Sparpotential erkannt?» wurde vom Bundeskanzler am 16. Dezember 2024 relativ ausführlich beantwortet. Trotzdem bleibt einiges im Unklaren und die Antworten werfen weiteren Fragen auf.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244562</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244562</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staatspolitik|Finanzwesen|Medien und Kommunikation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique d'Etat|Finances|Médias et communication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica nazionale|Finanze|Media e comunicazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.4595</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aufhebung des Zentrumslastenausgleichs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suppression de la compensation des charges des centres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eliminare la compensazione degli oneri dei centri urbani</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de modifier la législation relative à la péréquation financière et à la compensation des charges de sorte que la compensation des charges dues à des facteurs socio-démographiques (CCS) ne s’applique désormais plus qu’aux charges excessives liées à la structure de la population et que les charges des centres ne soient plus compensées.&amp;nbsp;&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die Gesetzgebung zum Finanz- und Lastenausgleich dahingehend anzupassen, dass der soziodemografische Lastenausgleich künftig nur mehr Sonderlasten aufgrund der Bevölkerungsstruktur ausgleicht und keinen Zentrumslastenausgleich mehr vorsieht.&amp;nbsp;&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244595</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244595</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staatspolitik|Finanzwesen|Soziale Fragen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique d'Etat|Finances|Questions sociales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica nazionale|Finanze|Questioni sociali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.4634</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Molina Fabian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Übernahme der EU-Richtlinie 2019/1158 zur Vereinbarkeit von Beruf und Privatleben</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reprise de la directive (UE) 2019/1158 concernant l’équilibre entre vie professionnelle et vie privée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recepimento della direttiva UE 2019/1158 relativa all’equilibrio tra attività professionale e vita familiare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de reprendre dans le droit suisse la directive (UE) 2019/1158 concernant l’équilibre entre vie professionnelle et vie privée.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die EU-Richtlinie 2019/118 zur Vereinbarkeit von Beruf und Privatleben ins Schweizer Recht zu übernehmen.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244634</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244634</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Europapolitik|Soziale Fragen|Beschäftigung und Arbeit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique européenne|Questions sociales|Emploi et travail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica europea|Questioni sociali|Occupazione e lavoro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.4660</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Widmer Céline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systemwechsel bei der Wohneigentumsbesteuerung. Steuerliche Folgen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changement de système d’imposition du logement. Conséquences fiscales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cambio di sistema nell'ambito dell'imposizione della proprietà abitativa. Conseguenze fiscali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Les chambres fédérales ont adopté une réforme de l’imposition du logement le 20.12.2024, qui bouleverse les équilibres dans ce domaine tout en amenant de grandes pertes fiscales.&amp;nbsp;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Le conseil fédéral est prié de répondre aux questions suivantes, au sujet de la réforme telle qu’elle a été adoptée par le parlement et de l’introduction d’un impôt réel sur les résidences secondaires :&amp;nbsp;&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;La BNS a annoncé une baisse des taux directeurs à 0.5%. Un scénario avec des taux hypothécaires moyens durablement en dessous de 1.5% devient de plus en plus crédibles. Quelles seraient les pertes fiscales liées à la réforme en cas de taux moyen à 1%&amp;nbsp; et à 1.25%?&amp;nbsp;&amp;nbsp;&lt;/li&gt;&lt;li&gt;Etant donné que la réforme entraine de grandes pertes fiscales, cela veut dire que certains contribuables vont être avantagés par rapport au reste de la population. Est-il correct de dire que les personnes qui toucheront la plus grande somme par rapport à la situation actuelle sont celles et ceux qui disposent de très grandes propriétés avec une énorme valeur et qui n’ont pas de dette liée à cette propriété ?&amp;nbsp; &amp;nbsp;&lt;/li&gt;&lt;li&gt;Combien de baisse d’impôt peut attendre un propriétaire d’une maison de maître d’une valeur de CHF 10'000'000.- et qui finance aujourd’hui son bien entièrement en fonds propres ? Quelle serait le changement de la situation fiscale d’un propriétaire qui dispose d’un bien d’une valeur de CHF 500'000, hypothéqué à hauteur de CHF 400'000.- avec un taux hypothécaire de 3%, et devant faire des frais d’entretiens pour CHF 10'000.-, s’il dispose d’un revenu imposable de 100'000.- ?&amp;nbsp; &amp;nbsp;&lt;/li&gt;&lt;li&gt;Le Conseil fédéral peut-il expliquer quelle est la relation entre d’une part la valeur d’une bien immobilier utilisé comme résidence principale et d’autre part l’allègement fiscal obtenu suite à l’introduction du changement de système d’imposition du logement?&amp;nbsp; &amp;nbsp;&lt;/li&gt;&lt;li&gt;Quels sont les effets de la réforme de l’imposition du logement sur la péréquation financière? En particulier, quel est l’effet sur l’équilibre de cette péréquation à long terme?&amp;nbsp; &amp;nbsp;&lt;/li&gt;&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Die Bundesversammlung hat am 20. Dezember 2024 eine Reform der Wohneigentumsbesteuerung verabschiedet, die das Gleichgewicht in diesem Bereich erheblich stört und gleichzeitig grosse Steuerausfälle mit sich bringt.&amp;nbsp;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Der Bundesrat wird gebeten, die folgenden Fragen zur Reform in der vom Parlament verabschiedeten Form und zur Einführung einer Objektsteuer auf Zweitwohnungen zu beantworten:&lt;/p&gt;&lt;p&gt;1. Die Schweizerische Nationalbank (SNB) hat eine Senkung des Leitzinses auf 0,5&amp;nbsp;Prozent angekündigt. Es ist immer wahrscheinlicher, dass die durchschnittlichen Hypothekarzinsen dauerhaft unter 1,5&amp;nbsp;Prozent liegen. Wie hoch wären die Steuerausfälle aufgrund der Reform bei einem durchschnittlichen Zinssatz von 1 Prozent oder 1,25 Prozent?&amp;nbsp;&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Die Reform führt zu grossen Steuerausfällen. Das bedeutet, dass einige Steuerzahler und Steuerzahlerinnen gegenüber dem Rest der Bevölkerung begünstigt werden. Kann man sagen, dass die Personen, die über sehr grosse Immobilien mit einem enormen Wert verfügen und keine Schulden im Zusammenhang mit diesen Immobilien haben, im Vergleich zur aktuellen Situation am stärksten profitieren?&amp;nbsp; &amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Mit welcher Steuersenkung kann ein Eigentümer einer herrschaftlichen Villa im Wert von 10&amp;nbsp;000&amp;nbsp;000 Franken rechnen, der seine Immobilie heute vollständig mit Eigenmitteln finanziert? Wie würde sich die steuerliche Situation einer Eigentümerin mit einem steuerpflichtigen Einkommen von 100 000 Franken ändern, wenn sie über eine Immobilie im Wert von 500&amp;nbsp;000 Franken verfügt, die mit einer Hypothek in Höhe von 400&amp;nbsp;000 Franken zu einem Hypothekarzins von 3&amp;nbsp;Prozent belastet ist, und sie Unterhaltskosten in Höhe von 10&amp;nbsp;000 Franken tragen muss?&amp;nbsp;&amp;nbsp;&lt;/p&gt;&lt;p&gt;4. &amp;nbsp;Kann der Bundesrat erklären, in welchem Verhältnis der Wert einer Immobilie, die als Erstwohnung genutzt wird, zur Steuererleichterung steht, die durch den Systemwechsel bei der Wohneigentumsbesteuerung erreicht wird?&amp;nbsp; &amp;nbsp;&lt;/p&gt;&lt;p&gt;5. Wie wirkt sich die Reform der Wohneigentumsbesteuerung auf den Finanzausgleich aus?&lt;/p&gt;&lt;p&gt;Welches sind insbesondere die langfristigen Auswirkungen auf das Gleichgewicht des Finanzausgleichs?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244660</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244660</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steuer|Raumplanung und Wohnungswesen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiscalité|Aménagement du territoire et logement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imposte|Pianificazione territoriale e alloggi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.1055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-12-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Was ist die Umweltpolitik des ASTRA im Rahmen seiner Ausschreibungen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quelle est la politique environnementale de l'OFROU dans le cadre de ses appels d'offres?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qual è la politica ambientale dell’USTRA in ambito appaltistico?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;L’OFROU réalise des travaux importants à la sortie de l'autoroute à Matran. Pour une question de prix uniquement, du gravier (grave de route principalement) est acheminé depuis un site du Jura français situé à environ 100km de Matran. Pour ne pas circuler à vide sur le retour, les poids-lourds transportent des éléments de chaussée rabotés et les amènent dans les décharges en France voisine. La distance aller-retour est de 200km environ alors que les mêmes matériaux sont disponibles dans un rayon de moins de 30km dans le canton de Fribourg ou 50km hors canton. Il s’ensuit des trajets et des engorgements supplémentaires, plus de CO2, plus de bruit, plus d’usure des infrastructures, de bruit et de poussières. De surcroit, des chauffeurs dont les conditions de travail sont très précaires remplacent des conducteurs domiciliés en Suisse qui bénéficient de bonnes conditions sociales. En utilisant des graviers locaux, on s'assure qu'ils sont exploités selon les normes locales avec du personnel local. Je remercie donc le Conseil fédéral de répondre aux questions suivantes:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;ul style="list-style-type:disc;"&gt;&lt;li&gt;Les soumissions provenant de l'OFROU prévoient-elles des filières d’approvisionnement et d’évacuation de graviers et autres matériaux minéraux&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Si non, est-il prévu de prendre en compte rapidement les éléments précités?&lt;/li&gt;&lt;li&gt;Si oui, sachant que l’empreinte CO2 du transport de ces matériaux lourds est importante, comment cet élément est-il mis en valeur&amp;nbsp;dans la soumission&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Comment ces aspects sont-ils contrôlés en pratique, sur le terrain&amp;nbsp;?&lt;/li&gt;&lt;li&gt;En cas de faute, quelles sont les conséquences&amp;nbsp;?&lt;/li&gt;&lt;/ul&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Das Bundesamt für Strassen (ASTRA) führt bei der Autobahnausfahrt Matran wichtige Bauarbeiten durch. Dabei wird einzig aus Kostengründen Kies (hauptsächlich als Strassenschotter) aus dem französischen Jura angeliefert, von einem Ort, der rund 100 Kilometer von Matran entfernt liegt. Um auf dem Rückweg Leerfahrten zu vermeiden, transportiert der Schwerverkehr von der Fahrbahn abgeschliffene Elemente ab und entsorgt diese im benachbarten Frankreich. Insgesamt werden rund 200 Kilometer zurückgelegt, obwohl dieselben Materialien in einem Umkreis von weniger als 30 Kilometern im Kanton Freiburg oder 50 Kilometern ausserhalb des Kantons verfügbar wären. Dies führt zu zusätzlichen Fahrten, mehr Stau, CO2, Lärm und Staub sowie zu einer verstärkten Abnutzung der Infrastrukturen. Zudem werden in der Schweiz wohnhafte Chauffeurinnen und Chauffeure, die von guten sozialen Bedingungen profitieren, durch solche mit sehr prekären Arbeitsbedingungen ersetzt. Die Verwendung von lokalem Kies stellt sicher, dass dieser nach lokalen Normen und mit lokalem Personal abgebaut wird. Ich bitte den Bundesrat, die folgenden Fragen zu beantworten:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;ul style="list-style-type:disc;"&gt;&lt;li&gt;Sehen die Ausschreibungen des ASTRA Liefer- und Entsorgungswege für Kies und andere mineralische Materialien vor?&lt;/li&gt;&lt;li&gt;Wenn nein: Ist geplant, die obgenannten Punkte rasch zu berücksichtigen?&lt;/li&gt;&lt;li&gt;Wenn ja: Wie wird dieser Aspekt in der Ausschreibung hervorgehoben, zumal bekannt ist, dass der Transport von Schwergut einen grossen CO2-Fussabdruck hat?&lt;/li&gt;&lt;li&gt;Wie werden diese Aspekte in der Praxis vor Ort kontrolliert?&lt;/li&gt;&lt;li&gt;Was wären die Folgen, wenn sie nicht kontrolliert werden?&lt;/li&gt;&lt;/ul&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20241055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20241055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beschäftigung und Arbeit|Verkehr|Umwelt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emploi et travail|Transports|Environnement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Occupazione e lavoro|Trasporti|Ambiente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.4459</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marti Min Li</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kann die Post einen Beitrag zur digitalen Inklusion leisten? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Poste peut-elle contribuer à l'inclusion numérique? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Posta può contribuire all'inclusione digitale? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Diverses études comme le Baromètre numérique&amp;nbsp;2024 de la Mobilière ont constaté que des compétences numériques de base font défaut à près d’un tiers de la population. Elles relèvent des disparités notables selon l’âge, le revenu et la formation. Même si l’âge joue un rôle en matière de compétences numériques, les personnes âgées ne sont en réalité pas les seules à connaître des difficultés dans l’utilisation des outils numériques comme les services bancaires et les billetteries en ligne ou les guichets virtuels des autorités. Ces lacunes vont souvent de pair avec un sentiment de gêne. &amp;nbsp;Certains, en particulier les jeunes, surestiment leurs propres compétences. De fait, le quotidien bascule toujours plus dans le numérique et exacerbe les lacunes en matière de compétences numériques. C’est pourquoi je prie le Conseil fédéral de répondre aux questions suivantes&amp;nbsp;:&amp;nbsp;&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Que pense-t-il du problème des compétences numériques lacunaires&amp;nbsp;? Comment pourrait-on y remédier&amp;nbsp;?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Les pouvoirs publics et les entreprises proches de la Confédération, par exemple, numérisent de plus en plus leurs services, et ne les proposent parfois plus que sous cette forme. Comment garantir leur accessibilité à tout le monde&amp;nbsp;?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Dans le cadre d’un projet pilote mené dans trois filiales, la Poste a proposé une assistance sur toutes sortes de problèmes relevant du numérique. Que pense le Conseil fédéral de ce projet&amp;nbsp;? La poste pourrait-elle contribuer à faire progresser l’inclusion numérique grâce à cette offre&amp;nbsp;?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Est-ce qu’une telle offre de la Poste ou d’autres entreprises pourraient aussi alléger le travail des autorités&amp;nbsp;?&amp;nbsp;&lt;/li&gt;&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Verschiedene Studien wie beispielsweise der Digitalbarometer 2024 der Mobiliar haben festgestellt, dass fast ein Drittel der Bevölkerung nicht über grundlegende digitale Kompetenzen verfügt. Dabei gibt es signifikante Unterschiede nach Alter, Einkommen und Bildung. Auch wenn das Alter bei den digitalen Kompetenzen eine Rolle spielt, sind es beileibe nicht nur ältere Menschen, die Mühe haben, digitale Anwendungen wie beispielsweise E-Banking, Billetkäufe oder digitale Behördengänge zu nutzen. Dies ist oft auch mit Scham verbunden. &amp;nbsp;Teilweise werden auch die eigenen Fähigkeiten überschätzt, gerade bei jüngeren Menschen. Da immer mehr Dinge des täglichen Lebens digitalisiert werden, stellt die mangelnde digitale Kompetenz ein zunehmendes Problem dar. In diesem Zusammenhang bitte ich den Bundesrat um die Beantwortung folgender Fragen:&amp;nbsp;&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Wie schätzt der Bundesrat das Problem der fehlenden digitalen Kompetenzen ein und wie könnten diese verbessert werden?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Auch Leistungen der öffentlichen Hand oder beispielsweise von bundesnahen Betrieben werden immer häufiger digitalisiert und teilweise nur noch digital angeboten. Wie kann sichergestellt werden, dass alle Personen Zugang zu diesen Leistungen haben?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Im Rahmen eines Pilotprojekts hat die Post in drei Filialen ein Angebot geschaffen, um Menschen bei digitalen Problemen aller Art zu unterstützen. Wie beurteilt der Bundesrat dieses Projekt? Könnte die Post mit diesem Angebot einen Beitrag leisten, die digitale Inklusion voranzutreiben?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Könnte eine entsprechende Dienstleistung der Post oder von anderen Betreibern auch dazu beitragen, Behörden zu entlasten?&amp;nbsp;&lt;/li&gt;&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244459</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244459</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staatspolitik|Soziale Fragen|Medien und Kommunikation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique d'Etat|Questions sociales|Médias et communication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica nazionale|Questioni sociali|Media e comunicazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.331</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanzielle Unterstützung für Imkerinnen und Imker bei geoklimatischen Ausnahmebedingungen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soutien financier direct aux apiculteurs et apicultrices lors de situations géoclimatiques exceptionnelles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sostegno finanziario diretto agli apicoltori in situazioni geoclimatiche eccezionali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Conformément à l'article 160, alinéa 1, de la Constitution fédérale et à l'article 84, lettre o, de la Constitution cantonale, le Canton demande aux Chambres fédérales d'accorder un soutien financier direct, comme des subsides, aux apiculteurs et apicultrices pour l'achat de sucre nécessaire au nourrissement des abeilles mellifères, ceci lorsque les situations géoclimatiques rendent ce nourrissement indispensable à la survie des colonies d'abeilles.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Gestützt auf Artikel&amp;nbsp;160 Absatz&amp;nbsp;1 der Bundesverfassung und Artikel&amp;nbsp;84 Buchstabe&amp;nbsp;o seiner Kantonsverfassung fordert der Kanton Jura die Bundesversammlung auf, den Imkerinnen und Imkern finanzielle Unterstützung, beispielsweise in Form von Subventionen, zu gewähren für den Kauf von Zucker, wenn dieser aufgrund der geoklimatischen Bedingungen an Honigbienen verfüttert werden muss, um deren Überleben sicherzustellen.&lt;/p&gt;</t>
+  </si>
+  <si>
     <t xml:space="preserve">Beratung in Kommission des Nationalrates abgeschlossen / Fin des discussions en commission du Conseil national</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20250301</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20250301</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.401</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commission de gestion Conseil des États</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-01-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eidgenössische Gerichte. Disziplinarsystem einführen, um das Vertrauen in diese Institutionen zu stärken</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tribunaux fédéraux. Introduire un système disciplinaire pour renforcer la confiance à leur égard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tribunali della Confederazione. Introdurre un sistema disciplinare per rafforzare la fiducia in queste istituzioni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Il y a lieu d’élaborer les bases légales permettant d’introduire une surveillance disciplinaire des juges des tribunaux fédéraux. Les principes de l’indépendance des juges, de l’autonomie des tribunaux en matière d’organisation et de la séparation des pouvoirs devront être respectés.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Es seien die gesetzlichen Grundlagen zu erarbeiten, um eine Disziplinaraufsicht über die Richterinnen und Richter an den eidgenössischen Gerichten einzuführen. Dabei ist den Grundsätzen der richterlichen Unabhängigkeit, der Organisationsautonomie und der Gewaltentrennung Rechnung zu tragen.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20250401</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20250401</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik|Gerichtswesen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat|Justice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale|Giustizia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.477</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-12-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Integrierter Ansatz für Service-Center des Service public</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pour une approche intégrée des centres de services dans le service public</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Per un approccio integrato per i centri di servizio del servizio pubblico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;L’Assemblée fédérale est chargée de créer les bases légales permettant de développer et de mettre en œuvre une approche intégrée des centres de services dans le service public. Ce faisant, elle intégrera l’infrastructure existante du réseau postal. L’objectif est de créer une infrastructure moderne et efficace pour la population et de garantir un réseau physique qui assure l’accès des personnes aux produits numériques et aux produits physiques.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Die Bundesversammlung wird beauftragt, die gesetzlichen Grundlagen zu schaffen, um einen integrierten Ansatz für ServiceCenter des Service Public zu entwickeln und umzusetzen. Die bestehende Infrastruktur von PostNetz ist dabei einzubeziehen. Ziel ist es, eine moderne und effiziente Infrastruktur für die Bevölkerung zu schaffen, ein physisches Netz zu sichern, das den Zugang der Menschen zu digitalen und physischen Produkten sichert.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20240477</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20240477</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik|Medien und Kommunikation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat|Médias et communication</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale|Media e comunicazione</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.4553</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einführung eines Mechanismus zum interkantonalen Ausgleich des alterungsbedingten Anstiegs der Krankenkassenprämien </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vieillissement de la population. Créer un mécanisme de compensation pour les primes de l’assurance-maladie </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Introdurre un meccanismo di compensazione intercantonale per i premi di cassa malati dovuti all’invecchiamento dalla popolazione </t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Dans son avis sur la motion Quadri 24.4209, qui le charge «&amp;nbsp;de proposer un mécanisme de compensation intercantonale de l’augmentation des primes de l’assurance-maladie due au vieillissement de la population&amp;nbsp;», le Conseil fédéral affirme: «&amp;nbsp;Le Conseil fédéral reste d’avis que la péréquation financière nationale assure un équilibre entre les cantons&amp;nbsp;» et souligne notamment que «&amp;nbsp;... la compensation des charges dans le cadre de la péréquation financière nationale comprend une composante sociodémographique, qui tient compte des coûts liés à la structure de la population, notamment à la pyramide des âges. Le Canton du Tessin reçoit déjà des contributions fédérales dans ce cadre.&amp;nbsp;»&lt;/p&gt;&lt;p&gt;Malheureusement, ce n’est pas ce que disent les montants définitifs des paiements compensatoires pour 2025 récemment publiés. Au contraire, le canton du Tessin ne reçoit rien au titre de la compensation sociodémographique, bien qu’il compte le plus grand nombre de personnes de 80 ans ou plus (7,6 % de la population résidante permanente, contre 5,7&amp;nbsp;% pour la moyenne nationale). Le moment est donc venu de reconnaître la situation particulière du Tessin, qui compte une proportion non négligeable de retraités âgés originaires de la Suisse alémanique.&amp;nbsp;&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Je prie donc le Conseil fédéral de répondre aux questions suivantes:&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Confirme-t-il que le Tessin ne reçoit aucune contribution au titre de la compensation sociodémographique, contrairement à ce qu’il affirme dans son avis sur la motion 24.4209?&lt;/li&gt;&lt;li&gt;Au vu de ce qui précède, convient-il que la péréquation financière nationale n’atteint pas son but?&lt;/li&gt;&lt;li&gt;Par conséquent, ne pense-t-il pas que la création d’un mécanisme de compensation intercantonale de l’augmentation des primes de l’assurance-maladie due au vieillissement de la population, demandée par la motion 24.4209, soit à la fois opportune et nécessaire?&amp;nbsp;&lt;/li&gt;&lt;/ul&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;In der Stellungnahme zur Motion Quadri 24.4209, die den Bundesrat beauftragte, einen Mechanismus zum interkantonalen Ausgleich des alterungsbedingten Anstiegs der Krankenkassenprämien einzuführen, hat der Bundesrat festgehalten: «Der Bundesrat ist weiterhin der Meinung, dass der nationale Finanzausgleich für ein Gleichgewicht zwischen den Kantonen sorgt. [...], insbesondere hat er ausgeführt, dass der nationale Finanzausgleich eine soziodemographische Komponente innerhalb des Lastenausgleichs enthält, der die Kosten aufgrund der Bevölkerungsstruktur, u. a. des Alters, berücksichtigt. Der Kanton [...] erhält bereits Beiträge vom Bund im Rahmen des Lastenausgleichs».&lt;/p&gt;&lt;p&gt;Leider decken sich aber die kürzlich veröffentlichten Berechnungen zu den Ausgleichszahlungen 2025 nicht mit diesen Aussagen. So erhält der Kanton Tessin keine Ausgleichszahlungen für den soziodemografischen Lastenausgleich, obwohl er einen besonders hohen Anteil an Personen im Alter von 80 Jahren und mehr im Verhältnis zur ständigen Wohnbevölkerung aufweist (7,6 % gegenüber dem schweizerischen Durchschnitt von 5,7 %). Es ist daher an der Zeit, die besondere Situation des Kantons Tessin anzuerkennen, wo ein nicht unerheblicher Teil der älteren Menschen Rentnerinnen und Rentner aus der Deutschschweiz sind.&amp;nbsp;&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Ich bitte deshalb den Bundesrat, folgende Fragen zu beantworten:&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Bestätigt der Bundesrat, dass der Kanton Tessin – anders als in der Stellungnahme zur Motion 24.4209 behauptet – keine Ausgleichszahlungen für den soziodemografischen Lastenausgleich erhält?&lt;/li&gt;&lt;li&gt;Teilt der Bundesrat in Anbetracht der obigen Ausführungen die Ansicht, dass der nationale Finanzausgleich seinen Zweck nicht erfüllt?&lt;/li&gt;&lt;li&gt;Hält der Bundesrat die Einführung eines Mechanismus zum interkantonalen Ausgleich des alterungsbedingten Anstiegs der Krankenkassenprämien, wie sie mit der Motion 24.4209 verlangt wird, nicht auch für sinnvoll und notwendig?&amp;nbsp;&lt;/li&gt;&lt;/ul&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244553</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244553</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik|Finanzwesen|Soziale Fragen|Gesundheit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat|Finances|Questions sociales|Santé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale|Finanze|Questioni sociali|Salute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.4562</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rechsteiner Thomas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Öffentlichkeitsarbeit des Bundes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relations publiques de la Confédération</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attività di pubbliche relazioni della Confederazione</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Le chancelier de la Confédération a répondu le 16&amp;nbsp;décembre 2024 de manière relativement détaillée à ma question 24.7932 «&amp;nbsp;400 fonctionnaires médias. Y a-t-il un potentiel d’économies&amp;nbsp;?&amp;nbsp;». Certains points restent toutefois flous, et les réponses fournies soulèvent d’autres questions.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Meine Frage 24.7932 «400 Medienbeamte – Sparpotential erkannt?» wurde vom Bundeskanzler am 16. Dezember 2024 relativ ausführlich beantwortet. Trotzdem bleibt einiges im Unklaren und die Antworten werfen weiteren Fragen auf.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244562</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244562</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik|Finanzwesen|Medien und Kommunikation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat|Finances|Médias et communication</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale|Finanze|Media e comunicazione</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.4595</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aufhebung des Zentrumslastenausgleichs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suppression de la compensation des charges des centres</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eliminare la compensazione degli oneri dei centri urbani</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de modifier la législation relative à la péréquation financière et à la compensation des charges de sorte que la compensation des charges dues à des facteurs socio-démographiques (CCS) ne s’applique désormais plus qu’aux charges excessives liées à la structure de la population et que les charges des centres ne soient plus compensées.&amp;nbsp;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die Gesetzgebung zum Finanz- und Lastenausgleich dahingehend anzupassen, dass der soziodemografische Lastenausgleich künftig nur mehr Sonderlasten aufgrund der Bevölkerungsstruktur ausgleicht und keinen Zentrumslastenausgleich mehr vorsieht.&amp;nbsp;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244595</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244595</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik|Finanzwesen|Soziale Fragen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat|Finances|Questions sociales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale|Finanze|Questioni sociali</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.4634</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Molina Fabian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Übernahme der EU-Richtlinie 2019/1158 zur Vereinbarkeit von Beruf und Privatleben</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reprise de la directive (UE) 2019/1158 concernant l’équilibre entre vie professionnelle et vie privée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recepimento della direttiva UE 2019/1158 relativa all’equilibrio tra attività professionale e vita familiare</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de reprendre dans le droit suisse la directive (UE) 2019/1158 concernant l’équilibre entre vie professionnelle et vie privée.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, die EU-Richtlinie 2019/118 zur Vereinbarkeit von Beruf und Privatleben ins Schweizer Recht zu übernehmen.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244634</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244634</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Europapolitik|Soziale Fragen|Beschäftigung und Arbeit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique européenne|Questions sociales|Emploi et travail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica europea|Questioni sociali|Occupazione e lavoro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.4660</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Widmer Céline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Systemwechsel bei der Wohneigentumsbesteuerung. Steuerliche Folgen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Changement de système d’imposition du logement. Conséquences fiscales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cambio di sistema nell'ambito dell'imposizione della proprietà abitativa. Conseguenze fiscali</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Les chambres fédérales ont adopté une réforme de l’imposition du logement le 20.12.2024, qui bouleverse les équilibres dans ce domaine tout en amenant de grandes pertes fiscales.&amp;nbsp;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Le conseil fédéral est prié de répondre aux questions suivantes, au sujet de la réforme telle qu’elle a été adoptée par le parlement et de l’introduction d’un impôt réel sur les résidences secondaires :&amp;nbsp;&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;La BNS a annoncé une baisse des taux directeurs à 0.5%. Un scénario avec des taux hypothécaires moyens durablement en dessous de 1.5% devient de plus en plus crédibles. Quelles seraient les pertes fiscales liées à la réforme en cas de taux moyen à 1%&amp;nbsp; et à 1.25%?&amp;nbsp;&amp;nbsp;&lt;/li&gt;&lt;li&gt;Etant donné que la réforme entraine de grandes pertes fiscales, cela veut dire que certains contribuables vont être avantagés par rapport au reste de la population. Est-il correct de dire que les personnes qui toucheront la plus grande somme par rapport à la situation actuelle sont celles et ceux qui disposent de très grandes propriétés avec une énorme valeur et qui n’ont pas de dette liée à cette propriété ?&amp;nbsp; &amp;nbsp;&lt;/li&gt;&lt;li&gt;Combien de baisse d’impôt peut attendre un propriétaire d’une maison de maître d’une valeur de CHF 10'000'000.- et qui finance aujourd’hui son bien entièrement en fonds propres ? Quelle serait le changement de la situation fiscale d’un propriétaire qui dispose d’un bien d’une valeur de CHF 500'000, hypothéqué à hauteur de CHF 400'000.- avec un taux hypothécaire de 3%, et devant faire des frais d’entretiens pour CHF 10'000.-, s’il dispose d’un revenu imposable de 100'000.- ?&amp;nbsp; &amp;nbsp;&lt;/li&gt;&lt;li&gt;Le Conseil fédéral peut-il expliquer quelle est la relation entre d’une part la valeur d’une bien immobilier utilisé comme résidence principale et d’autre part l’allègement fiscal obtenu suite à l’introduction du changement de système d’imposition du logement?&amp;nbsp; &amp;nbsp;&lt;/li&gt;&lt;li&gt;Quels sont les effets de la réforme de l’imposition du logement sur la péréquation financière? En particulier, quel est l’effet sur l’équilibre de cette péréquation à long terme?&amp;nbsp; &amp;nbsp;&lt;/li&gt;&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Die Bundesversammlung hat am 20. Dezember 2024 eine Reform der Wohneigentumsbesteuerung verabschiedet, die das Gleichgewicht in diesem Bereich erheblich stört und gleichzeitig grosse Steuerausfälle mit sich bringt.&amp;nbsp;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Der Bundesrat wird gebeten, die folgenden Fragen zur Reform in der vom Parlament verabschiedeten Form und zur Einführung einer Objektsteuer auf Zweitwohnungen zu beantworten:&lt;/p&gt;&lt;p&gt;1. Die Schweizerische Nationalbank (SNB) hat eine Senkung des Leitzinses auf 0,5&amp;nbsp;Prozent angekündigt. Es ist immer wahrscheinlicher, dass die durchschnittlichen Hypothekarzinsen dauerhaft unter 1,5&amp;nbsp;Prozent liegen. Wie hoch wären die Steuerausfälle aufgrund der Reform bei einem durchschnittlichen Zinssatz von 1 Prozent oder 1,25 Prozent?&amp;nbsp;&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Die Reform führt zu grossen Steuerausfällen. Das bedeutet, dass einige Steuerzahler und Steuerzahlerinnen gegenüber dem Rest der Bevölkerung begünstigt werden. Kann man sagen, dass die Personen, die über sehr grosse Immobilien mit einem enormen Wert verfügen und keine Schulden im Zusammenhang mit diesen Immobilien haben, im Vergleich zur aktuellen Situation am stärksten profitieren?&amp;nbsp; &amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Mit welcher Steuersenkung kann ein Eigentümer einer herrschaftlichen Villa im Wert von 10&amp;nbsp;000&amp;nbsp;000 Franken rechnen, der seine Immobilie heute vollständig mit Eigenmitteln finanziert? Wie würde sich die steuerliche Situation einer Eigentümerin mit einem steuerpflichtigen Einkommen von 100 000 Franken ändern, wenn sie über eine Immobilie im Wert von 500&amp;nbsp;000 Franken verfügt, die mit einer Hypothek in Höhe von 400&amp;nbsp;000 Franken zu einem Hypothekarzins von 3&amp;nbsp;Prozent belastet ist, und sie Unterhaltskosten in Höhe von 10&amp;nbsp;000 Franken tragen muss?&amp;nbsp;&amp;nbsp;&lt;/p&gt;&lt;p&gt;4. &amp;nbsp;Kann der Bundesrat erklären, in welchem Verhältnis der Wert einer Immobilie, die als Erstwohnung genutzt wird, zur Steuererleichterung steht, die durch den Systemwechsel bei der Wohneigentumsbesteuerung erreicht wird?&amp;nbsp; &amp;nbsp;&lt;/p&gt;&lt;p&gt;5. Wie wirkt sich die Reform der Wohneigentumsbesteuerung auf den Finanzausgleich aus?&lt;/p&gt;&lt;p&gt;Welches sind insbesondere die langfristigen Auswirkungen auf das Gleichgewicht des Finanzausgleichs?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244660</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244660</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Steuer|Raumplanung und Wohnungswesen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fiscalité|Aménagement du territoire et logement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imposte|Pianificazione territoriale e alloggi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.1055</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-12-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Was ist die Umweltpolitik des ASTRA im Rahmen seiner Ausschreibungen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quelle est la politique environnementale de l'OFROU dans le cadre de ses appels d'offres?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Qual è la politica ambientale dell’USTRA in ambito appaltistico?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;L’OFROU réalise des travaux importants à la sortie de l'autoroute à Matran. Pour une question de prix uniquement, du gravier (grave de route principalement) est acheminé depuis un site du Jura français situé à environ 100km de Matran. Pour ne pas circuler à vide sur le retour, les poids-lourds transportent des éléments de chaussée rabotés et les amènent dans les décharges en France voisine. La distance aller-retour est de 200km environ alors que les mêmes matériaux sont disponibles dans un rayon de moins de 30km dans le canton de Fribourg ou 50km hors canton. Il s’ensuit des trajets et des engorgements supplémentaires, plus de CO2, plus de bruit, plus d’usure des infrastructures, de bruit et de poussières. De surcroit, des chauffeurs dont les conditions de travail sont très précaires remplacent des conducteurs domiciliés en Suisse qui bénéficient de bonnes conditions sociales. En utilisant des graviers locaux, on s'assure qu'ils sont exploités selon les normes locales avec du personnel local. Je remercie donc le Conseil fédéral de répondre aux questions suivantes:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;ul style="list-style-type:disc;"&gt;&lt;li&gt;Les soumissions provenant de l'OFROU prévoient-elles des filières d’approvisionnement et d’évacuation de graviers et autres matériaux minéraux&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Si non, est-il prévu de prendre en compte rapidement les éléments précités?&lt;/li&gt;&lt;li&gt;Si oui, sachant que l’empreinte CO2 du transport de ces matériaux lourds est importante, comment cet élément est-il mis en valeur&amp;nbsp;dans la soumission&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Comment ces aspects sont-ils contrôlés en pratique, sur le terrain&amp;nbsp;?&lt;/li&gt;&lt;li&gt;En cas de faute, quelles sont les conséquences&amp;nbsp;?&lt;/li&gt;&lt;/ul&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Das Bundesamt für Strassen (ASTRA) führt bei der Autobahnausfahrt Matran wichtige Bauarbeiten durch. Dabei wird einzig aus Kostengründen Kies (hauptsächlich als Strassenschotter) aus dem französischen Jura angeliefert, von einem Ort, der rund 100 Kilometer von Matran entfernt liegt. Um auf dem Rückweg Leerfahrten zu vermeiden, transportiert der Schwerverkehr von der Fahrbahn abgeschliffene Elemente ab und entsorgt diese im benachbarten Frankreich. Insgesamt werden rund 200 Kilometer zurückgelegt, obwohl dieselben Materialien in einem Umkreis von weniger als 30 Kilometern im Kanton Freiburg oder 50 Kilometern ausserhalb des Kantons verfügbar wären. Dies führt zu zusätzlichen Fahrten, mehr Stau, CO2, Lärm und Staub sowie zu einer verstärkten Abnutzung der Infrastrukturen. Zudem werden in der Schweiz wohnhafte Chauffeurinnen und Chauffeure, die von guten sozialen Bedingungen profitieren, durch solche mit sehr prekären Arbeitsbedingungen ersetzt. Die Verwendung von lokalem Kies stellt sicher, dass dieser nach lokalen Normen und mit lokalem Personal abgebaut wird. Ich bitte den Bundesrat, die folgenden Fragen zu beantworten:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;ul style="list-style-type:disc;"&gt;&lt;li&gt;Sehen die Ausschreibungen des ASTRA Liefer- und Entsorgungswege für Kies und andere mineralische Materialien vor?&lt;/li&gt;&lt;li&gt;Wenn nein: Ist geplant, die obgenannten Punkte rasch zu berücksichtigen?&lt;/li&gt;&lt;li&gt;Wenn ja: Wie wird dieser Aspekt in der Ausschreibung hervorgehoben, zumal bekannt ist, dass der Transport von Schwergut einen grossen CO2-Fussabdruck hat?&lt;/li&gt;&lt;li&gt;Wie werden diese Aspekte in der Praxis vor Ort kontrolliert?&lt;/li&gt;&lt;li&gt;Was wären die Folgen, wenn sie nicht kontrolliert werden?&lt;/li&gt;&lt;/ul&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20241055</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20241055</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beschäftigung und Arbeit|Verkehr|Umwelt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Emploi et travail|Transports|Environnement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Occupazione e lavoro|Trasporti|Ambiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.4459</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marti Min Li</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kann die Post einen Beitrag zur digitalen Inklusion leisten? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Poste peut-elle contribuer à l'inclusion numérique? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Posta può contribuire all'inclusione digitale? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Diverses études comme le Baromètre numérique&amp;nbsp;2024 de la Mobilière ont constaté que des compétences numériques de base font défaut à près d’un tiers de la population. Elles relèvent des disparités notables selon l’âge, le revenu et la formation. Même si l’âge joue un rôle en matière de compétences numériques, les personnes âgées ne sont en réalité pas les seules à connaître des difficultés dans l’utilisation des outils numériques comme les services bancaires et les billetteries en ligne ou les guichets virtuels des autorités. Ces lacunes vont souvent de pair avec un sentiment de gêne. &amp;nbsp;Certains, en particulier les jeunes, surestiment leurs propres compétences. De fait, le quotidien bascule toujours plus dans le numérique et exacerbe les lacunes en matière de compétences numériques. C’est pourquoi je prie le Conseil fédéral de répondre aux questions suivantes&amp;nbsp;:&amp;nbsp;&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Que pense-t-il du problème des compétences numériques lacunaires&amp;nbsp;? Comment pourrait-on y remédier&amp;nbsp;?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Les pouvoirs publics et les entreprises proches de la Confédération, par exemple, numérisent de plus en plus leurs services, et ne les proposent parfois plus que sous cette forme. Comment garantir leur accessibilité à tout le monde&amp;nbsp;?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Dans le cadre d’un projet pilote mené dans trois filiales, la Poste a proposé une assistance sur toutes sortes de problèmes relevant du numérique. Que pense le Conseil fédéral de ce projet&amp;nbsp;? La poste pourrait-elle contribuer à faire progresser l’inclusion numérique grâce à cette offre&amp;nbsp;?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Est-ce qu’une telle offre de la Poste ou d’autres entreprises pourraient aussi alléger le travail des autorités&amp;nbsp;?&amp;nbsp;&lt;/li&gt;&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Verschiedene Studien wie beispielsweise der Digitalbarometer 2024 der Mobiliar haben festgestellt, dass fast ein Drittel der Bevölkerung nicht über grundlegende digitale Kompetenzen verfügt. Dabei gibt es signifikante Unterschiede nach Alter, Einkommen und Bildung. Auch wenn das Alter bei den digitalen Kompetenzen eine Rolle spielt, sind es beileibe nicht nur ältere Menschen, die Mühe haben, digitale Anwendungen wie beispielsweise E-Banking, Billetkäufe oder digitale Behördengänge zu nutzen. Dies ist oft auch mit Scham verbunden. &amp;nbsp;Teilweise werden auch die eigenen Fähigkeiten überschätzt, gerade bei jüngeren Menschen. Da immer mehr Dinge des täglichen Lebens digitalisiert werden, stellt die mangelnde digitale Kompetenz ein zunehmendes Problem dar. In diesem Zusammenhang bitte ich den Bundesrat um die Beantwortung folgender Fragen:&amp;nbsp;&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Wie schätzt der Bundesrat das Problem der fehlenden digitalen Kompetenzen ein und wie könnten diese verbessert werden?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Auch Leistungen der öffentlichen Hand oder beispielsweise von bundesnahen Betrieben werden immer häufiger digitalisiert und teilweise nur noch digital angeboten. Wie kann sichergestellt werden, dass alle Personen Zugang zu diesen Leistungen haben?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Im Rahmen eines Pilotprojekts hat die Post in drei Filialen ein Angebot geschaffen, um Menschen bei digitalen Problemen aller Art zu unterstützen. Wie beurteilt der Bundesrat dieses Projekt? Könnte die Post mit diesem Angebot einen Beitrag leisten, die digitale Inklusion voranzutreiben?&amp;nbsp;&lt;/li&gt;&lt;li&gt;Könnte eine entsprechende Dienstleistung der Post oder von anderen Betreibern auch dazu beitragen, Behörden zu entlasten?&amp;nbsp;&lt;/li&gt;&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244459</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20244459</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik|Soziale Fragen|Medien und Kommunikation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat|Questions sociales|Médias et communication</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale|Questioni sociali|Media e comunicazione</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.331</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanzielle Unterstützung für Imkerinnen und Imker bei geoklimatischen Ausnahmebedingungen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Soutien financier direct aux apiculteurs et apicultrices lors de situations géoclimatiques exceptionnelles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sostegno finanziario diretto agli apicoltori in situazioni geoclimatiche eccezionali</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Conformément à l'article 160, alinéa 1, de la Constitution fédérale et à l'article 84, lettre o, de la Constitution cantonale, le Canton demande aux Chambres fédérales d'accorder un soutien financier direct, comme des subsides, aux apiculteurs et apicultrices pour l'achat de sucre nécessaire au nourrissement des abeilles mellifères, ceci lorsque les situations géoclimatiques rendent ce nourrissement indispensable à la survie des colonies d'abeilles.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Gestützt auf Artikel&amp;nbsp;160 Absatz&amp;nbsp;1 der Bundesverfassung und Artikel&amp;nbsp;84 Buchstabe&amp;nbsp;o seiner Kantonsverfassung fordert der Kanton Jura die Bundesversammlung auf, den Imkerinnen und Imkern finanzielle Unterstützung, beispielsweise in Form von Subventionen, zu gewähren für den Kauf von Zucker, wenn dieser aufgrund der geoklimatischen Bedingungen an Honigbienen verfüttert werden muss, um deren Überleben sicherzustellen.&lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20240331</t>
@@ -9198,13 +9198,13 @@
         <v>779</v>
       </c>
       <c r="N65" t="s">
+        <v>170</v>
+      </c>
+      <c r="O65" t="s">
         <v>780</v>
       </c>
-      <c r="O65" t="s">
+      <c r="P65" t="s">
         <v>781</v>
-      </c>
-      <c r="P65" t="s">
-        <v>782</v>
       </c>
       <c r="Q65" t="s">
         <v>55</v>
@@ -9222,17 +9222,17 @@
         <v>20250401</v>
       </c>
       <c r="B66" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C66" t="s">
         <v>444</v>
       </c>
       <c r="D66" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E66"/>
       <c r="F66" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="G66" t="s">
         <v>27</v>
@@ -9241,40 +9241,40 @@
         <v>28</v>
       </c>
       <c r="I66" t="s">
+        <v>785</v>
+      </c>
+      <c r="J66" t="s">
         <v>786</v>
       </c>
-      <c r="J66" t="s">
+      <c r="K66" t="s">
         <v>787</v>
       </c>
-      <c r="K66" t="s">
+      <c r="L66" t="s">
         <v>788</v>
       </c>
-      <c r="L66" t="s">
+      <c r="M66" t="s">
         <v>789</v>
-      </c>
-      <c r="M66" t="s">
-        <v>790</v>
       </c>
       <c r="N66" t="s">
         <v>34</v>
       </c>
       <c r="O66" t="s">
+        <v>790</v>
+      </c>
+      <c r="P66" t="s">
         <v>791</v>
-      </c>
-      <c r="P66" t="s">
-        <v>792</v>
       </c>
       <c r="Q66" t="s">
         <v>55</v>
       </c>
       <c r="R66" t="s">
+        <v>792</v>
+      </c>
+      <c r="S66" t="s">
         <v>793</v>
       </c>
-      <c r="S66" t="s">
+      <c r="T66" t="s">
         <v>794</v>
-      </c>
-      <c r="T66" t="s">
-        <v>795</v>
       </c>
       <c r="U66" t="s">
         <v>59</v>
@@ -9286,7 +9286,7 @@
         <v>20240477</v>
       </c>
       <c r="B67" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="C67" t="s">
         <v>444</v>
@@ -9298,7 +9298,7 @@
         <v>62</v>
       </c>
       <c r="F67" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="G67" t="s">
         <v>45</v>
@@ -9307,40 +9307,40 @@
         <v>78</v>
       </c>
       <c r="I67" t="s">
+        <v>797</v>
+      </c>
+      <c r="J67" t="s">
         <v>798</v>
       </c>
-      <c r="J67" t="s">
+      <c r="K67" t="s">
         <v>799</v>
       </c>
-      <c r="K67" t="s">
+      <c r="L67" t="s">
         <v>800</v>
       </c>
-      <c r="L67" t="s">
+      <c r="M67" t="s">
         <v>801</v>
-      </c>
-      <c r="M67" t="s">
-        <v>802</v>
       </c>
       <c r="N67" t="s">
         <v>170</v>
       </c>
       <c r="O67" t="s">
+        <v>802</v>
+      </c>
+      <c r="P67" t="s">
         <v>803</v>
-      </c>
-      <c r="P67" t="s">
-        <v>804</v>
       </c>
       <c r="Q67" t="s">
         <v>55</v>
       </c>
       <c r="R67" t="s">
+        <v>804</v>
+      </c>
+      <c r="S67" t="s">
         <v>805</v>
       </c>
-      <c r="S67" t="s">
+      <c r="T67" t="s">
         <v>806</v>
-      </c>
-      <c r="T67" t="s">
-        <v>807</v>
       </c>
       <c r="U67" t="s">
         <v>59</v>
@@ -9352,7 +9352,7 @@
         <v>20244553</v>
       </c>
       <c r="B68" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="C68" t="s">
         <v>75</v>
@@ -9364,7 +9364,7 @@
         <v>653</v>
       </c>
       <c r="F68" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="G68" t="s">
         <v>45</v>
@@ -9373,40 +9373,40 @@
         <v>46</v>
       </c>
       <c r="I68" t="s">
+        <v>808</v>
+      </c>
+      <c r="J68" t="s">
         <v>809</v>
       </c>
-      <c r="J68" t="s">
+      <c r="K68" t="s">
         <v>810</v>
       </c>
-      <c r="K68" t="s">
+      <c r="L68" t="s">
         <v>811</v>
       </c>
-      <c r="L68" t="s">
+      <c r="M68" t="s">
         <v>812</v>
-      </c>
-      <c r="M68" t="s">
-        <v>813</v>
       </c>
       <c r="N68" t="s">
         <v>244</v>
       </c>
       <c r="O68" t="s">
+        <v>813</v>
+      </c>
+      <c r="P68" t="s">
         <v>814</v>
-      </c>
-      <c r="P68" t="s">
-        <v>815</v>
       </c>
       <c r="Q68" t="s">
         <v>247</v>
       </c>
       <c r="R68" t="s">
+        <v>815</v>
+      </c>
+      <c r="S68" t="s">
         <v>816</v>
       </c>
-      <c r="S68" t="s">
+      <c r="T68" t="s">
         <v>817</v>
-      </c>
-      <c r="T68" t="s">
-        <v>818</v>
       </c>
       <c r="U68" t="s">
         <v>59</v>
@@ -9418,61 +9418,61 @@
         <v>20244562</v>
       </c>
       <c r="B69" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="C69" t="s">
         <v>75</v>
       </c>
       <c r="D69" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="E69" t="s">
         <v>25</v>
       </c>
       <c r="F69" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="G69" t="s">
         <v>45</v>
       </c>
       <c r="H69" t="s">
+        <v>820</v>
+      </c>
+      <c r="I69" t="s">
         <v>821</v>
       </c>
-      <c r="I69" t="s">
+      <c r="J69" t="s">
         <v>822</v>
       </c>
-      <c r="J69" t="s">
+      <c r="K69" t="s">
         <v>823</v>
       </c>
-      <c r="K69" t="s">
+      <c r="L69" t="s">
         <v>824</v>
       </c>
-      <c r="L69" t="s">
+      <c r="M69" t="s">
         <v>825</v>
-      </c>
-      <c r="M69" t="s">
-        <v>826</v>
       </c>
       <c r="N69" t="s">
         <v>170</v>
       </c>
       <c r="O69" t="s">
+        <v>826</v>
+      </c>
+      <c r="P69" t="s">
         <v>827</v>
-      </c>
-      <c r="P69" t="s">
-        <v>828</v>
       </c>
       <c r="Q69" t="s">
         <v>195</v>
       </c>
       <c r="R69" t="s">
+        <v>828</v>
+      </c>
+      <c r="S69" t="s">
         <v>829</v>
       </c>
-      <c r="S69" t="s">
+      <c r="T69" t="s">
         <v>830</v>
-      </c>
-      <c r="T69" t="s">
-        <v>831</v>
       </c>
       <c r="U69" t="s">
         <v>59</v>
@@ -9484,7 +9484,7 @@
         <v>20244595</v>
       </c>
       <c r="B70" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="C70" t="s">
         <v>23</v>
@@ -9496,7 +9496,7 @@
         <v>104</v>
       </c>
       <c r="F70" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="G70" t="s">
         <v>45</v>
@@ -9505,40 +9505,40 @@
         <v>46</v>
       </c>
       <c r="I70" t="s">
+        <v>832</v>
+      </c>
+      <c r="J70" t="s">
         <v>833</v>
       </c>
-      <c r="J70" t="s">
+      <c r="K70" t="s">
         <v>834</v>
       </c>
-      <c r="K70" t="s">
+      <c r="L70" t="s">
         <v>835</v>
       </c>
-      <c r="L70" t="s">
+      <c r="M70" t="s">
         <v>836</v>
-      </c>
-      <c r="M70" t="s">
-        <v>837</v>
       </c>
       <c r="N70" t="s">
         <v>568</v>
       </c>
       <c r="O70" t="s">
+        <v>837</v>
+      </c>
+      <c r="P70" t="s">
         <v>838</v>
-      </c>
-      <c r="P70" t="s">
-        <v>839</v>
       </c>
       <c r="Q70" t="s">
         <v>247</v>
       </c>
       <c r="R70" t="s">
+        <v>839</v>
+      </c>
+      <c r="S70" t="s">
         <v>840</v>
       </c>
-      <c r="S70" t="s">
+      <c r="T70" t="s">
         <v>841</v>
-      </c>
-      <c r="T70" t="s">
-        <v>842</v>
       </c>
       <c r="U70" t="s">
         <v>59</v>
@@ -9550,19 +9550,19 @@
         <v>20244634</v>
       </c>
       <c r="B71" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="C71" t="s">
         <v>23</v>
       </c>
       <c r="D71" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="E71" t="s">
         <v>62</v>
       </c>
       <c r="F71" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="G71" t="s">
         <v>45</v>
@@ -9571,40 +9571,40 @@
         <v>28</v>
       </c>
       <c r="I71" t="s">
+        <v>844</v>
+      </c>
+      <c r="J71" t="s">
         <v>845</v>
       </c>
-      <c r="J71" t="s">
+      <c r="K71" t="s">
         <v>846</v>
       </c>
-      <c r="K71" t="s">
+      <c r="L71" t="s">
         <v>847</v>
       </c>
-      <c r="L71" t="s">
+      <c r="M71" t="s">
         <v>848</v>
-      </c>
-      <c r="M71" t="s">
-        <v>849</v>
       </c>
       <c r="N71" t="s">
         <v>244</v>
       </c>
       <c r="O71" t="s">
+        <v>849</v>
+      </c>
+      <c r="P71" t="s">
         <v>850</v>
-      </c>
-      <c r="P71" t="s">
-        <v>851</v>
       </c>
       <c r="Q71" t="s">
         <v>195</v>
       </c>
       <c r="R71" t="s">
+        <v>851</v>
+      </c>
+      <c r="S71" t="s">
         <v>852</v>
       </c>
-      <c r="S71" t="s">
+      <c r="T71" t="s">
         <v>853</v>
-      </c>
-      <c r="T71" t="s">
-        <v>854</v>
       </c>
       <c r="U71" t="s">
         <v>59</v>
@@ -9616,19 +9616,19 @@
         <v>20244660</v>
       </c>
       <c r="B72" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="C72" t="s">
         <v>75</v>
       </c>
       <c r="D72" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="E72" t="s">
         <v>62</v>
       </c>
       <c r="F72" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="G72" t="s">
         <v>45</v>
@@ -9637,40 +9637,40 @@
         <v>46</v>
       </c>
       <c r="I72" t="s">
+        <v>856</v>
+      </c>
+      <c r="J72" t="s">
         <v>857</v>
       </c>
-      <c r="J72" t="s">
+      <c r="K72" t="s">
         <v>858</v>
       </c>
-      <c r="K72" t="s">
+      <c r="L72" t="s">
         <v>859</v>
       </c>
-      <c r="L72" t="s">
+      <c r="M72" t="s">
         <v>860</v>
-      </c>
-      <c r="M72" t="s">
-        <v>861</v>
       </c>
       <c r="N72" t="s">
         <v>244</v>
       </c>
       <c r="O72" t="s">
+        <v>861</v>
+      </c>
+      <c r="P72" t="s">
         <v>862</v>
-      </c>
-      <c r="P72" t="s">
-        <v>863</v>
       </c>
       <c r="Q72" t="s">
         <v>247</v>
       </c>
       <c r="R72" t="s">
+        <v>863</v>
+      </c>
+      <c r="S72" t="s">
         <v>864</v>
       </c>
-      <c r="S72" t="s">
+      <c r="T72" t="s">
         <v>865</v>
-      </c>
-      <c r="T72" t="s">
-        <v>866</v>
       </c>
       <c r="U72" t="s">
         <v>59</v>
@@ -9682,7 +9682,7 @@
         <v>20241055</v>
       </c>
       <c r="B73" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="C73" t="s">
         <v>163</v>
@@ -9694,7 +9694,7 @@
         <v>25</v>
       </c>
       <c r="F73" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G73" t="s">
         <v>45</v>
@@ -9703,40 +9703,40 @@
         <v>78</v>
       </c>
       <c r="I73" t="s">
+        <v>868</v>
+      </c>
+      <c r="J73" t="s">
         <v>869</v>
       </c>
-      <c r="J73" t="s">
+      <c r="K73" t="s">
         <v>870</v>
       </c>
-      <c r="K73" t="s">
+      <c r="L73" t="s">
         <v>871</v>
       </c>
-      <c r="L73" t="s">
+      <c r="M73" t="s">
         <v>872</v>
-      </c>
-      <c r="M73" t="s">
-        <v>873</v>
       </c>
       <c r="N73" t="s">
         <v>170</v>
       </c>
       <c r="O73" t="s">
+        <v>873</v>
+      </c>
+      <c r="P73" t="s">
         <v>874</v>
-      </c>
-      <c r="P73" t="s">
-        <v>875</v>
       </c>
       <c r="Q73" t="s">
         <v>55</v>
       </c>
       <c r="R73" t="s">
+        <v>875</v>
+      </c>
+      <c r="S73" t="s">
         <v>876</v>
       </c>
-      <c r="S73" t="s">
+      <c r="T73" t="s">
         <v>877</v>
-      </c>
-      <c r="T73" t="s">
-        <v>878</v>
       </c>
       <c r="U73" t="s">
         <v>59</v>
@@ -9748,19 +9748,19 @@
         <v>20244459</v>
       </c>
       <c r="B74" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="C74" t="s">
         <v>75</v>
       </c>
       <c r="D74" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="E74" t="s">
         <v>62</v>
       </c>
       <c r="F74" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G74" t="s">
         <v>45</v>
@@ -9769,40 +9769,40 @@
         <v>78</v>
       </c>
       <c r="I74" t="s">
+        <v>880</v>
+      </c>
+      <c r="J74" t="s">
         <v>881</v>
       </c>
-      <c r="J74" t="s">
+      <c r="K74" t="s">
         <v>882</v>
       </c>
-      <c r="K74" t="s">
+      <c r="L74" t="s">
         <v>883</v>
       </c>
-      <c r="L74" t="s">
+      <c r="M74" t="s">
         <v>884</v>
-      </c>
-      <c r="M74" t="s">
-        <v>885</v>
       </c>
       <c r="N74" t="s">
         <v>244</v>
       </c>
       <c r="O74" t="s">
+        <v>885</v>
+      </c>
+      <c r="P74" t="s">
         <v>886</v>
-      </c>
-      <c r="P74" t="s">
-        <v>887</v>
       </c>
       <c r="Q74" t="s">
         <v>195</v>
       </c>
       <c r="R74" t="s">
+        <v>887</v>
+      </c>
+      <c r="S74" t="s">
         <v>888</v>
       </c>
-      <c r="S74" t="s">
+      <c r="T74" t="s">
         <v>889</v>
-      </c>
-      <c r="T74" t="s">
-        <v>890</v>
       </c>
       <c r="U74" t="s">
         <v>59</v>
@@ -9814,39 +9814,39 @@
         <v>20240331</v>
       </c>
       <c r="B75" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C75" t="s">
         <v>525</v>
       </c>
       <c r="D75" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="E75"/>
       <c r="F75" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G75"/>
       <c r="H75" t="s">
         <v>78</v>
       </c>
       <c r="I75" t="s">
+        <v>892</v>
+      </c>
+      <c r="J75" t="s">
         <v>893</v>
       </c>
-      <c r="J75" t="s">
+      <c r="K75" t="s">
         <v>894</v>
       </c>
-      <c r="K75" t="s">
+      <c r="L75" t="s">
         <v>895</v>
       </c>
-      <c r="L75" t="s">
+      <c r="M75" t="s">
         <v>896</v>
       </c>
-      <c r="M75" t="s">
+      <c r="N75" t="s">
         <v>897</v>
-      </c>
-      <c r="N75" t="s">
-        <v>780</v>
       </c>
       <c r="O75" t="s">
         <v>898</v>
@@ -10046,13 +10046,13 @@
         <v>55</v>
       </c>
       <c r="R78" t="s">
+        <v>804</v>
+      </c>
+      <c r="S78" t="s">
         <v>805</v>
       </c>
-      <c r="S78" t="s">
+      <c r="T78" t="s">
         <v>806</v>
-      </c>
-      <c r="T78" t="s">
-        <v>807</v>
       </c>
       <c r="U78" t="s">
         <v>59</v>
@@ -10126,7 +10126,7 @@
         <v>525</v>
       </c>
       <c r="D80" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="E80"/>
       <c r="F80" t="s">
@@ -10188,7 +10188,7 @@
         <v>525</v>
       </c>
       <c r="D81" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="E81"/>
       <c r="F81" t="s">
@@ -10214,7 +10214,7 @@
         <v>956</v>
       </c>
       <c r="N81" t="s">
-        <v>780</v>
+        <v>897</v>
       </c>
       <c r="O81" t="s">
         <v>957</v>
@@ -11296,7 +11296,7 @@
         <v>525</v>
       </c>
       <c r="D98" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="E98"/>
       <c r="F98" t="s">
@@ -11532,13 +11532,13 @@
         <v>247</v>
       </c>
       <c r="R101" t="s">
+        <v>815</v>
+      </c>
+      <c r="S101" t="s">
         <v>816</v>
       </c>
-      <c r="S101" t="s">
+      <c r="T101" t="s">
         <v>817</v>
-      </c>
-      <c r="T101" t="s">
-        <v>818</v>
       </c>
       <c r="U101" t="s">
         <v>59</v>
@@ -12070,7 +12070,7 @@
         <v>525</v>
       </c>
       <c r="D110" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="E110"/>
       <c r="F110" t="s">
@@ -13380,7 +13380,7 @@
         <v>23</v>
       </c>
       <c r="D130" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="E130" t="s">
         <v>62</v>
@@ -13900,7 +13900,7 @@
         <v>525</v>
       </c>
       <c r="D138" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="E138"/>
       <c r="F138" t="s">

</xml_diff>

<commit_message>
Update parliament data - 2026-05-27
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -137,6 +137,57 @@
     <t xml:space="preserve">2026-05-27</t>
   </si>
   <si>
+    <t xml:space="preserve">26.3323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ip.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brenzikofer Florence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERT-E-S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WBF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hochschulfinanzierung mit alternativen Finanzierungsmodellen sichern</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quels modèles de financement pour les hautes écoles ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Garantire il finanziamento delle scuole universitarie attraverso modelli alternativi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Je prie le Conseil fédéral de répondre aux questions suivantes&amp;nbsp;:&lt;/p&gt;&lt;ol&gt;&lt;li&gt;Parmi les propositions formulées ci-dessous, lesquelles considère-t-il comme réalisables du point de vue juridique, durables du point de vue de la politique financière et équilibrées du point de vue fédéral, et sur quels éléments fonde-t-il cette appréciation&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Quelle combinaison d’instruments lui paraît appropriée pour garantir la stabilité à long terme du financement des hautes écoles&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Voit-il un moyen de facturer, dans le cadre de la péréquation financière nationale, une proportion convenue de la partie non couverte des frais liés à un étudiant issu d’un canton sans haute école&amp;nbsp;? Si oui, quelle proportion&amp;nbsp;?&lt;/li&gt;&lt;li&gt;La création d’un fonds alimenté par les éventuels excédents résultant de la distribution des bénéfices de la Banque nationale suisse (BNS), dans le strict respect de l’indépendance de la BNS et des mécanismes de distribution en vigueur, lui paraît-il une piste digne d’intérêt&amp;nbsp;? Si non, pourquoi&amp;nbsp;?&lt;/li&gt;&lt;li&gt;La création d’un fonds de compensation et de stabilité affecté afin d’atténuer les fluctuations du financement des hautes écoles dues à des facteurs structurels et à la politique financière lui paraît-elle judicieuse&amp;nbsp;?&lt;/li&gt;&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;In diesem Zusammenhang stellen sich folgende Fragen:&lt;/p&gt;&lt;ol&gt;&lt;li&gt;Welche der aufgeführten Varianten erachtet der Bundesrat als rechtlich umsetzbar, finanzpolitisch nachhaltig und föderal ausgewogen und wie begründet er seine Einschätzung?&lt;/li&gt;&lt;li&gt;Welche Kombination von Instrumenten erscheint geeignet, um die langfristige Stabilität der Hochschulfinanzierung sicherzustellen?&lt;/li&gt;&lt;li&gt;Sieht der Bundesrat im Rahmen des nationalen Finanzausgleichs (NFA) die Möglichkeit, die Unterdeckung zu den Vollkosten für einen Studierenden aus einem Nichthochschulkanton zu einem vereinbarten Teil zur Verrechnung zu bringen? Und zu welchem Teil?&lt;/li&gt;&lt;li&gt;Sieht der Bundesrat in einer Fondslösung, gespiesen aus allfälligen Ausschüttungsüberschüssen der&amp;nbsp;Schweizerischen Nationalbank, unter Wahrung der Unabhängigkeit der Nationalbank und der geltenden Ausschüttungsmechanismen, einen möglichen Weg, den es sich zu prüfen lohnt?&amp;nbsp;Falls nein, wieso nicht?&lt;/li&gt;&lt;li&gt;Könnte die Schaffung eines zweckgebundenen Ausgleichs- und Stabilitätsfonds zur Abfederung finanzpolitischer und struktureller Schwankungen in der Hochschulfinanzierung ausgleichend wirken?&lt;/li&gt;&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Élu &amp; Conseil fédéral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanzwesen|Bildung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finances|Éducation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanze|Formazione</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.3411</t>
   </si>
   <si>
@@ -197,9 +248,6 @@
     <t xml:space="preserve">26.3121</t>
   </si>
   <si>
-    <t xml:space="preserve">Ip.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Juillard Charles</t>
   </si>
   <si>
@@ -290,12 +338,6 @@
     <t xml:space="preserve">Berli Rudi</t>
   </si>
   <si>
-    <t xml:space="preserve">VERT-E-S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WBF</t>
-  </si>
-  <si>
     <t xml:space="preserve">Die Verordnung über die Branchen- und Produzentenorganisationen muss geändert werden </t>
   </si>
   <si>
@@ -335,9 +377,6 @@
     <t xml:space="preserve">Tuosto Brenda</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-19</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bahnplanung. Darf der Bundesrat die Aufträge des Parlaments ignorieren?</t>
   </si>
   <si>
@@ -359,9 +398,6 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263228</t>
   </si>
   <si>
-    <t xml:space="preserve">Élu &amp; Conseil fédéral</t>
-  </si>
-  <si>
     <t xml:space="preserve">26.3131</t>
   </si>
   <si>
@@ -630,42 +666,6 @@
   </si>
   <si>
     <t xml:space="preserve">2026-04-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.3323</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brenzikofer Florence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hochschulfinanzierung mit alternativen Finanzierungsmodellen sichern</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quels modèles de financement pour les hautes écoles ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Garantire il finanziamento delle scuole universitarie attraverso modelli alternativi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Je prie le Conseil fédéral de répondre aux questions suivantes&amp;nbsp;:&lt;/p&gt;&lt;ol&gt;&lt;li&gt;Parmi les propositions formulées ci-dessous, lesquelles considère-t-il comme réalisables du point de vue juridique, durables du point de vue de la politique financière et équilibrées du point de vue fédéral, et sur quels éléments fonde-t-il cette appréciation&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Quelle combinaison d’instruments lui paraît appropriée pour garantir la stabilité à long terme du financement des hautes écoles&amp;nbsp;?&lt;/li&gt;&lt;li&gt;Voit-il un moyen de facturer, dans le cadre de la péréquation financière nationale, une proportion convenue de la partie non couverte des frais liés à un étudiant issu d’un canton sans haute école&amp;nbsp;? Si oui, quelle proportion&amp;nbsp;?&lt;/li&gt;&lt;li&gt;La création d’un fonds alimenté par les éventuels excédents résultant de la distribution des bénéfices de la Banque nationale suisse (BNS), dans le strict respect de l’indépendance de la BNS et des mécanismes de distribution en vigueur, lui paraît-il une piste digne d’intérêt&amp;nbsp;? Si non, pourquoi&amp;nbsp;?&lt;/li&gt;&lt;li&gt;La création d’un fonds de compensation et de stabilité affecté afin d’atténuer les fluctuations du financement des hautes écoles dues à des facteurs structurels et à la politique financière lui paraît-elle judicieuse&amp;nbsp;?&lt;/li&gt;&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;In diesem Zusammenhang stellen sich folgende Fragen:&lt;/p&gt;&lt;ol&gt;&lt;li&gt;Welche der aufgeführten Varianten erachtet der Bundesrat als rechtlich umsetzbar, finanzpolitisch nachhaltig und föderal ausgewogen und wie begründet er seine Einschätzung?&lt;/li&gt;&lt;li&gt;Welche Kombination von Instrumenten erscheint geeignet, um die langfristige Stabilität der Hochschulfinanzierung sicherzustellen?&lt;/li&gt;&lt;li&gt;Sieht der Bundesrat im Rahmen des nationalen Finanzausgleichs (NFA) die Möglichkeit, die Unterdeckung zu den Vollkosten für einen Studierenden aus einem Nichthochschulkanton zu einem vereinbarten Teil zur Verrechnung zu bringen? Und zu welchem Teil?&lt;/li&gt;&lt;li&gt;Sieht der Bundesrat in einer Fondslösung, gespiesen aus allfälligen Ausschüttungsüberschüssen der&amp;nbsp;Schweizerischen Nationalbank, unter Wahrung der Unabhängigkeit der Nationalbank und der geltenden Ausschüttungsmechanismen, einen möglichen Weg, den es sich zu prüfen lohnt?&amp;nbsp;Falls nein, wieso nicht?&lt;/li&gt;&lt;li&gt;Könnte die Schaffung eines zweckgebundenen Ausgleichs- und Stabilitätsfonds zur Abfederung finanzpolitischer und struktureller Schwankungen in der Hochschulfinanzierung ausgleichend wirken?&lt;/li&gt;&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263323</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263323</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanzwesen|Bildung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finances|Éducation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanze|Formazione</t>
   </si>
   <si>
     <t xml:space="preserve">26.7194</t>
@@ -5242,25 +5242,25 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>20263411</v>
+        <v>20263323</v>
       </c>
       <c r="B3" t="s">
         <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G3" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="H3" t="s">
         <v>46</v>
@@ -5281,82 +5281,82 @@
         <v>51</v>
       </c>
       <c r="N3" t="s">
+        <v>33</v>
+      </c>
+      <c r="O3" t="s">
         <v>52</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>53</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>54</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>55</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>56</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>57</v>
       </c>
-      <c r="T3" t="s">
-        <v>58</v>
-      </c>
       <c r="U3" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="V3"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20263121</v>
+        <v>20263411</v>
       </c>
       <c r="B4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
         <v>60</v>
       </c>
-      <c r="C4" t="s">
+      <c r="F4" t="s">
         <v>61</v>
       </c>
-      <c r="D4" t="s">
+      <c r="G4" t="s">
         <v>62</v>
       </c>
-      <c r="E4" t="s">
+      <c r="H4" t="s">
         <v>63</v>
       </c>
-      <c r="F4" t="s">
+      <c r="I4" t="s">
         <v>64</v>
       </c>
-      <c r="G4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>65</v>
       </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>66</v>
       </c>
-      <c r="J4" t="s">
+      <c r="L4" t="s">
         <v>67</v>
       </c>
-      <c r="K4" t="s">
+      <c r="M4" t="s">
         <v>68</v>
       </c>
-      <c r="L4" t="s">
+      <c r="N4" t="s">
         <v>69</v>
       </c>
-      <c r="M4" t="s">
+      <c r="O4" t="s">
         <v>70</v>
       </c>
-      <c r="N4" t="s">
-        <v>52</v>
-      </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>71</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>72</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>55</v>
       </c>
       <c r="R4" t="s">
         <v>73</v>
@@ -5368,166 +5368,166 @@
         <v>75</v>
       </c>
       <c r="U4" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="V4"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20263099</v>
+        <v>20263121</v>
       </c>
       <c r="B5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E5" t="s">
+        <v>79</v>
+      </c>
+      <c r="F5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G5" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I5" t="s">
+        <v>82</v>
+      </c>
+      <c r="J5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K5" t="s">
+        <v>84</v>
+      </c>
+      <c r="L5" t="s">
+        <v>85</v>
+      </c>
+      <c r="M5" t="s">
+        <v>86</v>
+      </c>
+      <c r="N5" t="s">
+        <v>69</v>
+      </c>
+      <c r="O5" t="s">
+        <v>87</v>
+      </c>
+      <c r="P5" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>72</v>
+      </c>
+      <c r="R5" t="s">
+        <v>89</v>
+      </c>
+      <c r="S5" t="s">
+        <v>90</v>
+      </c>
+      <c r="T5" t="s">
+        <v>91</v>
+      </c>
+      <c r="U5" t="s">
         <v>76</v>
-      </c>
-      <c r="C5" t="s">
-        <v>77</v>
-      </c>
-      <c r="D5" t="s">
-        <v>62</v>
-      </c>
-      <c r="E5" t="s">
-        <v>63</v>
-      </c>
-      <c r="F5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H5" t="s">
-        <v>79</v>
-      </c>
-      <c r="I5" t="s">
-        <v>80</v>
-      </c>
-      <c r="J5" t="s">
-        <v>81</v>
-      </c>
-      <c r="K5" t="s">
-        <v>82</v>
-      </c>
-      <c r="L5" t="s">
-        <v>83</v>
-      </c>
-      <c r="M5" t="s">
-        <v>84</v>
-      </c>
-      <c r="N5" t="s">
-        <v>52</v>
-      </c>
-      <c r="O5" t="s">
-        <v>85</v>
-      </c>
-      <c r="P5" t="s">
-        <v>86</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>55</v>
-      </c>
-      <c r="R5" t="s">
-        <v>87</v>
-      </c>
-      <c r="S5" t="s">
-        <v>88</v>
-      </c>
-      <c r="T5" t="s">
-        <v>89</v>
-      </c>
-      <c r="U5" t="s">
-        <v>59</v>
       </c>
       <c r="V5"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>20263497</v>
+        <v>20263099</v>
       </c>
       <c r="B6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>93</v>
       </c>
       <c r="D6" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="E6" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="F6" t="s">
-        <v>44</v>
+        <v>94</v>
       </c>
       <c r="G6" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="H6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="L6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="M6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="N6" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="O6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="P6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="Q6" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="R6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="S6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="T6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="U6" t="s">
-        <v>104</v>
+        <v>76</v>
       </c>
       <c r="V6"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>20263228</v>
+        <v>20263497</v>
       </c>
       <c r="B7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" t="s">
         <v>61</v>
-      </c>
-      <c r="D7" t="s">
-        <v>106</v>
-      </c>
-      <c r="E7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F7" t="s">
-        <v>107</v>
       </c>
       <c r="G7" t="s">
         <v>26</v>
       </c>
       <c r="H7" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="I7" t="s">
         <v>108</v>
@@ -5554,135 +5554,137 @@
         <v>114</v>
       </c>
       <c r="Q7" t="s">
+        <v>36</v>
+      </c>
+      <c r="R7" t="s">
         <v>115</v>
       </c>
-      <c r="R7" t="s">
-        <v>73</v>
-      </c>
       <c r="S7" t="s">
-        <v>74</v>
+        <v>116</v>
       </c>
       <c r="T7" t="s">
-        <v>75</v>
+        <v>117</v>
       </c>
       <c r="U7" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="V7"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>20263131</v>
+        <v>20263228</v>
       </c>
       <c r="B8" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
-        <v>117</v>
-      </c>
-      <c r="E8"/>
+        <v>120</v>
+      </c>
+      <c r="E8" t="s">
+        <v>60</v>
+      </c>
       <c r="F8" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="G8" t="s">
         <v>26</v>
       </c>
       <c r="H8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I8" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="J8" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="K8" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="L8" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="M8" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="N8" t="s">
         <v>33</v>
       </c>
       <c r="O8" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="P8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="Q8" t="s">
-        <v>125</v>
+        <v>54</v>
       </c>
       <c r="R8" t="s">
-        <v>126</v>
+        <v>89</v>
       </c>
       <c r="S8" t="s">
-        <v>127</v>
+        <v>90</v>
       </c>
       <c r="T8" t="s">
-        <v>128</v>
+        <v>91</v>
       </c>
       <c r="U8" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="V8"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>20263374</v>
+        <v>20263131</v>
       </c>
       <c r="B9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C9" t="s">
         <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="G9" t="s">
         <v>26</v>
       </c>
       <c r="H9" t="s">
-        <v>27</v>
+        <v>95</v>
       </c>
       <c r="I9" t="s">
+        <v>130</v>
+      </c>
+      <c r="J9" t="s">
         <v>131</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>132</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>133</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>134</v>
-      </c>
-      <c r="M9" t="s">
-        <v>135</v>
       </c>
       <c r="N9" t="s">
         <v>33</v>
       </c>
       <c r="O9" t="s">
+        <v>135</v>
+      </c>
+      <c r="P9" t="s">
         <v>136</v>
       </c>
-      <c r="P9" t="s">
+      <c r="Q9" t="s">
         <v>137</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>115</v>
       </c>
       <c r="R9" t="s">
         <v>138</v>
@@ -5694,166 +5696,164 @@
         <v>140</v>
       </c>
       <c r="U9" t="s">
-        <v>141</v>
+        <v>118</v>
       </c>
       <c r="V9"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>20263454</v>
+        <v>20263374</v>
       </c>
       <c r="B10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
         <v>142</v>
       </c>
-      <c r="C10" t="s">
+      <c r="E10"/>
+      <c r="F10" t="s">
         <v>61</v>
-      </c>
-      <c r="D10" t="s">
-        <v>143</v>
-      </c>
-      <c r="E10" t="s">
-        <v>144</v>
-      </c>
-      <c r="F10" t="s">
-        <v>44</v>
       </c>
       <c r="G10" t="s">
         <v>26</v>
       </c>
       <c r="H10" t="s">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="I10" t="s">
+        <v>143</v>
+      </c>
+      <c r="J10" t="s">
+        <v>144</v>
+      </c>
+      <c r="K10" t="s">
         <v>145</v>
       </c>
-      <c r="J10" t="s">
+      <c r="L10" t="s">
         <v>146</v>
       </c>
-      <c r="K10" t="s">
+      <c r="M10" t="s">
         <v>147</v>
-      </c>
-      <c r="L10" t="s">
-        <v>148</v>
-      </c>
-      <c r="M10" t="s">
-        <v>149</v>
       </c>
       <c r="N10" t="s">
         <v>33</v>
       </c>
       <c r="O10" t="s">
+        <v>148</v>
+      </c>
+      <c r="P10" t="s">
+        <v>149</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>54</v>
+      </c>
+      <c r="R10" t="s">
         <v>150</v>
       </c>
-      <c r="P10" t="s">
+      <c r="S10" t="s">
         <v>151</v>
       </c>
-      <c r="Q10" t="s">
-        <v>55</v>
-      </c>
-      <c r="R10" t="s">
+      <c r="T10" t="s">
         <v>152</v>
       </c>
-      <c r="S10" t="s">
+      <c r="U10" t="s">
         <v>153</v>
-      </c>
-      <c r="T10" t="s">
-        <v>154</v>
-      </c>
-      <c r="U10" t="s">
-        <v>141</v>
       </c>
       <c r="V10"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>20263192</v>
+        <v>20263454</v>
       </c>
       <c r="B11" t="s">
+        <v>154</v>
+      </c>
+      <c r="C11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" t="s">
         <v>155</v>
       </c>
-      <c r="C11" t="s">
+      <c r="E11" t="s">
+        <v>156</v>
+      </c>
+      <c r="F11" t="s">
         <v>61</v>
-      </c>
-      <c r="D11" t="s">
-        <v>156</v>
-      </c>
-      <c r="E11" t="s">
-        <v>144</v>
-      </c>
-      <c r="F11" t="s">
-        <v>157</v>
       </c>
       <c r="G11" t="s">
         <v>26</v>
       </c>
       <c r="H11" t="s">
+        <v>81</v>
+      </c>
+      <c r="I11" t="s">
+        <v>157</v>
+      </c>
+      <c r="J11" t="s">
         <v>158</v>
       </c>
-      <c r="I11" t="s">
+      <c r="K11" t="s">
         <v>159</v>
       </c>
-      <c r="J11" t="s">
+      <c r="L11" t="s">
         <v>160</v>
       </c>
-      <c r="K11" t="s">
+      <c r="M11" t="s">
         <v>161</v>
-      </c>
-      <c r="L11" t="s">
-        <v>162</v>
-      </c>
-      <c r="M11" t="s">
-        <v>163</v>
       </c>
       <c r="N11" t="s">
         <v>33</v>
       </c>
       <c r="O11" t="s">
+        <v>162</v>
+      </c>
+      <c r="P11" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>72</v>
+      </c>
+      <c r="R11" t="s">
         <v>164</v>
       </c>
-      <c r="P11" t="s">
+      <c r="S11" t="s">
         <v>165</v>
       </c>
-      <c r="Q11" t="s">
-        <v>36</v>
-      </c>
-      <c r="R11" t="s">
+      <c r="T11" t="s">
         <v>166</v>
       </c>
-      <c r="S11" t="s">
-        <v>167</v>
-      </c>
-      <c r="T11" t="s">
-        <v>168</v>
-      </c>
       <c r="U11" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="V11"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>20263120</v>
+        <v>20263192</v>
       </c>
       <c r="B12" t="s">
+        <v>167</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" t="s">
+        <v>168</v>
+      </c>
+      <c r="E12" t="s">
+        <v>156</v>
+      </c>
+      <c r="F12" t="s">
         <v>169</v>
-      </c>
-      <c r="C12" t="s">
-        <v>23</v>
-      </c>
-      <c r="D12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E12" t="s">
-        <v>144</v>
-      </c>
-      <c r="F12" t="s">
-        <v>64</v>
       </c>
       <c r="G12" t="s">
         <v>26</v>
       </c>
       <c r="H12" t="s">
-        <v>46</v>
+        <v>170</v>
       </c>
       <c r="I12" t="s">
         <v>171</v>
@@ -5880,7 +5880,7 @@
         <v>177</v>
       </c>
       <c r="Q12" t="s">
-        <v>125</v>
+        <v>36</v>
       </c>
       <c r="R12" t="s">
         <v>178</v>
@@ -5892,209 +5892,207 @@
         <v>180</v>
       </c>
       <c r="U12" t="s">
-        <v>181</v>
+        <v>153</v>
       </c>
       <c r="V12"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>20263069</v>
+        <v>20263120</v>
       </c>
       <c r="B13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" t="s">
         <v>182</v>
       </c>
-      <c r="C13" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13" t="s">
-        <v>183</v>
-      </c>
       <c r="E13" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F13" t="s">
-        <v>184</v>
+        <v>80</v>
       </c>
       <c r="G13" t="s">
         <v>26</v>
       </c>
       <c r="H13" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I13" t="s">
+        <v>183</v>
+      </c>
+      <c r="J13" t="s">
+        <v>184</v>
+      </c>
+      <c r="K13" t="s">
         <v>185</v>
       </c>
-      <c r="J13" t="s">
+      <c r="L13" t="s">
         <v>186</v>
       </c>
-      <c r="K13" t="s">
+      <c r="M13" t="s">
         <v>187</v>
-      </c>
-      <c r="L13" t="s">
-        <v>188</v>
-      </c>
-      <c r="M13" t="s">
-        <v>189</v>
       </c>
       <c r="N13" t="s">
         <v>33</v>
       </c>
       <c r="O13" t="s">
+        <v>188</v>
+      </c>
+      <c r="P13" t="s">
+        <v>189</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>137</v>
+      </c>
+      <c r="R13" t="s">
         <v>190</v>
       </c>
-      <c r="P13" t="s">
+      <c r="S13" t="s">
         <v>191</v>
       </c>
-      <c r="Q13" t="s">
-        <v>115</v>
-      </c>
-      <c r="R13" t="s">
-        <v>152</v>
-      </c>
-      <c r="S13" t="s">
-        <v>153</v>
-      </c>
       <c r="T13" t="s">
-        <v>154</v>
+        <v>192</v>
       </c>
       <c r="U13" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="V13"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>20254774</v>
+        <v>20263069</v>
       </c>
       <c r="B14" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C14" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>62</v>
+        <v>195</v>
       </c>
       <c r="E14" t="s">
-        <v>63</v>
+        <v>156</v>
       </c>
       <c r="F14" t="s">
+        <v>196</v>
+      </c>
+      <c r="G14" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" t="s">
+        <v>81</v>
+      </c>
+      <c r="I14" t="s">
+        <v>197</v>
+      </c>
+      <c r="J14" t="s">
+        <v>198</v>
+      </c>
+      <c r="K14" t="s">
+        <v>199</v>
+      </c>
+      <c r="L14" t="s">
+        <v>200</v>
+      </c>
+      <c r="M14" t="s">
+        <v>201</v>
+      </c>
+      <c r="N14" t="s">
+        <v>33</v>
+      </c>
+      <c r="O14" t="s">
+        <v>202</v>
+      </c>
+      <c r="P14" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>54</v>
+      </c>
+      <c r="R14" t="s">
+        <v>164</v>
+      </c>
+      <c r="S14" t="s">
+        <v>165</v>
+      </c>
+      <c r="T14" t="s">
+        <v>166</v>
+      </c>
+      <c r="U14" t="s">
         <v>193</v>
-      </c>
-      <c r="G14" t="s">
-        <v>45</v>
-      </c>
-      <c r="H14" t="s">
-        <v>79</v>
-      </c>
-      <c r="I14" t="s">
-        <v>194</v>
-      </c>
-      <c r="J14" t="s">
-        <v>195</v>
-      </c>
-      <c r="K14" t="s">
-        <v>196</v>
-      </c>
-      <c r="L14" t="s">
-        <v>197</v>
-      </c>
-      <c r="M14" t="s">
-        <v>198</v>
-      </c>
-      <c r="N14" t="s">
-        <v>199</v>
-      </c>
-      <c r="O14" t="s">
-        <v>200</v>
-      </c>
-      <c r="P14" t="s">
-        <v>201</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>55</v>
-      </c>
-      <c r="R14" t="s">
-        <v>202</v>
-      </c>
-      <c r="S14" t="s">
-        <v>203</v>
-      </c>
-      <c r="T14" t="s">
-        <v>204</v>
-      </c>
-      <c r="U14" t="s">
-        <v>205</v>
       </c>
       <c r="V14"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>20263323</v>
+        <v>20254774</v>
       </c>
       <c r="B15" t="s">
+        <v>204</v>
+      </c>
+      <c r="C15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" t="s">
+        <v>205</v>
+      </c>
+      <c r="G15" t="s">
+        <v>62</v>
+      </c>
+      <c r="H15" t="s">
+        <v>95</v>
+      </c>
+      <c r="I15" t="s">
         <v>206</v>
       </c>
-      <c r="C15" t="s">
-        <v>61</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="J15" t="s">
         <v>207</v>
       </c>
-      <c r="E15" t="s">
-        <v>92</v>
-      </c>
-      <c r="F15" t="s">
-        <v>107</v>
-      </c>
-      <c r="G15" t="s">
-        <v>26</v>
-      </c>
-      <c r="H15" t="s">
-        <v>93</v>
-      </c>
-      <c r="I15" t="s">
+      <c r="K15" t="s">
         <v>208</v>
       </c>
-      <c r="J15" t="s">
+      <c r="L15" t="s">
         <v>209</v>
       </c>
-      <c r="K15" t="s">
+      <c r="M15" t="s">
         <v>210</v>
       </c>
-      <c r="L15" t="s">
+      <c r="N15" t="s">
         <v>211</v>
       </c>
-      <c r="M15" t="s">
+      <c r="O15" t="s">
         <v>212</v>
       </c>
-      <c r="N15" t="s">
-        <v>33</v>
-      </c>
-      <c r="O15" t="s">
+      <c r="P15" t="s">
         <v>213</v>
       </c>
-      <c r="P15" t="s">
+      <c r="Q15" t="s">
+        <v>72</v>
+      </c>
+      <c r="R15" t="s">
         <v>214</v>
       </c>
-      <c r="Q15" t="s">
-        <v>115</v>
-      </c>
-      <c r="R15" t="s">
+      <c r="S15" t="s">
         <v>215</v>
       </c>
-      <c r="S15" t="s">
+      <c r="T15" t="s">
         <v>216</v>
       </c>
-      <c r="T15" t="s">
+      <c r="U15" t="s">
         <v>217</v>
       </c>
-      <c r="U15" t="s">
-        <v>40</v>
-      </c>
-      <c r="V15" t="s">
-        <v>40</v>
-      </c>
+      <c r="V15"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -6110,7 +6108,7 @@
         <v>220</v>
       </c>
       <c r="E16" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F16" t="s">
         <v>221</v>
@@ -6119,7 +6117,7 @@
         <v>26</v>
       </c>
       <c r="H16" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="I16" t="s">
         <v>222</v>
@@ -6144,7 +6142,7 @@
         <v>228</v>
       </c>
       <c r="Q16" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="R16" t="s">
         <v>229</v>
@@ -6177,13 +6175,13 @@
         <v>235</v>
       </c>
       <c r="F17" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="G17" t="s">
         <v>26</v>
       </c>
       <c r="H17" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I17" t="s">
         <v>236</v>
@@ -6241,7 +6239,7 @@
       </c>
       <c r="G18"/>
       <c r="H18" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I18" t="s">
         <v>248</v>
@@ -6264,16 +6262,16 @@
         <v>253</v>
       </c>
       <c r="Q18" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="R18" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="S18" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="T18" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="U18" t="s">
         <v>232</v>
@@ -6291,10 +6289,10 @@
         <v>219</v>
       </c>
       <c r="D19" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="E19" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F19" t="s">
         <v>255</v>
@@ -6303,7 +6301,7 @@
         <v>26</v>
       </c>
       <c r="H19" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I19" t="s">
         <v>256</v>
@@ -6328,7 +6326,7 @@
         <v>261</v>
       </c>
       <c r="Q19" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R19" t="s">
         <v>262</v>
@@ -6392,7 +6390,7 @@
         <v>274</v>
       </c>
       <c r="Q20" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R20" t="s">
         <v>275</v>
@@ -6416,7 +6414,7 @@
         <v>278</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
         <v>279</v>
@@ -6425,7 +6423,7 @@
         <v>280</v>
       </c>
       <c r="F21" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="G21" t="s">
         <v>26</v>
@@ -6458,7 +6456,7 @@
         <v>287</v>
       </c>
       <c r="Q21" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R21" t="s">
         <v>288</v>
@@ -6482,22 +6480,22 @@
         <v>291</v>
       </c>
       <c r="C22" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D22" t="s">
         <v>292</v>
       </c>
       <c r="E22" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F22" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="G22" t="s">
         <v>26</v>
       </c>
       <c r="H22" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I22" t="s">
         <v>293</v>
@@ -6551,16 +6549,16 @@
         <v>23</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="E23" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F23" t="s">
         <v>304</v>
       </c>
       <c r="G23" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H23" t="s">
         <v>305</v>
@@ -6590,7 +6588,7 @@
         <v>313</v>
       </c>
       <c r="Q23" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="R23" t="s">
         <v>314</v>
@@ -6614,22 +6612,22 @@
         <v>317</v>
       </c>
       <c r="C24" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="D24" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="E24" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F24" t="s">
         <v>304</v>
       </c>
       <c r="G24" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H24" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I24" t="s">
         <v>318</v>
@@ -6656,7 +6654,7 @@
         <v>325</v>
       </c>
       <c r="Q24" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="R24" t="s">
         <v>326</v>
@@ -6680,19 +6678,19 @@
         <v>329</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D25" t="s">
         <v>330</v>
       </c>
       <c r="E25" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F25" t="s">
         <v>331</v>
       </c>
       <c r="G25" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H25" t="s">
         <v>27</v>
@@ -6749,10 +6747,10 @@
         <v>23</v>
       </c>
       <c r="D26" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="E26" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F26" t="s">
         <v>343</v>
@@ -6812,13 +6810,13 @@
         <v>351</v>
       </c>
       <c r="C27" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D27" t="s">
         <v>220</v>
       </c>
       <c r="E27" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F27" t="s">
         <v>343</v>
@@ -6827,7 +6825,7 @@
         <v>26</v>
       </c>
       <c r="H27" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I27" t="s">
         <v>352</v>
@@ -6854,7 +6852,7 @@
         <v>358</v>
       </c>
       <c r="Q27" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="R27" t="s">
         <v>359</v>
@@ -6884,7 +6882,7 @@
         <v>363</v>
       </c>
       <c r="E28" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F28" t="s">
         <v>364</v>
@@ -6918,7 +6916,7 @@
         <v>370</v>
       </c>
       <c r="Q28" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R28" t="s">
         <v>371</v>
@@ -6945,10 +6943,10 @@
         <v>219</v>
       </c>
       <c r="D29" t="s">
+        <v>168</v>
+      </c>
+      <c r="E29" t="s">
         <v>156</v>
-      </c>
-      <c r="E29" t="s">
-        <v>144</v>
       </c>
       <c r="F29" t="s">
         <v>364</v>
@@ -6957,7 +6955,7 @@
         <v>26</v>
       </c>
       <c r="H29" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I29" t="s">
         <v>375</v>
@@ -6982,16 +6980,16 @@
         <v>380</v>
       </c>
       <c r="Q29" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R29" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="S29" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="T29" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="U29" t="s">
         <v>232</v>
@@ -7006,7 +7004,7 @@
         <v>381</v>
       </c>
       <c r="C30" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="D30" t="s">
         <v>382</v>
@@ -7019,7 +7017,7 @@
         <v>26</v>
       </c>
       <c r="H30" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I30" t="s">
         <v>384</v>
@@ -7046,7 +7044,7 @@
         <v>390</v>
       </c>
       <c r="Q30" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R30" t="s">
         <v>391</v>
@@ -7076,13 +7074,13 @@
         <v>395</v>
       </c>
       <c r="E31" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F31" t="s">
         <v>396</v>
       </c>
       <c r="G31" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H31" t="s">
         <v>27</v>
@@ -7112,7 +7110,7 @@
         <v>403</v>
       </c>
       <c r="Q31" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R31" t="s">
         <v>404</v>
@@ -7136,13 +7134,13 @@
         <v>407</v>
       </c>
       <c r="C32" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="D32" t="s">
         <v>408</v>
       </c>
       <c r="E32" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F32" t="s">
         <v>396</v>
@@ -7178,16 +7176,16 @@
         <v>415</v>
       </c>
       <c r="Q32" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R32" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="S32" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="T32" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="U32" t="s">
         <v>232</v>
@@ -7202,13 +7200,13 @@
         <v>416</v>
       </c>
       <c r="C33" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D33" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="E33" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F33" t="s">
         <v>396</v>
@@ -7217,7 +7215,7 @@
         <v>26</v>
       </c>
       <c r="H33" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I33" t="s">
         <v>417</v>
@@ -7244,16 +7242,16 @@
         <v>423</v>
       </c>
       <c r="Q33" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R33" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="S33" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="T33" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="U33" t="s">
         <v>232</v>
@@ -7271,19 +7269,19 @@
         <v>23</v>
       </c>
       <c r="D34" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="E34" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F34" t="s">
         <v>396</v>
       </c>
       <c r="G34" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H34" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I34" t="s">
         <v>425</v>
@@ -7310,7 +7308,7 @@
         <v>431</v>
       </c>
       <c r="Q34" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="R34" t="s">
         <v>432</v>
@@ -7334,13 +7332,13 @@
         <v>435</v>
       </c>
       <c r="C35" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D35" t="s">
         <v>436</v>
       </c>
       <c r="E35" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F35" t="s">
         <v>437</v>
@@ -7376,7 +7374,7 @@
         <v>444</v>
       </c>
       <c r="Q35" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R35" t="s">
         <v>288</v>
@@ -7400,22 +7398,22 @@
         <v>445</v>
       </c>
       <c r="C36" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D36" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="E36" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F36" t="s">
         <v>446</v>
       </c>
       <c r="G36" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H36" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="I36" t="s">
         <v>447</v>
@@ -7442,7 +7440,7 @@
         <v>453</v>
       </c>
       <c r="Q36" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R36" t="s">
         <v>454</v>
@@ -7466,13 +7464,13 @@
         <v>457</v>
       </c>
       <c r="C37" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D37" t="s">
         <v>458</v>
       </c>
       <c r="E37" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F37" t="s">
         <v>446</v>
@@ -7532,19 +7530,19 @@
         <v>469</v>
       </c>
       <c r="C38" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D38" t="s">
         <v>470</v>
       </c>
       <c r="E38" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F38" t="s">
         <v>471</v>
       </c>
       <c r="G38" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H38" t="s">
         <v>27</v>
@@ -7574,7 +7572,7 @@
         <v>478</v>
       </c>
       <c r="Q38" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R38" t="s">
         <v>479</v>
@@ -7601,10 +7599,10 @@
         <v>483</v>
       </c>
       <c r="D39" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="E39" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F39" t="s">
         <v>484</v>
@@ -7640,7 +7638,7 @@
         <v>492</v>
       </c>
       <c r="Q39" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="R39" t="s">
         <v>493</v>
@@ -7679,7 +7677,7 @@
         <v>26</v>
       </c>
       <c r="H40" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I40" t="s">
         <v>499</v>
@@ -7706,7 +7704,7 @@
         <v>505</v>
       </c>
       <c r="Q40" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R40" t="s">
         <v>506</v>
@@ -7770,7 +7768,7 @@
         <v>517</v>
       </c>
       <c r="Q41" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R41" t="s">
         <v>288</v>
@@ -7800,7 +7798,7 @@
         <v>519</v>
       </c>
       <c r="E42" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F42" t="s">
         <v>498</v>
@@ -7809,7 +7807,7 @@
         <v>26</v>
       </c>
       <c r="H42" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="I42" t="s">
         <v>520</v>
@@ -7864,7 +7862,7 @@
         <v>458</v>
       </c>
       <c r="E43" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F43" t="s">
         <v>530</v>
@@ -7873,7 +7871,7 @@
         <v>26</v>
       </c>
       <c r="H43" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I43" t="s">
         <v>531</v>
@@ -7898,7 +7896,7 @@
         <v>536</v>
       </c>
       <c r="Q43" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R43" t="s">
         <v>537</v>
@@ -7922,13 +7920,13 @@
         <v>540</v>
       </c>
       <c r="C44" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D44" t="s">
         <v>541</v>
       </c>
       <c r="E44" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F44" t="s">
         <v>542</v>
@@ -7964,7 +7962,7 @@
         <v>549</v>
       </c>
       <c r="Q44" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R44" t="s">
         <v>550</v>
@@ -7994,7 +7992,7 @@
         <v>541</v>
       </c>
       <c r="E45" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F45" t="s">
         <v>542</v>
@@ -8028,7 +8026,7 @@
         <v>559</v>
       </c>
       <c r="Q45" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R45" t="s">
         <v>560</v>
@@ -8090,7 +8088,7 @@
         <v>574</v>
       </c>
       <c r="Q46" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R46"/>
       <c r="S46"/>
@@ -8108,13 +8106,13 @@
         <v>575</v>
       </c>
       <c r="C47" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D47" t="s">
         <v>576</v>
       </c>
       <c r="E47" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F47" t="s">
         <v>577</v>
@@ -8123,7 +8121,7 @@
         <v>26</v>
       </c>
       <c r="H47" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I47" t="s">
         <v>578</v>
@@ -8174,13 +8172,13 @@
         <v>588</v>
       </c>
       <c r="C48" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D48" t="s">
         <v>589</v>
       </c>
       <c r="E48" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F48" t="s">
         <v>577</v>
@@ -8189,7 +8187,7 @@
         <v>26</v>
       </c>
       <c r="H48" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I48" t="s">
         <v>590</v>
@@ -8216,7 +8214,7 @@
         <v>596</v>
       </c>
       <c r="Q48" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R48" t="s">
         <v>597</v>
@@ -8240,13 +8238,13 @@
         <v>600</v>
       </c>
       <c r="C49" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="D49" t="s">
         <v>601</v>
       </c>
       <c r="E49" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F49" t="s">
         <v>577</v>
@@ -8282,7 +8280,7 @@
         <v>609</v>
       </c>
       <c r="Q49" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R49" t="s">
         <v>610</v>
@@ -8309,7 +8307,7 @@
         <v>23</v>
       </c>
       <c r="D50" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="E50"/>
       <c r="F50" t="s">
@@ -8346,7 +8344,7 @@
         <v>621</v>
       </c>
       <c r="Q50" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R50" t="s">
         <v>622</v>
@@ -8370,13 +8368,13 @@
         <v>625</v>
       </c>
       <c r="C51" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D51" t="s">
         <v>626</v>
       </c>
       <c r="E51" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F51" t="s">
         <v>614</v>
@@ -8385,7 +8383,7 @@
         <v>26</v>
       </c>
       <c r="H51" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I51" t="s">
         <v>627</v>
@@ -8436,13 +8434,13 @@
         <v>637</v>
       </c>
       <c r="C52" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D52" t="s">
         <v>638</v>
       </c>
       <c r="E52" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F52" t="s">
         <v>639</v>
@@ -8451,7 +8449,7 @@
         <v>26</v>
       </c>
       <c r="H52" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I52" t="s">
         <v>640</v>
@@ -8478,16 +8476,16 @@
         <v>646</v>
       </c>
       <c r="Q52" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R52" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="S52" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="T52" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="U52" t="s">
         <v>232</v>
@@ -8502,7 +8500,7 @@
         <v>647</v>
       </c>
       <c r="C53" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="D53" t="s">
         <v>648</v>
@@ -8515,7 +8513,7 @@
         <v>26</v>
       </c>
       <c r="H53" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I53" t="s">
         <v>649</v>
@@ -8542,7 +8540,7 @@
         <v>655</v>
       </c>
       <c r="Q53" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R53" t="s">
         <v>656</v>
@@ -8566,13 +8564,13 @@
         <v>659</v>
       </c>
       <c r="C54" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D54" t="s">
         <v>408</v>
       </c>
       <c r="E54" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F54" t="s">
         <v>639</v>
@@ -8581,7 +8579,7 @@
         <v>26</v>
       </c>
       <c r="H54" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I54" t="s">
         <v>660</v>
@@ -8608,7 +8606,7 @@
         <v>666</v>
       </c>
       <c r="Q54" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R54" t="s">
         <v>667</v>
@@ -8632,7 +8630,7 @@
         <v>670</v>
       </c>
       <c r="C55" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D55" t="s">
         <v>671</v>
@@ -8644,10 +8642,10 @@
         <v>672</v>
       </c>
       <c r="G55" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H55" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I55" t="s">
         <v>673</v>
@@ -8674,7 +8672,7 @@
         <v>679</v>
       </c>
       <c r="Q55" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R55" t="s">
         <v>585</v>
@@ -8704,7 +8702,7 @@
         <v>681</v>
       </c>
       <c r="E56" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F56" t="s">
         <v>682</v>
@@ -8713,7 +8711,7 @@
         <v>26</v>
       </c>
       <c r="H56" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I56" t="s">
         <v>683</v>
@@ -8740,16 +8738,16 @@
         <v>689</v>
       </c>
       <c r="Q56" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R56" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="S56" t="s">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="T56" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="U56" t="s">
         <v>232</v>
@@ -8836,7 +8834,7 @@
         <v>458</v>
       </c>
       <c r="E58" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F58" t="s">
         <v>693</v>
@@ -8872,7 +8870,7 @@
         <v>711</v>
       </c>
       <c r="Q58" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R58" t="s">
         <v>712</v>
@@ -8936,7 +8934,7 @@
         <v>723</v>
       </c>
       <c r="Q59" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R59" t="s">
         <v>712</v>
@@ -8960,13 +8958,13 @@
         <v>724</v>
       </c>
       <c r="C60" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="D60" t="s">
         <v>725</v>
       </c>
       <c r="E60" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F60" t="s">
         <v>726</v>
@@ -9002,7 +9000,7 @@
         <v>734</v>
       </c>
       <c r="Q60" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R60" t="s">
         <v>735</v>
@@ -9026,13 +9024,13 @@
         <v>738</v>
       </c>
       <c r="C61" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D61" t="s">
         <v>739</v>
       </c>
       <c r="E61" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F61" t="s">
         <v>726</v>
@@ -9041,7 +9039,7 @@
         <v>26</v>
       </c>
       <c r="H61" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I61" t="s">
         <v>740</v>
@@ -9068,7 +9066,7 @@
         <v>746</v>
       </c>
       <c r="Q61" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R61" t="s">
         <v>747</v>
@@ -9092,13 +9090,13 @@
         <v>750</v>
       </c>
       <c r="C62" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D62" t="s">
         <v>751</v>
       </c>
       <c r="E62" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F62" t="s">
         <v>726</v>
@@ -9107,7 +9105,7 @@
         <v>26</v>
       </c>
       <c r="H62" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I62" t="s">
         <v>752</v>
@@ -9164,16 +9162,16 @@
         <v>760</v>
       </c>
       <c r="E63" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F63" t="s">
         <v>761</v>
       </c>
       <c r="G63" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H63" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I63" t="s">
         <v>762</v>
@@ -9200,7 +9198,7 @@
         <v>768</v>
       </c>
       <c r="Q63" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R63" t="s">
         <v>769</v>
@@ -9227,16 +9225,16 @@
         <v>23</v>
       </c>
       <c r="D64" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="E64" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F64" t="s">
         <v>761</v>
       </c>
       <c r="G64" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H64" t="s">
         <v>27</v>
@@ -9266,7 +9264,7 @@
         <v>779</v>
       </c>
       <c r="Q64" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R64" t="s">
         <v>712</v>
@@ -9290,22 +9288,22 @@
         <v>780</v>
       </c>
       <c r="C65" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D65" t="s">
         <v>330</v>
       </c>
       <c r="E65" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F65" t="s">
         <v>781</v>
       </c>
       <c r="G65" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H65" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I65" t="s">
         <v>782</v>
@@ -9356,13 +9354,13 @@
         <v>792</v>
       </c>
       <c r="C66" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D66" t="s">
         <v>626</v>
       </c>
       <c r="E66" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F66" t="s">
         <v>793</v>
@@ -9371,7 +9369,7 @@
         <v>26</v>
       </c>
       <c r="H66" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I66" t="s">
         <v>794</v>
@@ -9398,7 +9396,7 @@
         <v>800</v>
       </c>
       <c r="Q66" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R66" t="s">
         <v>801</v>
@@ -9433,7 +9431,7 @@
       </c>
       <c r="G67"/>
       <c r="H67" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I67" t="s">
         <v>807</v>
@@ -9451,7 +9449,7 @@
         <v>811</v>
       </c>
       <c r="N67" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="O67" t="s">
         <v>812</v>
@@ -9460,7 +9458,7 @@
         <v>813</v>
       </c>
       <c r="Q67" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R67"/>
       <c r="S67"/>
@@ -9489,7 +9487,7 @@
       </c>
       <c r="G68"/>
       <c r="H68" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I68" t="s">
         <v>568</v>
@@ -9516,7 +9514,7 @@
         <v>820</v>
       </c>
       <c r="Q68" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R68"/>
       <c r="S68"/>
@@ -9544,10 +9542,10 @@
         <v>823</v>
       </c>
       <c r="G69" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H69" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I69" t="s">
         <v>824</v>
@@ -9565,7 +9563,7 @@
         <v>828</v>
       </c>
       <c r="N69" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="O69" t="s">
         <v>829</v>
@@ -9574,7 +9572,7 @@
         <v>830</v>
       </c>
       <c r="Q69" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R69" t="s">
         <v>831</v>
@@ -9604,7 +9602,7 @@
         <v>589</v>
       </c>
       <c r="E70" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F70" t="s">
         <v>835</v>
@@ -9613,7 +9611,7 @@
         <v>26</v>
       </c>
       <c r="H70" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I70" t="s">
         <v>836</v>
@@ -9640,7 +9638,7 @@
         <v>842</v>
       </c>
       <c r="Q70" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R70" t="s">
         <v>843</v>
@@ -9664,7 +9662,7 @@
         <v>846</v>
       </c>
       <c r="C71" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D71" t="s">
         <v>691</v>
@@ -9706,7 +9704,7 @@
         <v>853</v>
       </c>
       <c r="Q71" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R71" t="s">
         <v>854</v>
@@ -9730,13 +9728,13 @@
         <v>857</v>
       </c>
       <c r="C72" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D72" t="s">
         <v>858</v>
       </c>
       <c r="E72" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F72" t="s">
         <v>835</v>
@@ -9745,7 +9743,7 @@
         <v>26</v>
       </c>
       <c r="H72" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="I72" t="s">
         <v>859</v>
@@ -9802,7 +9800,7 @@
         <v>408</v>
       </c>
       <c r="E73" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F73" t="s">
         <v>835</v>
@@ -9838,7 +9836,7 @@
         <v>876</v>
       </c>
       <c r="Q73" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R73" t="s">
         <v>877</v>
@@ -9868,7 +9866,7 @@
         <v>881</v>
       </c>
       <c r="E74" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F74" t="s">
         <v>835</v>
@@ -9877,7 +9875,7 @@
         <v>26</v>
       </c>
       <c r="H74" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I74" t="s">
         <v>882</v>
@@ -9928,13 +9926,13 @@
         <v>892</v>
       </c>
       <c r="C75" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D75" t="s">
         <v>893</v>
       </c>
       <c r="E75" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F75" t="s">
         <v>835</v>
@@ -9970,7 +9968,7 @@
         <v>900</v>
       </c>
       <c r="Q75" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R75" t="s">
         <v>901</v>
@@ -10000,7 +9998,7 @@
         <v>519</v>
       </c>
       <c r="E76" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F76" t="s">
         <v>905</v>
@@ -10009,7 +10007,7 @@
         <v>26</v>
       </c>
       <c r="H76" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I76" t="s">
         <v>906</v>
@@ -10036,7 +10034,7 @@
         <v>912</v>
       </c>
       <c r="Q76" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R76" t="s">
         <v>913</v>
@@ -10060,13 +10058,13 @@
         <v>916</v>
       </c>
       <c r="C77" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D77" t="s">
         <v>917</v>
       </c>
       <c r="E77" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F77" t="s">
         <v>905</v>
@@ -10075,7 +10073,7 @@
         <v>26</v>
       </c>
       <c r="H77" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I77" t="s">
         <v>918</v>
@@ -10137,7 +10135,7 @@
       </c>
       <c r="G78"/>
       <c r="H78" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I78" t="s">
         <v>930</v>
@@ -10164,7 +10162,7 @@
         <v>936</v>
       </c>
       <c r="Q78" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R78"/>
       <c r="S78"/>
@@ -10185,10 +10183,10 @@
         <v>23</v>
       </c>
       <c r="D79" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="E79" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F79" t="s">
         <v>938</v>
@@ -10224,7 +10222,7 @@
         <v>944</v>
       </c>
       <c r="Q79" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R79" t="s">
         <v>404</v>
@@ -10254,7 +10252,7 @@
         <v>946</v>
       </c>
       <c r="E80" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F80" t="s">
         <v>947</v>
@@ -10263,7 +10261,7 @@
         <v>26</v>
       </c>
       <c r="H80" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I80" t="s">
         <v>948</v>
@@ -10288,7 +10286,7 @@
         <v>953</v>
       </c>
       <c r="Q80" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R80" t="s">
         <v>954</v>
@@ -10318,7 +10316,7 @@
         <v>958</v>
       </c>
       <c r="E81" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F81" t="s">
         <v>959</v>
@@ -10327,7 +10325,7 @@
         <v>26</v>
       </c>
       <c r="H81" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I81" t="s">
         <v>960</v>
@@ -10352,7 +10350,7 @@
         <v>965</v>
       </c>
       <c r="Q81" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R81" t="s">
         <v>843</v>
@@ -10385,7 +10383,7 @@
       </c>
       <c r="G82"/>
       <c r="H82" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I82" t="s">
         <v>968</v>
@@ -10408,7 +10406,7 @@
         <v>972</v>
       </c>
       <c r="Q82" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="R82" t="s">
         <v>973</v>
@@ -10443,7 +10441,7 @@
       </c>
       <c r="G83"/>
       <c r="H83" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I83" t="s">
         <v>978</v>
@@ -10461,7 +10459,7 @@
         <v>982</v>
       </c>
       <c r="N83" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="O83" t="s">
         <v>983</v>
@@ -10470,7 +10468,7 @@
         <v>984</v>
       </c>
       <c r="Q83" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R83" t="s">
         <v>985</v>
@@ -10505,7 +10503,7 @@
       </c>
       <c r="G84"/>
       <c r="H84" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I84" t="s">
         <v>989</v>
@@ -10532,7 +10530,7 @@
         <v>996</v>
       </c>
       <c r="Q84" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R84" t="s">
         <v>997</v>
@@ -10571,7 +10569,7 @@
         <v>26</v>
       </c>
       <c r="H85" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I85" t="s">
         <v>1002</v>
@@ -10628,7 +10626,7 @@
         <v>1013</v>
       </c>
       <c r="E86" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F86" t="s">
         <v>1014</v>
@@ -10637,7 +10635,7 @@
         <v>26</v>
       </c>
       <c r="H86" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="I86" t="s">
         <v>1015</v>
@@ -10688,13 +10686,13 @@
         <v>1025</v>
       </c>
       <c r="C87" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D87" t="s">
         <v>1026</v>
       </c>
       <c r="E87" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F87" t="s">
         <v>1014</v>
@@ -10703,7 +10701,7 @@
         <v>26</v>
       </c>
       <c r="H87" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I87" t="s">
         <v>1027</v>
@@ -10730,7 +10728,7 @@
         <v>1033</v>
       </c>
       <c r="Q87" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R87" t="s">
         <v>667</v>
@@ -10760,7 +10758,7 @@
         <v>1035</v>
       </c>
       <c r="E88" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F88" t="s">
         <v>1014</v>
@@ -10796,7 +10794,7 @@
         <v>1042</v>
       </c>
       <c r="Q88" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R88" t="s">
         <v>1043</v>
@@ -10820,13 +10818,13 @@
         <v>1046</v>
       </c>
       <c r="C89" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D89" t="s">
         <v>1047</v>
       </c>
       <c r="E89" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F89" t="s">
         <v>1014</v>
@@ -10835,7 +10833,7 @@
         <v>26</v>
       </c>
       <c r="H89" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="I89" t="s">
         <v>1048</v>
@@ -10862,7 +10860,7 @@
         <v>1054</v>
       </c>
       <c r="Q89" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R89" t="s">
         <v>585</v>
@@ -10892,7 +10890,7 @@
         <v>1056</v>
       </c>
       <c r="E90" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F90" t="s">
         <v>1057</v>
@@ -10901,7 +10899,7 @@
         <v>26</v>
       </c>
       <c r="H90" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="I90" t="s">
         <v>1058</v>
@@ -10958,7 +10956,7 @@
         <v>458</v>
       </c>
       <c r="E91" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F91" t="s">
         <v>1066</v>
@@ -10967,7 +10965,7 @@
         <v>26</v>
       </c>
       <c r="H91" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I91" t="s">
         <v>1067</v>
@@ -10992,16 +10990,16 @@
         <v>1072</v>
       </c>
       <c r="Q91" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R91" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="S91" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="T91" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="U91" t="s">
         <v>232</v>
@@ -11016,13 +11014,13 @@
         <v>1073</v>
       </c>
       <c r="C92" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D92" t="s">
-        <v>207</v>
+        <v>43</v>
       </c>
       <c r="E92" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F92" t="s">
         <v>1074</v>
@@ -11031,7 +11029,7 @@
         <v>26</v>
       </c>
       <c r="H92" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I92" t="s">
         <v>1075</v>
@@ -11058,16 +11056,16 @@
         <v>1081</v>
       </c>
       <c r="Q92" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R92" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="S92" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="T92" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="U92" t="s">
         <v>232</v>
@@ -11088,7 +11086,7 @@
         <v>1047</v>
       </c>
       <c r="E93" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F93" t="s">
         <v>1083</v>
@@ -11097,7 +11095,7 @@
         <v>26</v>
       </c>
       <c r="H93" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I93" t="s">
         <v>1084</v>
@@ -11122,7 +11120,7 @@
         <v>1089</v>
       </c>
       <c r="Q93" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R93" t="s">
         <v>506</v>
@@ -11152,7 +11150,7 @@
         <v>458</v>
       </c>
       <c r="E94" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F94" t="s">
         <v>1083</v>
@@ -11161,7 +11159,7 @@
         <v>26</v>
       </c>
       <c r="H94" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I94" t="s">
         <v>1091</v>
@@ -11186,16 +11184,16 @@
         <v>1096</v>
       </c>
       <c r="Q94" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R94" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="S94" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="T94" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="U94" t="s">
         <v>232</v>
@@ -11216,7 +11214,7 @@
         <v>458</v>
       </c>
       <c r="E95" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F95" t="s">
         <v>1083</v>
@@ -11225,7 +11223,7 @@
         <v>26</v>
       </c>
       <c r="H95" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I95" t="s">
         <v>1091</v>
@@ -11250,16 +11248,16 @@
         <v>1101</v>
       </c>
       <c r="Q95" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R95" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="S95" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="T95" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="U95" t="s">
         <v>232</v>
@@ -11280,7 +11278,7 @@
         <v>458</v>
       </c>
       <c r="E96" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F96" t="s">
         <v>1083</v>
@@ -11289,7 +11287,7 @@
         <v>26</v>
       </c>
       <c r="H96" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I96" t="s">
         <v>1091</v>
@@ -11314,16 +11312,16 @@
         <v>1106</v>
       </c>
       <c r="Q96" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R96" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="S96" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="T96" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="U96" t="s">
         <v>232</v>
@@ -11338,13 +11336,13 @@
         <v>1107</v>
       </c>
       <c r="C97" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D97" t="s">
         <v>541</v>
       </c>
       <c r="E97" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F97" t="s">
         <v>1108</v>
@@ -11353,7 +11351,7 @@
         <v>26</v>
       </c>
       <c r="H97" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I97" t="s">
         <v>1109</v>
@@ -11380,7 +11378,7 @@
         <v>1115</v>
       </c>
       <c r="Q97" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R97" t="s">
         <v>1116</v>
@@ -11404,13 +11402,13 @@
         <v>1119</v>
       </c>
       <c r="C98" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D98" t="s">
         <v>601</v>
       </c>
       <c r="E98" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F98" t="s">
         <v>1120</v>
@@ -11446,16 +11444,16 @@
         <v>1127</v>
       </c>
       <c r="Q98" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R98" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="S98" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="T98" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="U98" t="s">
         <v>232</v>
@@ -11470,13 +11468,13 @@
         <v>1128</v>
       </c>
       <c r="C99" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D99" t="s">
         <v>1129</v>
       </c>
       <c r="E99" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F99" t="s">
         <v>1120</v>
@@ -11485,7 +11483,7 @@
         <v>26</v>
       </c>
       <c r="H99" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I99" t="s">
         <v>1130</v>
@@ -11512,7 +11510,7 @@
         <v>1136</v>
       </c>
       <c r="Q99" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R99" t="s">
         <v>1137</v>
@@ -11536,13 +11534,13 @@
         <v>1140</v>
       </c>
       <c r="C100" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D100" t="s">
         <v>1141</v>
       </c>
       <c r="E100" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F100" t="s">
         <v>1120</v>
@@ -11631,7 +11629,7 @@
         <v>1158</v>
       </c>
       <c r="N101" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="O101" t="s">
         <v>1159</v>
@@ -11640,7 +11638,7 @@
         <v>1160</v>
       </c>
       <c r="Q101" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R101" t="s">
         <v>1161</v>
@@ -11670,7 +11668,7 @@
         <v>436</v>
       </c>
       <c r="E102" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F102" t="s">
         <v>1153</v>
@@ -11679,7 +11677,7 @@
         <v>26</v>
       </c>
       <c r="H102" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="I102" t="s">
         <v>1165</v>
@@ -11736,7 +11734,7 @@
         <v>1176</v>
       </c>
       <c r="E103" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F103" t="s">
         <v>1153</v>
@@ -11745,7 +11743,7 @@
         <v>26</v>
       </c>
       <c r="H103" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I103" t="s">
         <v>1177</v>
@@ -11796,13 +11794,13 @@
         <v>1187</v>
       </c>
       <c r="C104" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D104" t="s">
         <v>1188</v>
       </c>
       <c r="E104" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F104" t="s">
         <v>1153</v>
@@ -11811,7 +11809,7 @@
         <v>26</v>
       </c>
       <c r="H104" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I104" t="s">
         <v>1189</v>
@@ -11838,7 +11836,7 @@
         <v>1195</v>
       </c>
       <c r="Q104" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R104" t="s">
         <v>854</v>
@@ -11868,7 +11866,7 @@
         <v>589</v>
       </c>
       <c r="E105" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F105" t="s">
         <v>1153</v>
@@ -11877,7 +11875,7 @@
         <v>26</v>
       </c>
       <c r="H105" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I105" t="s">
         <v>1197</v>
@@ -11934,7 +11932,7 @@
         <v>541</v>
       </c>
       <c r="E106" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F106" t="s">
         <v>1153</v>
@@ -11970,7 +11968,7 @@
         <v>1215</v>
       </c>
       <c r="Q106" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R106" t="s">
         <v>1216</v>
@@ -11994,13 +11992,13 @@
         <v>1219</v>
       </c>
       <c r="C107" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D107" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="E107" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F107" t="s">
         <v>1220</v>
@@ -12009,7 +12007,7 @@
         <v>26</v>
       </c>
       <c r="H107" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I107" t="s">
         <v>1221</v>
@@ -12036,16 +12034,16 @@
         <v>1227</v>
       </c>
       <c r="Q107" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R107" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="S107" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="T107" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="U107" t="s">
         <v>232</v>
@@ -12066,7 +12064,7 @@
         <v>408</v>
       </c>
       <c r="E108" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F108" t="s">
         <v>1229</v>
@@ -12102,7 +12100,7 @@
         <v>1236</v>
       </c>
       <c r="Q108" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R108" t="s">
         <v>712</v>
@@ -12132,7 +12130,7 @@
         <v>1238</v>
       </c>
       <c r="E109" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F109" t="s">
         <v>1239</v>
@@ -12166,7 +12164,7 @@
         <v>1245</v>
       </c>
       <c r="Q109" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R109" t="s">
         <v>712</v>
@@ -12196,7 +12194,7 @@
         <v>1247</v>
       </c>
       <c r="E110" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F110" t="s">
         <v>1239</v>
@@ -12205,7 +12203,7 @@
         <v>26</v>
       </c>
       <c r="H110" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I110" t="s">
         <v>1248</v>
@@ -12230,7 +12228,7 @@
         <v>1253</v>
       </c>
       <c r="Q110" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R110" t="s">
         <v>1254</v>
@@ -12254,13 +12252,13 @@
         <v>1257</v>
       </c>
       <c r="C111" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="D111" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="E111" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F111" t="s">
         <v>1258</v>
@@ -12269,7 +12267,7 @@
         <v>26</v>
       </c>
       <c r="H111" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I111" t="s">
         <v>1259</v>
@@ -12296,7 +12294,7 @@
         <v>1265</v>
       </c>
       <c r="Q111" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R111" t="s">
         <v>789</v>
@@ -12329,7 +12327,7 @@
       </c>
       <c r="G112"/>
       <c r="H112" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I112" t="s">
         <v>1268</v>
@@ -12352,7 +12350,7 @@
         <v>1273</v>
       </c>
       <c r="Q112" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="R112" t="s">
         <v>1274</v>
@@ -12387,7 +12385,7 @@
       </c>
       <c r="G113"/>
       <c r="H113" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="I113" t="s">
         <v>1279</v>
@@ -12414,7 +12412,7 @@
         <v>1285</v>
       </c>
       <c r="Q113" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R113" t="s">
         <v>1286</v>
@@ -12438,13 +12436,13 @@
         <v>1289</v>
       </c>
       <c r="C114" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D114" t="s">
         <v>1290</v>
       </c>
       <c r="E114" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F114" t="s">
         <v>1291</v>
@@ -12453,7 +12451,7 @@
         <v>26</v>
       </c>
       <c r="H114" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I114" t="s">
         <v>1292</v>
@@ -12480,7 +12478,7 @@
         <v>1298</v>
       </c>
       <c r="Q114" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R114" t="s">
         <v>1299</v>
@@ -12504,13 +12502,13 @@
         <v>1302</v>
       </c>
       <c r="C115" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D115" t="s">
         <v>1303</v>
       </c>
       <c r="E115" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F115" t="s">
         <v>1304</v>
@@ -12519,7 +12517,7 @@
         <v>26</v>
       </c>
       <c r="H115" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I115" t="s">
         <v>1305</v>
@@ -12546,7 +12544,7 @@
         <v>1311</v>
       </c>
       <c r="Q115" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R115" t="s">
         <v>1312</v>
@@ -12570,22 +12568,22 @@
         <v>1315</v>
       </c>
       <c r="C116" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D116" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="E116" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F116" t="s">
         <v>1304</v>
       </c>
       <c r="G116" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H116" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I116" t="s">
         <v>1316</v>
@@ -12612,7 +12610,7 @@
         <v>1322</v>
       </c>
       <c r="Q116" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R116" t="s">
         <v>667</v>
@@ -12636,22 +12634,22 @@
         <v>1323</v>
       </c>
       <c r="C117" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="D117" t="s">
         <v>330</v>
       </c>
       <c r="E117" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F117" t="s">
         <v>1324</v>
       </c>
       <c r="G117" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H117" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I117" t="s">
         <v>1325</v>
@@ -12708,7 +12706,7 @@
         <v>1333</v>
       </c>
       <c r="E118" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F118" t="s">
         <v>1324</v>
@@ -12717,7 +12715,7 @@
         <v>26</v>
       </c>
       <c r="H118" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I118" t="s">
         <v>1334</v>
@@ -12744,7 +12742,7 @@
         <v>1340</v>
       </c>
       <c r="Q118" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R118" t="s">
         <v>1341</v>
@@ -12783,7 +12781,7 @@
         <v>26</v>
       </c>
       <c r="H119" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="I119" t="s">
         <v>1347</v>
@@ -12834,13 +12832,13 @@
         <v>1357</v>
       </c>
       <c r="C120" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D120" t="s">
         <v>292</v>
       </c>
       <c r="E120" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F120" t="s">
         <v>1324</v>
@@ -12849,7 +12847,7 @@
         <v>26</v>
       </c>
       <c r="H120" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I120" t="s">
         <v>1358</v>
@@ -12876,7 +12874,7 @@
         <v>1364</v>
       </c>
       <c r="Q120" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R120" t="s">
         <v>1365</v>
@@ -12900,13 +12898,13 @@
         <v>1368</v>
       </c>
       <c r="C121" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D121" t="s">
         <v>1333</v>
       </c>
       <c r="E121" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F121" t="s">
         <v>1324</v>
@@ -12915,7 +12913,7 @@
         <v>26</v>
       </c>
       <c r="H121" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I121" t="s">
         <v>1369</v>
@@ -12942,7 +12940,7 @@
         <v>1375</v>
       </c>
       <c r="Q121" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R121" t="s">
         <v>1376</v>
@@ -12966,13 +12964,13 @@
         <v>1379</v>
       </c>
       <c r="C122" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D122" t="s">
         <v>1035</v>
       </c>
       <c r="E122" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F122" t="s">
         <v>1324</v>
@@ -13032,13 +13030,13 @@
         <v>1390</v>
       </c>
       <c r="C123" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D123" t="s">
         <v>1391</v>
       </c>
       <c r="E123" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F123" t="s">
         <v>1392</v>
@@ -13098,13 +13096,13 @@
         <v>1400</v>
       </c>
       <c r="C124" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D124" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="E124" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F124" t="s">
         <v>1401</v>
@@ -13140,7 +13138,7 @@
         <v>1408</v>
       </c>
       <c r="Q124" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R124" t="s">
         <v>288</v>
@@ -13164,22 +13162,22 @@
         <v>1409</v>
       </c>
       <c r="C125" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D125" t="s">
         <v>1410</v>
       </c>
       <c r="E125" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F125" t="s">
         <v>1411</v>
       </c>
       <c r="G125" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H125" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I125" t="s">
         <v>1412</v>
@@ -13206,7 +13204,7 @@
         <v>1418</v>
       </c>
       <c r="Q125" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R125" t="s">
         <v>634</v>
@@ -13230,22 +13228,22 @@
         <v>1419</v>
       </c>
       <c r="C126" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="D126" t="s">
         <v>1420</v>
       </c>
       <c r="E126" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F126" t="s">
         <v>1421</v>
       </c>
       <c r="G126" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H126" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I126" t="s">
         <v>1422</v>
@@ -13272,7 +13270,7 @@
         <v>1428</v>
       </c>
       <c r="Q126" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R126" t="s">
         <v>1184</v>
@@ -13302,7 +13300,7 @@
         <v>541</v>
       </c>
       <c r="E127" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F127" t="s">
         <v>1421</v>
@@ -13311,7 +13309,7 @@
         <v>26</v>
       </c>
       <c r="H127" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I127" t="s">
         <v>1430</v>
@@ -13336,16 +13334,16 @@
         <v>1435</v>
       </c>
       <c r="Q127" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R127" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="S127" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="T127" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="U127" t="s">
         <v>232</v>
@@ -13363,10 +13361,10 @@
         <v>219</v>
       </c>
       <c r="D128" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="E128" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F128" t="s">
         <v>1437</v>
@@ -13375,7 +13373,7 @@
         <v>26</v>
       </c>
       <c r="H128" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I128" t="s">
         <v>1438</v>
@@ -13400,16 +13398,16 @@
         <v>1443</v>
       </c>
       <c r="Q128" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R128" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="S128" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="T128" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="U128" t="s">
         <v>232</v>
@@ -13437,7 +13435,7 @@
         <v>26</v>
       </c>
       <c r="H129" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I129" t="s">
         <v>1446</v>
@@ -13464,7 +13462,7 @@
         <v>1452</v>
       </c>
       <c r="Q129" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R129" t="s">
         <v>1453</v>
@@ -13488,13 +13486,13 @@
         <v>1456</v>
       </c>
       <c r="C130" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D130" t="s">
         <v>751</v>
       </c>
       <c r="E130" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F130" t="s">
         <v>1457</v>
@@ -13503,7 +13501,7 @@
         <v>26</v>
       </c>
       <c r="H130" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I130" t="s">
         <v>1458</v>
@@ -13560,7 +13558,7 @@
         <v>576</v>
       </c>
       <c r="E131" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F131" t="s">
         <v>1457</v>
@@ -13569,7 +13567,7 @@
         <v>26</v>
       </c>
       <c r="H131" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I131" t="s">
         <v>1469</v>
@@ -13626,13 +13624,13 @@
         <v>1480</v>
       </c>
       <c r="E132" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F132" t="s">
         <v>1481</v>
       </c>
       <c r="G132" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H132" t="s">
         <v>727</v>
@@ -13692,7 +13690,7 @@
         <v>881</v>
       </c>
       <c r="E133" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="F133" t="s">
         <v>1481</v>
@@ -13752,7 +13750,7 @@
         <v>1498</v>
       </c>
       <c r="C134" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D134" t="s">
         <v>1499</v>
@@ -13767,7 +13765,7 @@
         <v>26</v>
       </c>
       <c r="H134" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="I134" t="s">
         <v>1501</v>
@@ -13818,22 +13816,22 @@
         <v>1508</v>
       </c>
       <c r="C135" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D135" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="E135" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F135" t="s">
         <v>1509</v>
       </c>
       <c r="G135" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H135" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I135" t="s">
         <v>1510</v>
@@ -13860,7 +13858,7 @@
         <v>1516</v>
       </c>
       <c r="Q135" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R135" t="s">
         <v>1517</v>
@@ -13884,13 +13882,13 @@
         <v>1520</v>
       </c>
       <c r="C136" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="D136" t="s">
         <v>541</v>
       </c>
       <c r="E136" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="F136" t="s">
         <v>1521</v>
@@ -13899,7 +13897,7 @@
         <v>26</v>
       </c>
       <c r="H136" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I136" t="s">
         <v>1522</v>
@@ -13926,7 +13924,7 @@
         <v>1528</v>
       </c>
       <c r="Q136" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R136" t="s">
         <v>1529</v>
@@ -13956,7 +13954,7 @@
         <v>1533</v>
       </c>
       <c r="E137" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F137" t="s">
         <v>1521</v>
@@ -13965,7 +13963,7 @@
         <v>26</v>
       </c>
       <c r="H137" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I137" t="s">
         <v>1534</v>
@@ -14020,7 +14018,7 @@
         <v>1533</v>
       </c>
       <c r="E138" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="F138" t="s">
         <v>1521</v>
@@ -14029,7 +14027,7 @@
         <v>26</v>
       </c>
       <c r="H138" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I138" t="s">
         <v>1541</v>
@@ -14054,7 +14052,7 @@
         <v>1546</v>
       </c>
       <c r="Q138" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R138" t="s">
         <v>1529</v>
@@ -14093,7 +14091,7 @@
         <v>26</v>
       </c>
       <c r="H139" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="I139" t="s">
         <v>1550</v>
@@ -14118,7 +14116,7 @@
         <v>1555</v>
       </c>
       <c r="Q139" t="s">
-        <v>115</v>
+        <v>54</v>
       </c>
       <c r="R139" t="s">
         <v>506</v>
@@ -14148,7 +14146,7 @@
         <v>1333</v>
       </c>
       <c r="E140" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="F140" t="s">
         <v>1557</v>
@@ -14157,7 +14155,7 @@
         <v>26</v>
       </c>
       <c r="H140" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="I140" t="s">
         <v>1558</v>
@@ -14217,7 +14215,7 @@
       </c>
       <c r="G141"/>
       <c r="H141" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="I141" t="s">
         <v>1569</v>
@@ -14244,7 +14242,7 @@
         <v>1575</v>
       </c>
       <c r="Q141" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="R141" t="s">
         <v>1576</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-06-02
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -305,10 +305,10 @@
     <t xml:space="preserve">Rechtliche Abklärungen und Potenzial von künstlicher Intelligenz in den Bereichen Polizei und innere Sicherheit</t>
   </si>
   <si>
-    <t xml:space="preserve">Clarifications juridiques et potentiel de l'utilisation de l'intelligence artificielle (IA) dans les domaines de la police et de la sécurité intérieure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chiarimenti giuridici e potenzialità dell'impiego dell'intelligenza artificiale (IA) nei settori della polizia e della sicurezza interna</t>
+    <t xml:space="preserve">Clarifications juridiques et potentiel de l'utilisation de l'intelligence artificielle dans les domaines de la police et de la sécurité intérieure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chiarimenti giuridici e potenzialità dell'impiego dell'intelligenza artificiale nei settori della polizia e della sicurezza interna</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de présenter un rapport concernant l’utilisation de l’intelligence artificielle (IA) dans les domaines de la police, de la sécurité intérieure et de la poursuite pénale exposant le potentiel, les bases légales et les limites constitutionnelles, notamment pour la protection de la vie privée. Sur la base de ces conclusions, il devra soumettre au Parlement des lignes directrices pour une utilisation cohérente et conforme aux droits fondamentaux de l’IA dans les domaines de la police, de la sécurité intérieure et de la poursuite pénale, tout en respectant la souveraineté numérique de la Suisse. Le rapport devra notamment :&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;1. Démontrer le potentiel et les domaines d’application des technologies d’IA pour rendre la lutte contre la criminalité plus efficace et contribuer à la sauvegarde de la sécurité intérieure.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;2. Analyser le cadre juridique existant pour l’utilisation des technologies d’IA dans le domaine de la sécurité et identifier les éventuelles lacunes du cadre juridique.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;3. Expliquer les limites constitutionnelles à l’utilisation des technologies d’IA dans les domaines de la police et de la sécurité et définir des conditions cadre et les lignes directrices pour l’utilisation de ces technologies.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;4. Démontrer comment les exigences en matière de protection de la vie privée peuvent être satisfaites lors de l'utilisation des technologies d'IA dans les domaines de la police et de la sécurité.&amp;nbsp;&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;5. Expliquer comment la souveraineté numérique de la Suisse peut être préservée et la dépendance vis-à-vis des prestataires externes évitée lors de l'acquisition et de l'exploitation des technologies d'IA dans le secteur de la sécurité.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-06-03
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -158,6 +158,60 @@
     <t xml:space="preserve">Politica nazionale|Media e comunicazione|Protezione sociale</t>
   </si>
   <si>
+    <t xml:space="preserve">26.3121</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ip.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juillard Charles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Centre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UVEK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dank einer leistungsfähigen Nationalstrasse N18 Kultur- und Wirtschaftsräume effektiv miteinander verbinden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relier efficacement des espaces culturels et économiques grâce à une route nationale N18 performante</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collegare efficacemente spazi culturali ed economici attraverso una strada nazionale N18 efficiente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Fin janvier 2026, le Conseil fédéral a publié les paramètres du programme « Transports ’45 »dans lequel le projet d’amélioration structurelle de la liaison routière Delémont- Bâle a été retenu. Mais, le report au-delà de 2055 des projets routiers le long de la N18 entre Bâle et Delémont – à l’exception de la décharge du centre de Laufen (horizon 2055) – suscite une forte incompréhension de la part des élus, des populations et des milieux économiques en particulier. Ce renoncement de fait à une meilleure accessibilité et à de réelles perspectives de développement économique contredit directement les résultats de l’étude de corridor N18 menée sous la direction de l’OFROU selon les méthodes les plus récentes. C’est aussi une question de crédibilité des institutions par un respect de la cohérence des politiques publiques.&lt;/p&gt;&lt;p&gt;La N18 est un élément essentiel du réseau routier national : elle relie l’agglomération bâloise à l’Arc lémanique et unit deux espaces culturels et&amp;nbsp;économiques majeurs. Elle connecte&amp;nbsp;également le Laufonnais, région dynamique, ainsi que la capitale cantonale Delémont au réseau à haute performance. Elle contribue ainsi&amp;nbsp;à la cohésion nationale et au rapprochement des communautés linguistiques.&lt;/p&gt;&lt;p&gt;Sous l’effet de la croissance démographique, ce tronçon devient toutefois un goulet d’étranglement, avec l’une des plus fortes densités de bouchons du pays. De plus, le trafic actuel porte atteinte à la qualité de vie dans les centres et compromet la sécurité du trafic motorisé et cycliste. Une modernisation rapide du corridor est donc prioritaire.&lt;/p&gt;&lt;p&gt;Dans ce contexte, je prie le Conseil fédéral de répondre aux questions suivantes :&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Comment évalue-t-il la nécessité d’éliminer les goulets d’étranglement sur la N18 entre Angenstein et Delémont ?&lt;/li&gt;&lt;li&gt;Considère-t-il le tunnel du Muggenberg comme une mesure durable pour améliorer la sécurité au point noir d’Angenstein ?&lt;/li&gt;&lt;li&gt;Comment apprécie-t-il l’utilité des projets recommandés dans l’étude de corridor N18 (tunnel du Muggenberg, contournements Laufen–Zwingen et Delémont, décharge de Laufen) pour renforcer la connexion des entreprises de la région Laufonnais–Thierstein–Delémont ?&lt;/li&gt;&lt;li&gt;Estime-t-il que les contournements Laufen–Zwingen et Delémont constituent des mesures appropriées pour soulager les zones habitées concernées ?&lt;/li&gt;&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Ende Januar&amp;nbsp;2026 hat der Bundesrat die Eckwerte des Programms «Verkehr&amp;nbsp;’45» veröffentlicht. Das Vorhaben einer strukturellen Verbesserung der Strassenverbindung Delémont–Basel wurde darin berücksichtigt. Dass die Strassenbauprojekte entlang der Nationalstrasse&amp;nbsp;18 (N18) zwischen Basel und Delémont – mit Ausnahme der Zentrumsentlastung Laufen (Realisierungshorizont&amp;nbsp;2055) – aber bis nach 2055 aufgeschoben werden sollen, stösst bei Politik, Bevölkerung und insbesondere in Wirtschaftskreisen auf grosses Unverständnis. Diese Entscheidung gegen bessere Erreichbarkeit und wirtschaftliche Entwicklung widerspricht den Ergebnissen der Korridorstudie&amp;nbsp;N18, die unter der Federführung des Bundesamts für Strassen (ASTRA) nach neuesten Methoden durchgeführt wurde. Es geht dabei auch um die Glaubwürdigkeit der Institutionen, von denen eine kohärente öffentliche Politik erwartet wird.&lt;/p&gt;&lt;p&gt;Die N18 ist ein wesentlicher Bestandteil des nationalen Strassennetzes: Sie verbindet den Grossraum Basel mit der Genferseeregion und damit zwei wichtige Kultur- und Wirtschaftsräume. Sie schliesst zudem das dynamische Laufental und den Kantonshauptort Delémont an das Hochleistungsstrassennetz an. Damit trägt sie zum nationalen Zusammenhalt und zur Annäherung der Sprachgemeinschaften bei.&lt;/p&gt;&lt;p&gt;Aufgrund des Bevölkerungswachstums entwickelt sich dieser Strassenabschnitt jedoch zunehmend zu einem Engpass – mit einer der schweizweit höchsten Staudichten. Gleichzeitig leidet die Lebensqualität in den Ortszentren, und die Sicherheit des Auto- und Veloverkehrs wird gefährdet. Eine rasche Modernisierung des Korridors hat daher Priorität.&lt;/p&gt;&lt;p&gt;Daher bitte ich den Bundesrat um Beantwortung folgender Fragen:&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Wie beurteilt er die Notwendigkeit, die Engpässe auf der N18 zwischen Angenstein und Delémont zu beseitigen?&lt;/li&gt;&lt;li&gt;Ist der Muggenbergtunnel seines Erachtens eine nachhaltige Massnahme zur Verbesserung der Sicherheit am Unfallhotspot Angenstein?&lt;/li&gt;&lt;li&gt;Wie bewertet er den Nutzen der in der Korridorstudie&amp;nbsp;N18 empfohlenen Projekte (Muggenbergtunnel, Umfahrungen Laufen–Zwingen und Delémont, Zentrumsentlastung Laufen) für eine verbesserte Anbindung der Unternehmen in der Region Laufen–Thierstein–Delémont?&lt;/li&gt;&lt;li&gt;Sind die Umfahrungen Laufen–Zwingen und Delémont seines Erachtens geeignete Massnahmen zur Entlastung der betroffenen Wohngebiete?&lt;/li&gt;&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erledigt / Liquidé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263121</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263121</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verkehr|Raumplanung und Wohnungswesen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transports|Aménagement du territoire et logement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trasporti|Pianificazione territoriale e alloggi</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.3518</t>
   </si>
   <si>
@@ -215,9 +269,6 @@
     <t xml:space="preserve">26.3323</t>
   </si>
   <si>
-    <t xml:space="preserve">Ip.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Brenzikofer Florence</t>
   </si>
   <si>
@@ -272,9 +323,6 @@
     <t xml:space="preserve">2026-03-20</t>
   </si>
   <si>
-    <t xml:space="preserve">SR</t>
-  </si>
-  <si>
     <t xml:space="preserve">EDI</t>
   </si>
   <si>
@@ -312,54 +360,6 @@
   </si>
   <si>
     <t xml:space="preserve">2026-05-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.3121</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juillard Charles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Centre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UVEK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dank einer leistungsfähigen Nationalstrasse N18 Kultur- und Wirtschaftsräume effektiv miteinander verbinden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relier efficacement des espaces culturels et économiques grâce à une route nationale N18 performante</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collegare efficacemente spazi culturali ed economici attraverso una strada nazionale N18 efficiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Fin janvier 2026, le Conseil fédéral a publié les paramètres du programme « Transports ’45 »dans lequel le projet d’amélioration structurelle de la liaison routière Delémont- Bâle a été retenu. Mais, le report au-delà de 2055 des projets routiers le long de la N18 entre Bâle et Delémont – à l’exception de la décharge du centre de Laufen (horizon 2055) – suscite une forte incompréhension de la part des élus, des populations et des milieux économiques en particulier. Ce renoncement de fait à une meilleure accessibilité et à de réelles perspectives de développement économique contredit directement les résultats de l’étude de corridor N18 menée sous la direction de l’OFROU selon les méthodes les plus récentes. C’est aussi une question de crédibilité des institutions par un respect de la cohérence des politiques publiques.&lt;/p&gt;&lt;p&gt;La N18 est un élément essentiel du réseau routier national : elle relie l’agglomération bâloise à l’Arc lémanique et unit deux espaces culturels et&amp;nbsp;économiques majeurs. Elle connecte&amp;nbsp;également le Laufonnais, région dynamique, ainsi que la capitale cantonale Delémont au réseau à haute performance. Elle contribue ainsi&amp;nbsp;à la cohésion nationale et au rapprochement des communautés linguistiques.&lt;/p&gt;&lt;p&gt;Sous l’effet de la croissance démographique, ce tronçon devient toutefois un goulet d’étranglement, avec l’une des plus fortes densités de bouchons du pays. De plus, le trafic actuel porte atteinte à la qualité de vie dans les centres et compromet la sécurité du trafic motorisé et cycliste. Une modernisation rapide du corridor est donc prioritaire.&lt;/p&gt;&lt;p&gt;Dans ce contexte, je prie le Conseil fédéral de répondre aux questions suivantes :&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Comment évalue-t-il la nécessité d’éliminer les goulets d’étranglement sur la N18 entre Angenstein et Delémont ?&lt;/li&gt;&lt;li&gt;Considère-t-il le tunnel du Muggenberg comme une mesure durable pour améliorer la sécurité au point noir d’Angenstein ?&lt;/li&gt;&lt;li&gt;Comment apprécie-t-il l’utilité des projets recommandés dans l’étude de corridor N18 (tunnel du Muggenberg, contournements Laufen–Zwingen et Delémont, décharge de Laufen) pour renforcer la connexion des entreprises de la région Laufonnais–Thierstein–Delémont ?&lt;/li&gt;&lt;li&gt;Estime-t-il que les contournements Laufen–Zwingen et Delémont constituent des mesures appropriées pour soulager les zones habitées concernées ?&lt;/li&gt;&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Ende Januar&amp;nbsp;2026 hat der Bundesrat die Eckwerte des Programms «Verkehr&amp;nbsp;’45» veröffentlicht. Das Vorhaben einer strukturellen Verbesserung der Strassenverbindung Delémont–Basel wurde darin berücksichtigt. Dass die Strassenbauprojekte entlang der Nationalstrasse&amp;nbsp;18 (N18) zwischen Basel und Delémont – mit Ausnahme der Zentrumsentlastung Laufen (Realisierungshorizont&amp;nbsp;2055) – aber bis nach 2055 aufgeschoben werden sollen, stösst bei Politik, Bevölkerung und insbesondere in Wirtschaftskreisen auf grosses Unverständnis. Diese Entscheidung gegen bessere Erreichbarkeit und wirtschaftliche Entwicklung widerspricht den Ergebnissen der Korridorstudie&amp;nbsp;N18, die unter der Federführung des Bundesamts für Strassen (ASTRA) nach neuesten Methoden durchgeführt wurde. Es geht dabei auch um die Glaubwürdigkeit der Institutionen, von denen eine kohärente öffentliche Politik erwartet wird.&lt;/p&gt;&lt;p&gt;Die N18 ist ein wesentlicher Bestandteil des nationalen Strassennetzes: Sie verbindet den Grossraum Basel mit der Genferseeregion und damit zwei wichtige Kultur- und Wirtschaftsräume. Sie schliesst zudem das dynamische Laufental und den Kantonshauptort Delémont an das Hochleistungsstrassennetz an. Damit trägt sie zum nationalen Zusammenhalt und zur Annäherung der Sprachgemeinschaften bei.&lt;/p&gt;&lt;p&gt;Aufgrund des Bevölkerungswachstums entwickelt sich dieser Strassenabschnitt jedoch zunehmend zu einem Engpass – mit einer der schweizweit höchsten Staudichten. Gleichzeitig leidet die Lebensqualität in den Ortszentren, und die Sicherheit des Auto- und Veloverkehrs wird gefährdet. Eine rasche Modernisierung des Korridors hat daher Priorität.&lt;/p&gt;&lt;p&gt;Daher bitte ich den Bundesrat um Beantwortung folgender Fragen:&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Wie beurteilt er die Notwendigkeit, die Engpässe auf der N18 zwischen Angenstein und Delémont zu beseitigen?&lt;/li&gt;&lt;li&gt;Ist der Muggenbergtunnel seines Erachtens eine nachhaltige Massnahme zur Verbesserung der Sicherheit am Unfallhotspot Angenstein?&lt;/li&gt;&lt;li&gt;Wie bewertet er den Nutzen der in der Korridorstudie&amp;nbsp;N18 empfohlenen Projekte (Muggenbergtunnel, Umfahrungen Laufen–Zwingen und Delémont, Zentrumsentlastung Laufen) für eine verbesserte Anbindung der Unternehmen in der Region Laufen–Thierstein–Delémont?&lt;/li&gt;&lt;li&gt;Sind die Umfahrungen Laufen–Zwingen und Delémont seines Erachtens geeignete Massnahmen zur Entlastung der betroffenen Wohngebiete?&lt;/li&gt;&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Erledigt / Liquidé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263121</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263121</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verkehr|Raumplanung und Wohnungswesen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transports|Aménagement du territoire et logement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trasporti|Pianificazione territoriale e alloggi</t>
   </si>
   <si>
     <t xml:space="preserve">26.3099</t>
@@ -5358,7 +5358,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20263518</v>
+        <v>20263121</v>
       </c>
       <c r="B4" t="s">
         <v>48</v>
@@ -5369,60 +5369,62 @@
       <c r="D4" t="s">
         <v>50</v>
       </c>
-      <c r="E4"/>
+      <c r="E4" t="s">
+        <v>51</v>
+      </c>
       <c r="F4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G4" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="H4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="J4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="K4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="M4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="N4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="O4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="P4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q4" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="R4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="T4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="U4" t="s">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="V4"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20263323</v>
+        <v>20263518</v>
       </c>
       <c r="B5" t="s">
         <v>66</v>
@@ -5433,35 +5435,33 @@
       <c r="D5" t="s">
         <v>68</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5"/>
+      <c r="F5" t="s">
         <v>69</v>
-      </c>
-      <c r="F5" t="s">
-        <v>70</v>
       </c>
       <c r="G5" t="s">
         <v>27</v>
       </c>
       <c r="H5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I5" t="s">
         <v>71</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>72</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>73</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>74</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>75</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>76</v>
-      </c>
-      <c r="N5" t="s">
-        <v>58</v>
       </c>
       <c r="O5" t="s">
         <v>77</v>
@@ -5482,52 +5482,52 @@
         <v>82</v>
       </c>
       <c r="U5" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="V5"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>20263411</v>
+        <v>20263323</v>
       </c>
       <c r="B6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C6" t="s">
         <v>49</v>
       </c>
       <c r="D6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="F6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G6" t="s">
-        <v>86</v>
+        <v>27</v>
       </c>
       <c r="H6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="M6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="N6" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="O6" t="s">
         <v>94</v>
@@ -5536,25 +5536,25 @@
         <v>95</v>
       </c>
       <c r="Q6" t="s">
-        <v>34</v>
+        <v>96</v>
       </c>
       <c r="R6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="S6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="T6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="U6" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="V6"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>20263121</v>
+        <v>20263411</v>
       </c>
       <c r="B7" t="s">
         <v>100</v>
@@ -5566,59 +5566,57 @@
         <v>101</v>
       </c>
       <c r="E7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" t="s">
         <v>102</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
+        <v>53</v>
+      </c>
+      <c r="H7" t="s">
         <v>103</v>
       </c>
-      <c r="G7" t="s">
-        <v>86</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>104</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>105</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>106</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>107</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>108</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>109</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>110</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>111</v>
-      </c>
-      <c r="P7" t="s">
-        <v>112</v>
       </c>
       <c r="Q7" t="s">
         <v>34</v>
       </c>
       <c r="R7" t="s">
+        <v>112</v>
+      </c>
+      <c r="S7" t="s">
         <v>113</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>114</v>
       </c>
-      <c r="T7" t="s">
+      <c r="U7" t="s">
         <v>115</v>
       </c>
-      <c r="U7" t="s">
-        <v>26</v>
-      </c>
-      <c r="V7" t="s">
-        <v>26</v>
-      </c>
+      <c r="V7"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -5631,16 +5629,16 @@
         <v>117</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="E8" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
         <v>118</v>
       </c>
       <c r="G8" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H8" t="s">
         <v>119</v>
@@ -5661,7 +5659,7 @@
         <v>124</v>
       </c>
       <c r="N8" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="O8" t="s">
         <v>125</v>
@@ -5682,7 +5680,7 @@
         <v>129</v>
       </c>
       <c r="U8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="V8"/>
     </row>
@@ -5694,22 +5692,22 @@
         <v>130</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D9" t="s">
         <v>131</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F9" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="G9" t="s">
         <v>27</v>
       </c>
       <c r="H9" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I9" t="s">
         <v>132</v>
@@ -5727,7 +5725,7 @@
         <v>136</v>
       </c>
       <c r="N9" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O9" t="s">
         <v>137</v>
@@ -5736,7 +5734,7 @@
         <v>138</v>
       </c>
       <c r="Q9" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R9" t="s">
         <v>139</v>
@@ -5760,7 +5758,7 @@
         <v>143</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D10" t="s">
         <v>144</v>
@@ -5769,13 +5767,13 @@
         <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="G10" t="s">
         <v>27</v>
       </c>
       <c r="H10" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I10" t="s">
         <v>145</v>
@@ -5793,7 +5791,7 @@
         <v>149</v>
       </c>
       <c r="N10" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O10" t="s">
         <v>150</v>
@@ -5802,16 +5800,16 @@
         <v>151</v>
       </c>
       <c r="Q10" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R10" t="s">
-        <v>113</v>
+        <v>63</v>
       </c>
       <c r="S10" t="s">
-        <v>114</v>
+        <v>64</v>
       </c>
       <c r="T10" t="s">
-        <v>115</v>
+        <v>65</v>
       </c>
       <c r="U10" t="s">
         <v>142</v>
@@ -5826,14 +5824,14 @@
         <v>152</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D11" t="s">
         <v>153</v>
       </c>
       <c r="E11"/>
       <c r="F11" t="s">
-        <v>103</v>
+        <v>52</v>
       </c>
       <c r="G11" t="s">
         <v>27</v>
@@ -5857,7 +5855,7 @@
         <v>158</v>
       </c>
       <c r="N11" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O11" t="s">
         <v>159</v>
@@ -5890,20 +5888,20 @@
         <v>165</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D12" t="s">
         <v>166</v>
       </c>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="G12" t="s">
         <v>27</v>
       </c>
       <c r="H12" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I12" t="s">
         <v>167</v>
@@ -5921,7 +5919,7 @@
         <v>171</v>
       </c>
       <c r="N12" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O12" t="s">
         <v>172</v>
@@ -5930,7 +5928,7 @@
         <v>173</v>
       </c>
       <c r="Q12" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R12" t="s">
         <v>174</v>
@@ -5954,7 +5952,7 @@
         <v>178</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D13" t="s">
         <v>39</v>
@@ -5963,13 +5961,13 @@
         <v>40</v>
       </c>
       <c r="F13" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="G13" t="s">
         <v>27</v>
       </c>
       <c r="H13" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I13" t="s">
         <v>179</v>
@@ -5987,7 +5985,7 @@
         <v>183</v>
       </c>
       <c r="N13" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O13" t="s">
         <v>184</v>
@@ -6020,7 +6018,7 @@
         <v>189</v>
       </c>
       <c r="C14" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D14" t="s">
         <v>190</v>
@@ -6053,7 +6051,7 @@
         <v>197</v>
       </c>
       <c r="N14" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O14" t="s">
         <v>198</v>
@@ -6062,7 +6060,7 @@
         <v>199</v>
       </c>
       <c r="Q14" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R14" t="s">
         <v>200</v>
@@ -6086,7 +6084,7 @@
         <v>203</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D15" t="s">
         <v>204</v>
@@ -6095,13 +6093,13 @@
         <v>40</v>
       </c>
       <c r="F15" t="s">
-        <v>103</v>
+        <v>52</v>
       </c>
       <c r="G15" t="s">
         <v>27</v>
       </c>
       <c r="H15" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I15" t="s">
         <v>205</v>
@@ -6119,7 +6117,7 @@
         <v>209</v>
       </c>
       <c r="N15" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O15" t="s">
         <v>210</v>
@@ -6152,7 +6150,7 @@
         <v>216</v>
       </c>
       <c r="C16" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D16" t="s">
         <v>217</v>
@@ -6167,7 +6165,7 @@
         <v>27</v>
       </c>
       <c r="H16" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I16" t="s">
         <v>219</v>
@@ -6185,7 +6183,7 @@
         <v>223</v>
       </c>
       <c r="N16" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O16" t="s">
         <v>224</v>
@@ -6194,7 +6192,7 @@
         <v>225</v>
       </c>
       <c r="Q16" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R16" t="s">
         <v>186</v>
@@ -6218,19 +6216,19 @@
         <v>226</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D17" t="s">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="E17" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F17" t="s">
         <v>227</v>
       </c>
       <c r="G17" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H17" t="s">
         <v>119</v>
@@ -6299,7 +6297,7 @@
         <v>27</v>
       </c>
       <c r="H18" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I18" t="s">
         <v>243</v>
@@ -6315,7 +6313,7 @@
         <v>246</v>
       </c>
       <c r="N18" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O18" t="s">
         <v>247</v>
@@ -6379,7 +6377,7 @@
         <v>259</v>
       </c>
       <c r="N19" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O19" t="s">
         <v>260</v>
@@ -6388,7 +6386,7 @@
         <v>261</v>
       </c>
       <c r="Q19" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R19" t="s">
         <v>262</v>
@@ -6474,7 +6472,7 @@
         <v>131</v>
       </c>
       <c r="E21" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F21" t="s">
         <v>275</v>
@@ -6483,7 +6481,7 @@
         <v>27</v>
       </c>
       <c r="H21" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I21" t="s">
         <v>276</v>
@@ -6499,7 +6497,7 @@
         <v>279</v>
       </c>
       <c r="N21" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O21" t="s">
         <v>280</v>
@@ -6532,7 +6530,7 @@
         <v>285</v>
       </c>
       <c r="C22" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D22" t="s">
         <v>286</v>
@@ -6545,7 +6543,7 @@
         <v>27</v>
       </c>
       <c r="H22" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I22" t="s">
         <v>288</v>
@@ -6563,7 +6561,7 @@
         <v>292</v>
       </c>
       <c r="N22" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O22" t="s">
         <v>293</v>
@@ -6596,7 +6594,7 @@
         <v>298</v>
       </c>
       <c r="C23" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D23" t="s">
         <v>299</v>
@@ -6611,7 +6609,7 @@
         <v>27</v>
       </c>
       <c r="H23" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I23" t="s">
         <v>301</v>
@@ -6629,7 +6627,7 @@
         <v>305</v>
       </c>
       <c r="N23" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O23" t="s">
         <v>306</v>
@@ -6638,7 +6636,7 @@
         <v>307</v>
       </c>
       <c r="Q23" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R23" t="s">
         <v>308</v>
@@ -6662,7 +6660,7 @@
         <v>311</v>
       </c>
       <c r="C24" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D24" t="s">
         <v>312</v>
@@ -6677,7 +6675,7 @@
         <v>27</v>
       </c>
       <c r="H24" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I24" t="s">
         <v>313</v>
@@ -6695,7 +6693,7 @@
         <v>317</v>
       </c>
       <c r="N24" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O24" t="s">
         <v>318</v>
@@ -6704,7 +6702,7 @@
         <v>319</v>
       </c>
       <c r="Q24" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R24" t="s">
         <v>320</v>
@@ -6728,19 +6726,19 @@
         <v>323</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D25" t="s">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="E25" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F25" t="s">
         <v>324</v>
       </c>
       <c r="G25" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H25" t="s">
         <v>325</v>
@@ -6797,16 +6795,16 @@
         <v>117</v>
       </c>
       <c r="D26" t="s">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="E26" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F26" t="s">
         <v>324</v>
       </c>
       <c r="G26" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H26" t="s">
         <v>119</v>
@@ -6860,22 +6858,22 @@
         <v>349</v>
       </c>
       <c r="C27" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D27" t="s">
         <v>350</v>
       </c>
       <c r="E27" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F27" t="s">
         <v>351</v>
       </c>
       <c r="G27" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H27" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I27" t="s">
         <v>352</v>
@@ -6893,7 +6891,7 @@
         <v>356</v>
       </c>
       <c r="N27" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O27" t="s">
         <v>357</v>
@@ -6902,7 +6900,7 @@
         <v>358</v>
       </c>
       <c r="Q27" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R27" t="s">
         <v>359</v>
@@ -6926,7 +6924,7 @@
         <v>362</v>
       </c>
       <c r="C28" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D28" t="s">
         <v>204</v>
@@ -6941,7 +6939,7 @@
         <v>27</v>
       </c>
       <c r="H28" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I28" t="s">
         <v>364</v>
@@ -6959,7 +6957,7 @@
         <v>368</v>
       </c>
       <c r="N28" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O28" t="s">
         <v>369</v>
@@ -6968,7 +6966,7 @@
         <v>370</v>
       </c>
       <c r="Q28" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R28" t="s">
         <v>295</v>
@@ -6992,7 +6990,7 @@
         <v>371</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D29" t="s">
         <v>241</v>
@@ -7007,7 +7005,7 @@
         <v>27</v>
       </c>
       <c r="H29" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I29" t="s">
         <v>372</v>
@@ -7025,7 +7023,7 @@
         <v>376</v>
       </c>
       <c r="N29" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O29" t="s">
         <v>377</v>
@@ -7089,7 +7087,7 @@
         <v>388</v>
       </c>
       <c r="N30" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O30" t="s">
         <v>389</v>
@@ -7153,7 +7151,7 @@
         <v>398</v>
       </c>
       <c r="N31" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O31" t="s">
         <v>399</v>
@@ -7199,7 +7197,7 @@
         <v>27</v>
       </c>
       <c r="H32" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I32" t="s">
         <v>404</v>
@@ -7250,7 +7248,7 @@
         <v>414</v>
       </c>
       <c r="C33" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D33" t="s">
         <v>415</v>
@@ -7262,10 +7260,10 @@
         <v>416</v>
       </c>
       <c r="G33" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H33" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I33" t="s">
         <v>417</v>
@@ -7283,7 +7281,7 @@
         <v>421</v>
       </c>
       <c r="N33" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O33" t="s">
         <v>422</v>
@@ -7322,7 +7320,7 @@
         <v>428</v>
       </c>
       <c r="E34" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F34" t="s">
         <v>416</v>
@@ -7331,7 +7329,7 @@
         <v>27</v>
       </c>
       <c r="H34" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I34" t="s">
         <v>429</v>
@@ -7349,7 +7347,7 @@
         <v>433</v>
       </c>
       <c r="N34" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O34" t="s">
         <v>434</v>
@@ -7382,7 +7380,7 @@
         <v>436</v>
       </c>
       <c r="C35" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D35" t="s">
         <v>144</v>
@@ -7397,7 +7395,7 @@
         <v>27</v>
       </c>
       <c r="H35" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I35" t="s">
         <v>437</v>
@@ -7415,7 +7413,7 @@
         <v>441</v>
       </c>
       <c r="N35" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O35" t="s">
         <v>442</v>
@@ -7424,7 +7422,7 @@
         <v>443</v>
       </c>
       <c r="Q35" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R35" t="s">
         <v>186</v>
@@ -7448,10 +7446,10 @@
         <v>444</v>
       </c>
       <c r="C36" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D36" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="E36" t="s">
         <v>25</v>
@@ -7460,10 +7458,10 @@
         <v>416</v>
       </c>
       <c r="G36" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H36" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I36" t="s">
         <v>445</v>
@@ -7514,13 +7512,13 @@
         <v>455</v>
       </c>
       <c r="C37" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D37" t="s">
         <v>456</v>
       </c>
       <c r="E37" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F37" t="s">
         <v>457</v>
@@ -7529,7 +7527,7 @@
         <v>27</v>
       </c>
       <c r="H37" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I37" t="s">
         <v>458</v>
@@ -7547,7 +7545,7 @@
         <v>462</v>
       </c>
       <c r="N37" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O37" t="s">
         <v>463</v>
@@ -7556,7 +7554,7 @@
         <v>464</v>
       </c>
       <c r="Q37" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R37" t="s">
         <v>308</v>
@@ -7580,22 +7578,22 @@
         <v>465</v>
       </c>
       <c r="C38" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D38" t="s">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="E38" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F38" t="s">
         <v>466</v>
       </c>
       <c r="G38" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H38" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I38" t="s">
         <v>467</v>
@@ -7613,7 +7611,7 @@
         <v>471</v>
       </c>
       <c r="N38" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O38" t="s">
         <v>472</v>
@@ -7622,7 +7620,7 @@
         <v>473</v>
       </c>
       <c r="Q38" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R38" t="s">
         <v>474</v>
@@ -7646,7 +7644,7 @@
         <v>477</v>
       </c>
       <c r="C39" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D39" t="s">
         <v>478</v>
@@ -7679,7 +7677,7 @@
         <v>483</v>
       </c>
       <c r="N39" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O39" t="s">
         <v>484</v>
@@ -7688,7 +7686,7 @@
         <v>485</v>
       </c>
       <c r="Q39" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R39" t="s">
         <v>486</v>
@@ -7712,22 +7710,22 @@
         <v>489</v>
       </c>
       <c r="C40" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D40" t="s">
         <v>490</v>
       </c>
       <c r="E40" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F40" t="s">
         <v>491</v>
       </c>
       <c r="G40" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H40" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I40" t="s">
         <v>492</v>
@@ -7745,7 +7743,7 @@
         <v>496</v>
       </c>
       <c r="N40" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O40" t="s">
         <v>497</v>
@@ -7754,7 +7752,7 @@
         <v>498</v>
       </c>
       <c r="Q40" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R40" t="s">
         <v>499</v>
@@ -7793,7 +7791,7 @@
         <v>27</v>
       </c>
       <c r="H41" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I41" t="s">
         <v>505</v>
@@ -7844,7 +7842,7 @@
         <v>516</v>
       </c>
       <c r="C42" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D42" t="s">
         <v>517</v>
@@ -7859,7 +7857,7 @@
         <v>27</v>
       </c>
       <c r="H42" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I42" t="s">
         <v>519</v>
@@ -7877,7 +7875,7 @@
         <v>523</v>
       </c>
       <c r="N42" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O42" t="s">
         <v>524</v>
@@ -7925,7 +7923,7 @@
         <v>27</v>
       </c>
       <c r="H43" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I43" t="s">
         <v>532</v>
@@ -7941,7 +7939,7 @@
         <v>535</v>
       </c>
       <c r="N43" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O43" t="s">
         <v>536</v>
@@ -7950,7 +7948,7 @@
         <v>537</v>
       </c>
       <c r="Q43" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R43" t="s">
         <v>308</v>
@@ -7980,7 +7978,7 @@
         <v>539</v>
       </c>
       <c r="E44" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F44" t="s">
         <v>518</v>
@@ -7989,7 +7987,7 @@
         <v>27</v>
       </c>
       <c r="H44" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I44" t="s">
         <v>540</v>
@@ -8005,7 +8003,7 @@
         <v>543</v>
       </c>
       <c r="N44" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O44" t="s">
         <v>544</v>
@@ -8014,7 +8012,7 @@
         <v>545</v>
       </c>
       <c r="Q44" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R44" t="s">
         <v>546</v>
@@ -8069,7 +8067,7 @@
         <v>554</v>
       </c>
       <c r="N45" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O45" t="s">
         <v>555</v>
@@ -8078,7 +8076,7 @@
         <v>556</v>
       </c>
       <c r="Q45" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R45" t="s">
         <v>557</v>
@@ -8102,7 +8100,7 @@
         <v>560</v>
       </c>
       <c r="C46" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D46" t="s">
         <v>561</v>
@@ -8135,7 +8133,7 @@
         <v>567</v>
       </c>
       <c r="N46" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O46" t="s">
         <v>568</v>
@@ -8199,7 +8197,7 @@
         <v>577</v>
       </c>
       <c r="N47" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O47" t="s">
         <v>578</v>
@@ -8288,7 +8286,7 @@
         <v>595</v>
       </c>
       <c r="C49" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D49" t="s">
         <v>596</v>
@@ -8303,7 +8301,7 @@
         <v>27</v>
       </c>
       <c r="H49" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I49" t="s">
         <v>598</v>
@@ -8321,7 +8319,7 @@
         <v>602</v>
       </c>
       <c r="N49" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O49" t="s">
         <v>603</v>
@@ -8330,7 +8328,7 @@
         <v>604</v>
       </c>
       <c r="Q49" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R49" t="s">
         <v>605</v>
@@ -8354,7 +8352,7 @@
         <v>608</v>
       </c>
       <c r="C50" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D50" t="s">
         <v>609</v>
@@ -8369,7 +8367,7 @@
         <v>27</v>
       </c>
       <c r="H50" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I50" t="s">
         <v>610</v>
@@ -8387,7 +8385,7 @@
         <v>614</v>
       </c>
       <c r="N50" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O50" t="s">
         <v>615</v>
@@ -8426,7 +8424,7 @@
         <v>621</v>
       </c>
       <c r="E51" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F51" t="s">
         <v>597</v>
@@ -8435,7 +8433,7 @@
         <v>27</v>
       </c>
       <c r="H51" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I51" t="s">
         <v>622</v>
@@ -8486,7 +8484,7 @@
         <v>633</v>
       </c>
       <c r="C52" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D52" t="s">
         <v>166</v>
@@ -8499,7 +8497,7 @@
         <v>27</v>
       </c>
       <c r="H52" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I52" t="s">
         <v>635</v>
@@ -8517,7 +8515,7 @@
         <v>639</v>
       </c>
       <c r="N52" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O52" t="s">
         <v>640</v>
@@ -8526,7 +8524,7 @@
         <v>641</v>
       </c>
       <c r="Q52" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R52" t="s">
         <v>642</v>
@@ -8550,7 +8548,7 @@
         <v>645</v>
       </c>
       <c r="C53" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D53" t="s">
         <v>646</v>
@@ -8565,7 +8563,7 @@
         <v>27</v>
       </c>
       <c r="H53" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I53" t="s">
         <v>647</v>
@@ -8583,7 +8581,7 @@
         <v>651</v>
       </c>
       <c r="N53" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O53" t="s">
         <v>652</v>
@@ -8592,7 +8590,7 @@
         <v>653</v>
       </c>
       <c r="Q53" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R53" t="s">
         <v>654</v>
@@ -8616,7 +8614,7 @@
         <v>657</v>
       </c>
       <c r="C54" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D54" t="s">
         <v>658</v>
@@ -8631,7 +8629,7 @@
         <v>27</v>
       </c>
       <c r="H54" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I54" t="s">
         <v>660</v>
@@ -8649,7 +8647,7 @@
         <v>664</v>
       </c>
       <c r="N54" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O54" t="s">
         <v>665</v>
@@ -8658,7 +8656,7 @@
         <v>666</v>
       </c>
       <c r="Q54" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R54" t="s">
         <v>186</v>
@@ -8695,7 +8693,7 @@
         <v>27</v>
       </c>
       <c r="H55" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I55" t="s">
         <v>669</v>
@@ -8746,13 +8744,13 @@
         <v>679</v>
       </c>
       <c r="C56" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D56" t="s">
         <v>428</v>
       </c>
       <c r="E56" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F56" t="s">
         <v>659</v>
@@ -8761,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="H56" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I56" t="s">
         <v>680</v>
@@ -8779,7 +8777,7 @@
         <v>684</v>
       </c>
       <c r="N56" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O56" t="s">
         <v>685</v>
@@ -8788,7 +8786,7 @@
         <v>686</v>
       </c>
       <c r="Q56" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R56" t="s">
         <v>687</v>
@@ -8812,7 +8810,7 @@
         <v>690</v>
       </c>
       <c r="C57" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D57" t="s">
         <v>691</v>
@@ -8824,10 +8822,10 @@
         <v>692</v>
       </c>
       <c r="G57" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H57" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I57" t="s">
         <v>693</v>
@@ -8845,7 +8843,7 @@
         <v>697</v>
       </c>
       <c r="N57" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O57" t="s">
         <v>698</v>
@@ -8878,7 +8876,7 @@
         <v>700</v>
       </c>
       <c r="C58" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D58" t="s">
         <v>701</v>
@@ -8893,7 +8891,7 @@
         <v>27</v>
       </c>
       <c r="H58" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I58" t="s">
         <v>703</v>
@@ -8911,7 +8909,7 @@
         <v>707</v>
       </c>
       <c r="N58" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O58" t="s">
         <v>708</v>
@@ -8923,13 +8921,13 @@
         <v>161</v>
       </c>
       <c r="R58" t="s">
-        <v>113</v>
+        <v>63</v>
       </c>
       <c r="S58" t="s">
-        <v>114</v>
+        <v>64</v>
       </c>
       <c r="T58" t="s">
-        <v>115</v>
+        <v>65</v>
       </c>
       <c r="U58" t="s">
         <v>252</v>
@@ -8944,7 +8942,7 @@
         <v>710</v>
       </c>
       <c r="C59" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D59" t="s">
         <v>711</v>
@@ -8959,7 +8957,7 @@
         <v>27</v>
       </c>
       <c r="H59" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I59" t="s">
         <v>714</v>
@@ -8977,7 +8975,7 @@
         <v>718</v>
       </c>
       <c r="N59" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O59" t="s">
         <v>719</v>
@@ -8986,7 +8984,7 @@
         <v>720</v>
       </c>
       <c r="Q59" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R59" t="s">
         <v>721</v>
@@ -9010,7 +9008,7 @@
         <v>724</v>
       </c>
       <c r="C60" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D60" t="s">
         <v>478</v>
@@ -9025,7 +9023,7 @@
         <v>27</v>
       </c>
       <c r="H60" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I60" t="s">
         <v>725</v>
@@ -9043,7 +9041,7 @@
         <v>729</v>
       </c>
       <c r="N60" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O60" t="s">
         <v>730</v>
@@ -9052,7 +9050,7 @@
         <v>731</v>
       </c>
       <c r="Q60" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R60" t="s">
         <v>732</v>
@@ -9076,7 +9074,7 @@
         <v>735</v>
       </c>
       <c r="C61" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D61" t="s">
         <v>286</v>
@@ -9089,7 +9087,7 @@
         <v>27</v>
       </c>
       <c r="H61" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I61" t="s">
         <v>737</v>
@@ -9116,7 +9114,7 @@
         <v>743</v>
       </c>
       <c r="Q61" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R61" t="s">
         <v>732</v>
@@ -9146,7 +9144,7 @@
         <v>745</v>
       </c>
       <c r="E62" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F62" t="s">
         <v>746</v>
@@ -9206,13 +9204,13 @@
         <v>758</v>
       </c>
       <c r="C63" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D63" t="s">
         <v>759</v>
       </c>
       <c r="E63" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F63" t="s">
         <v>746</v>
@@ -9221,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="H63" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I63" t="s">
         <v>760</v>
@@ -9239,7 +9237,7 @@
         <v>764</v>
       </c>
       <c r="N63" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O63" t="s">
         <v>765</v>
@@ -9272,13 +9270,13 @@
         <v>770</v>
       </c>
       <c r="C64" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D64" t="s">
         <v>771</v>
       </c>
       <c r="E64" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F64" t="s">
         <v>746</v>
@@ -9287,7 +9285,7 @@
         <v>27</v>
       </c>
       <c r="H64" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I64" t="s">
         <v>772</v>
@@ -9305,7 +9303,7 @@
         <v>776</v>
       </c>
       <c r="N64" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O64" t="s">
         <v>777</v>
@@ -9314,7 +9312,7 @@
         <v>778</v>
       </c>
       <c r="Q64" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R64" t="s">
         <v>526</v>
@@ -9338,22 +9336,22 @@
         <v>779</v>
       </c>
       <c r="C65" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D65" t="s">
         <v>780</v>
       </c>
       <c r="E65" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F65" t="s">
         <v>781</v>
       </c>
       <c r="G65" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H65" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I65" t="s">
         <v>782</v>
@@ -9371,7 +9369,7 @@
         <v>786</v>
       </c>
       <c r="N65" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O65" t="s">
         <v>787</v>
@@ -9380,7 +9378,7 @@
         <v>788</v>
       </c>
       <c r="Q65" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R65" t="s">
         <v>789</v>
@@ -9404,22 +9402,22 @@
         <v>792</v>
       </c>
       <c r="C66" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D66" t="s">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="E66" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F66" t="s">
         <v>781</v>
       </c>
       <c r="G66" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H66" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I66" t="s">
         <v>793</v>
@@ -9446,7 +9444,7 @@
         <v>799</v>
       </c>
       <c r="Q66" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R66" t="s">
         <v>732</v>
@@ -9470,22 +9468,22 @@
         <v>800</v>
       </c>
       <c r="C67" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D67" t="s">
         <v>350</v>
       </c>
       <c r="E67" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F67" t="s">
         <v>801</v>
       </c>
       <c r="G67" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H67" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I67" t="s">
         <v>802</v>
@@ -9503,7 +9501,7 @@
         <v>806</v>
       </c>
       <c r="N67" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O67" t="s">
         <v>807</v>
@@ -9512,7 +9510,7 @@
         <v>808</v>
       </c>
       <c r="Q67" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R67" t="s">
         <v>809</v>
@@ -9536,7 +9534,7 @@
         <v>812</v>
       </c>
       <c r="C68" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D68" t="s">
         <v>646</v>
@@ -9551,7 +9549,7 @@
         <v>27</v>
       </c>
       <c r="H68" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I68" t="s">
         <v>814</v>
@@ -9569,7 +9567,7 @@
         <v>818</v>
       </c>
       <c r="N68" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O68" t="s">
         <v>819</v>
@@ -9613,7 +9611,7 @@
       </c>
       <c r="G69"/>
       <c r="H69" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I69" t="s">
         <v>827</v>
@@ -9687,7 +9685,7 @@
         <v>838</v>
       </c>
       <c r="N70" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O70" t="s">
         <v>839</v>
@@ -9724,7 +9722,7 @@
         <v>843</v>
       </c>
       <c r="G71" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H71" t="s">
         <v>119</v>
@@ -9793,7 +9791,7 @@
         <v>27</v>
       </c>
       <c r="H72" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I72" t="s">
         <v>856</v>
@@ -9811,7 +9809,7 @@
         <v>860</v>
       </c>
       <c r="N72" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O72" t="s">
         <v>861</v>
@@ -9844,7 +9842,7 @@
         <v>866</v>
       </c>
       <c r="C73" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D73" t="s">
         <v>711</v>
@@ -9859,7 +9857,7 @@
         <v>27</v>
       </c>
       <c r="H73" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I73" t="s">
         <v>867</v>
@@ -9877,7 +9875,7 @@
         <v>871</v>
       </c>
       <c r="N73" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O73" t="s">
         <v>872</v>
@@ -9886,7 +9884,7 @@
         <v>873</v>
       </c>
       <c r="Q73" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R73" t="s">
         <v>874</v>
@@ -9910,13 +9908,13 @@
         <v>877</v>
       </c>
       <c r="C74" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D74" t="s">
         <v>878</v>
       </c>
       <c r="E74" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F74" t="s">
         <v>855</v>
@@ -9943,7 +9941,7 @@
         <v>883</v>
       </c>
       <c r="N74" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O74" t="s">
         <v>884</v>
@@ -9952,7 +9950,7 @@
         <v>885</v>
       </c>
       <c r="Q74" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R74" t="s">
         <v>886</v>
@@ -9976,13 +9974,13 @@
         <v>889</v>
       </c>
       <c r="C75" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D75" t="s">
         <v>428</v>
       </c>
       <c r="E75" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F75" t="s">
         <v>855</v>
@@ -9991,7 +9989,7 @@
         <v>27</v>
       </c>
       <c r="H75" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I75" t="s">
         <v>890</v>
@@ -10018,7 +10016,7 @@
         <v>896</v>
       </c>
       <c r="Q75" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R75" t="s">
         <v>897</v>
@@ -10042,7 +10040,7 @@
         <v>900</v>
       </c>
       <c r="C76" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D76" t="s">
         <v>901</v>
@@ -10075,7 +10073,7 @@
         <v>906</v>
       </c>
       <c r="N76" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O76" t="s">
         <v>907</v>
@@ -10084,7 +10082,7 @@
         <v>908</v>
       </c>
       <c r="Q76" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R76" t="s">
         <v>909</v>
@@ -10108,7 +10106,7 @@
         <v>912</v>
       </c>
       <c r="C77" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D77" t="s">
         <v>913</v>
@@ -10123,7 +10121,7 @@
         <v>27</v>
       </c>
       <c r="H77" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I77" t="s">
         <v>914</v>
@@ -10141,7 +10139,7 @@
         <v>918</v>
       </c>
       <c r="N77" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O77" t="s">
         <v>919</v>
@@ -10150,7 +10148,7 @@
         <v>920</v>
       </c>
       <c r="Q77" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R77" t="s">
         <v>921</v>
@@ -10180,7 +10178,7 @@
         <v>539</v>
       </c>
       <c r="E78" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F78" t="s">
         <v>925</v>
@@ -10189,7 +10187,7 @@
         <v>27</v>
       </c>
       <c r="H78" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I78" t="s">
         <v>926</v>
@@ -10207,7 +10205,7 @@
         <v>930</v>
       </c>
       <c r="N78" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O78" t="s">
         <v>931</v>
@@ -10240,7 +10238,7 @@
         <v>936</v>
       </c>
       <c r="C79" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D79" t="s">
         <v>937</v>
@@ -10255,7 +10253,7 @@
         <v>27</v>
       </c>
       <c r="H79" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I79" t="s">
         <v>938</v>
@@ -10273,7 +10271,7 @@
         <v>942</v>
       </c>
       <c r="N79" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O79" t="s">
         <v>943</v>
@@ -10282,7 +10280,7 @@
         <v>944</v>
       </c>
       <c r="Q79" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R79" t="s">
         <v>945</v>
@@ -10317,7 +10315,7 @@
       </c>
       <c r="G80"/>
       <c r="H80" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I80" t="s">
         <v>950</v>
@@ -10362,7 +10360,7 @@
         <v>957</v>
       </c>
       <c r="C81" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D81" t="s">
         <v>39</v>
@@ -10377,7 +10375,7 @@
         <v>27</v>
       </c>
       <c r="H81" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I81" t="s">
         <v>417</v>
@@ -10395,7 +10393,7 @@
         <v>962</v>
       </c>
       <c r="N81" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O81" t="s">
         <v>963</v>
@@ -10459,7 +10457,7 @@
         <v>971</v>
       </c>
       <c r="N82" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O82" t="s">
         <v>972</v>
@@ -10507,7 +10505,7 @@
         <v>27</v>
       </c>
       <c r="H83" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I83" t="s">
         <v>980</v>
@@ -10523,7 +10521,7 @@
         <v>983</v>
       </c>
       <c r="N83" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O83" t="s">
         <v>984</v>
@@ -10579,7 +10577,7 @@
       <c r="L84"/>
       <c r="M84"/>
       <c r="N84" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O84" t="s">
         <v>991</v>
@@ -10623,7 +10621,7 @@
       </c>
       <c r="G85"/>
       <c r="H85" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I85" t="s">
         <v>998</v>
@@ -10685,7 +10683,7 @@
       </c>
       <c r="G86"/>
       <c r="H86" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I86" t="s">
         <v>1009</v>
@@ -10736,7 +10734,7 @@
         <v>1020</v>
       </c>
       <c r="C87" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D87" t="s">
         <v>711</v>
@@ -10751,7 +10749,7 @@
         <v>27</v>
       </c>
       <c r="H87" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I87" t="s">
         <v>1022</v>
@@ -10769,7 +10767,7 @@
         <v>1026</v>
       </c>
       <c r="N87" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O87" t="s">
         <v>1027</v>
@@ -10778,7 +10776,7 @@
         <v>1028</v>
       </c>
       <c r="Q87" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R87" t="s">
         <v>1029</v>
@@ -10802,13 +10800,13 @@
         <v>1032</v>
       </c>
       <c r="C88" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D88" t="s">
         <v>1033</v>
       </c>
       <c r="E88" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F88" t="s">
         <v>1034</v>
@@ -10817,7 +10815,7 @@
         <v>27</v>
       </c>
       <c r="H88" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I88" t="s">
         <v>1035</v>
@@ -10835,7 +10833,7 @@
         <v>1039</v>
       </c>
       <c r="N88" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O88" t="s">
         <v>1040</v>
@@ -10844,7 +10842,7 @@
         <v>1041</v>
       </c>
       <c r="Q88" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R88" t="s">
         <v>1042</v>
@@ -10868,7 +10866,7 @@
         <v>1045</v>
       </c>
       <c r="C89" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D89" t="s">
         <v>1046</v>
@@ -10883,7 +10881,7 @@
         <v>27</v>
       </c>
       <c r="H89" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I89" t="s">
         <v>1047</v>
@@ -10901,7 +10899,7 @@
         <v>1051</v>
       </c>
       <c r="N89" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O89" t="s">
         <v>1052</v>
@@ -10934,7 +10932,7 @@
         <v>1054</v>
       </c>
       <c r="C90" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D90" t="s">
         <v>1055</v>
@@ -10949,7 +10947,7 @@
         <v>27</v>
       </c>
       <c r="H90" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I90" t="s">
         <v>1056</v>
@@ -10967,7 +10965,7 @@
         <v>1060</v>
       </c>
       <c r="N90" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O90" t="s">
         <v>1061</v>
@@ -10976,7 +10974,7 @@
         <v>1062</v>
       </c>
       <c r="Q90" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R90" t="s">
         <v>1063</v>
@@ -11000,13 +10998,13 @@
         <v>1066</v>
       </c>
       <c r="C91" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D91" t="s">
         <v>1067</v>
       </c>
       <c r="E91" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F91" t="s">
         <v>1034</v>
@@ -11015,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="H91" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I91" t="s">
         <v>1068</v>
@@ -11033,7 +11031,7 @@
         <v>1072</v>
       </c>
       <c r="N91" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O91" t="s">
         <v>1073</v>
@@ -11042,7 +11040,7 @@
         <v>1074</v>
       </c>
       <c r="Q91" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R91" t="s">
         <v>605</v>
@@ -11066,13 +11064,13 @@
         <v>1075</v>
       </c>
       <c r="C92" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D92" t="s">
         <v>1076</v>
       </c>
       <c r="E92" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F92" t="s">
         <v>1077</v>
@@ -11081,7 +11079,7 @@
         <v>27</v>
       </c>
       <c r="H92" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I92" t="s">
         <v>1078</v>
@@ -11099,7 +11097,7 @@
         <v>1082</v>
       </c>
       <c r="N92" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O92" t="s">
         <v>1083</v>
@@ -11108,7 +11106,7 @@
         <v>1084</v>
       </c>
       <c r="Q92" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R92" t="s">
         <v>391</v>
@@ -11163,7 +11161,7 @@
         <v>1090</v>
       </c>
       <c r="N93" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O93" t="s">
         <v>1091</v>
@@ -11172,7 +11170,7 @@
         <v>1092</v>
       </c>
       <c r="Q93" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R93" t="s">
         <v>200</v>
@@ -11196,13 +11194,13 @@
         <v>1093</v>
       </c>
       <c r="C94" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D94" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="E94" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F94" t="s">
         <v>1094</v>
@@ -11211,7 +11209,7 @@
         <v>27</v>
       </c>
       <c r="H94" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I94" t="s">
         <v>1095</v>
@@ -11229,7 +11227,7 @@
         <v>1099</v>
       </c>
       <c r="N94" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O94" t="s">
         <v>1100</v>
@@ -11238,7 +11236,7 @@
         <v>1101</v>
       </c>
       <c r="Q94" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R94" t="s">
         <v>186</v>
@@ -11268,7 +11266,7 @@
         <v>1067</v>
       </c>
       <c r="E95" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F95" t="s">
         <v>1103</v>
@@ -11277,7 +11275,7 @@
         <v>27</v>
       </c>
       <c r="H95" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I95" t="s">
         <v>1104</v>
@@ -11293,7 +11291,7 @@
         <v>1107</v>
       </c>
       <c r="N95" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O95" t="s">
         <v>1108</v>
@@ -11357,7 +11355,7 @@
         <v>1114</v>
       </c>
       <c r="N96" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O96" t="s">
         <v>1115</v>
@@ -11366,7 +11364,7 @@
         <v>1116</v>
       </c>
       <c r="Q96" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R96" t="s">
         <v>200</v>
@@ -11421,7 +11419,7 @@
         <v>1119</v>
       </c>
       <c r="N97" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O97" t="s">
         <v>1120</v>
@@ -11430,7 +11428,7 @@
         <v>1121</v>
       </c>
       <c r="Q97" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R97" t="s">
         <v>200</v>
@@ -11485,7 +11483,7 @@
         <v>1124</v>
       </c>
       <c r="N98" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O98" t="s">
         <v>1125</v>
@@ -11494,7 +11492,7 @@
         <v>1126</v>
       </c>
       <c r="Q98" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R98" t="s">
         <v>200</v>
@@ -11518,7 +11516,7 @@
         <v>1127</v>
       </c>
       <c r="C99" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D99" t="s">
         <v>561</v>
@@ -11533,7 +11531,7 @@
         <v>27</v>
       </c>
       <c r="H99" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I99" t="s">
         <v>1129</v>
@@ -11551,7 +11549,7 @@
         <v>1133</v>
       </c>
       <c r="N99" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O99" t="s">
         <v>1134</v>
@@ -11584,13 +11582,13 @@
         <v>1139</v>
       </c>
       <c r="C100" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D100" t="s">
         <v>621</v>
       </c>
       <c r="E100" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F100" t="s">
         <v>1140</v>
@@ -11599,7 +11597,7 @@
         <v>27</v>
       </c>
       <c r="H100" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I100" t="s">
         <v>1141</v>
@@ -11617,7 +11615,7 @@
         <v>1145</v>
       </c>
       <c r="N100" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O100" t="s">
         <v>1146</v>
@@ -11650,7 +11648,7 @@
         <v>1148</v>
       </c>
       <c r="C101" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D101" t="s">
         <v>1149</v>
@@ -11665,7 +11663,7 @@
         <v>27</v>
       </c>
       <c r="H101" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I101" t="s">
         <v>1150</v>
@@ -11683,7 +11681,7 @@
         <v>1154</v>
       </c>
       <c r="N101" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O101" t="s">
         <v>1155</v>
@@ -11716,13 +11714,13 @@
         <v>1160</v>
       </c>
       <c r="C102" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D102" t="s">
         <v>1161</v>
       </c>
       <c r="E102" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F102" t="s">
         <v>1140</v>
@@ -11731,7 +11729,7 @@
         <v>27</v>
       </c>
       <c r="H102" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I102" t="s">
         <v>1162</v>
@@ -11749,7 +11747,7 @@
         <v>1166</v>
       </c>
       <c r="N102" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O102" t="s">
         <v>1167</v>
@@ -11758,7 +11756,7 @@
         <v>1168</v>
       </c>
       <c r="Q102" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R102" t="s">
         <v>1169</v>
@@ -11844,13 +11842,13 @@
         <v>1184</v>
       </c>
       <c r="C104" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D104" t="s">
         <v>456</v>
       </c>
       <c r="E104" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F104" t="s">
         <v>1173</v>
@@ -11859,7 +11857,7 @@
         <v>27</v>
       </c>
       <c r="H104" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I104" t="s">
         <v>1185</v>
@@ -11877,7 +11875,7 @@
         <v>1189</v>
       </c>
       <c r="N104" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O104" t="s">
         <v>1190</v>
@@ -11886,7 +11884,7 @@
         <v>1191</v>
       </c>
       <c r="Q104" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R104" t="s">
         <v>1192</v>
@@ -11910,13 +11908,13 @@
         <v>1195</v>
       </c>
       <c r="C105" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D105" t="s">
         <v>1196</v>
       </c>
       <c r="E105" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F105" t="s">
         <v>1173</v>
@@ -11925,7 +11923,7 @@
         <v>27</v>
       </c>
       <c r="H105" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I105" t="s">
         <v>1197</v>
@@ -11943,7 +11941,7 @@
         <v>1201</v>
       </c>
       <c r="N105" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O105" t="s">
         <v>1202</v>
@@ -11952,7 +11950,7 @@
         <v>1203</v>
       </c>
       <c r="Q105" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R105" t="s">
         <v>1204</v>
@@ -11976,7 +11974,7 @@
         <v>1207</v>
       </c>
       <c r="C106" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D106" t="s">
         <v>1208</v>
@@ -11991,7 +11989,7 @@
         <v>27</v>
       </c>
       <c r="H106" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I106" t="s">
         <v>1209</v>
@@ -12009,7 +12007,7 @@
         <v>1213</v>
       </c>
       <c r="N106" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O106" t="s">
         <v>1214</v>
@@ -12018,7 +12016,7 @@
         <v>1215</v>
       </c>
       <c r="Q106" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R106" t="s">
         <v>874</v>
@@ -12042,7 +12040,7 @@
         <v>1216</v>
       </c>
       <c r="C107" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D107" t="s">
         <v>609</v>
@@ -12057,7 +12055,7 @@
         <v>27</v>
       </c>
       <c r="H107" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I107" t="s">
         <v>1217</v>
@@ -12075,7 +12073,7 @@
         <v>1221</v>
       </c>
       <c r="N107" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O107" t="s">
         <v>1222</v>
@@ -12084,7 +12082,7 @@
         <v>1223</v>
       </c>
       <c r="Q107" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R107" t="s">
         <v>1224</v>
@@ -12108,7 +12106,7 @@
         <v>1227</v>
       </c>
       <c r="C108" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D108" t="s">
         <v>561</v>
@@ -12123,7 +12121,7 @@
         <v>27</v>
       </c>
       <c r="H108" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I108" t="s">
         <v>1228</v>
@@ -12174,7 +12172,7 @@
         <v>1239</v>
       </c>
       <c r="C109" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D109" t="s">
         <v>39</v>
@@ -12189,7 +12187,7 @@
         <v>27</v>
       </c>
       <c r="H109" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I109" t="s">
         <v>1241</v>
@@ -12207,7 +12205,7 @@
         <v>1245</v>
       </c>
       <c r="N109" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O109" t="s">
         <v>1246</v>
@@ -12240,13 +12238,13 @@
         <v>1248</v>
       </c>
       <c r="C110" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D110" t="s">
         <v>428</v>
       </c>
       <c r="E110" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F110" t="s">
         <v>1249</v>
@@ -12255,7 +12253,7 @@
         <v>27</v>
       </c>
       <c r="H110" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I110" t="s">
         <v>1250</v>
@@ -12273,7 +12271,7 @@
         <v>1254</v>
       </c>
       <c r="N110" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O110" t="s">
         <v>1255</v>
@@ -12282,7 +12280,7 @@
         <v>1256</v>
       </c>
       <c r="Q110" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R110" t="s">
         <v>732</v>
@@ -12321,7 +12319,7 @@
         <v>27</v>
       </c>
       <c r="H111" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I111" t="s">
         <v>1260</v>
@@ -12337,7 +12335,7 @@
         <v>1263</v>
       </c>
       <c r="N111" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O111" t="s">
         <v>1264</v>
@@ -12385,7 +12383,7 @@
         <v>27</v>
       </c>
       <c r="H112" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I112" t="s">
         <v>1268</v>
@@ -12401,7 +12399,7 @@
         <v>1271</v>
       </c>
       <c r="N112" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O112" t="s">
         <v>1272</v>
@@ -12449,7 +12447,7 @@
         <v>27</v>
       </c>
       <c r="H113" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I113" t="s">
         <v>1279</v>
@@ -12467,7 +12465,7 @@
         <v>1283</v>
       </c>
       <c r="N113" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="O113" t="s">
         <v>1284</v>
@@ -12476,7 +12474,7 @@
         <v>1285</v>
       </c>
       <c r="Q113" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R113" t="s">
         <v>809</v>
@@ -12618,7 +12616,7 @@
         <v>1309</v>
       </c>
       <c r="C116" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D116" t="s">
         <v>1310</v>
@@ -12633,7 +12631,7 @@
         <v>27</v>
       </c>
       <c r="H116" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I116" t="s">
         <v>1312</v>
@@ -12651,7 +12649,7 @@
         <v>1316</v>
       </c>
       <c r="N116" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O116" t="s">
         <v>1317</v>
@@ -12660,7 +12658,7 @@
         <v>1318</v>
       </c>
       <c r="Q116" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R116" t="s">
         <v>1319</v>
@@ -12684,7 +12682,7 @@
         <v>1322</v>
       </c>
       <c r="C117" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D117" t="s">
         <v>1323</v>
@@ -12699,7 +12697,7 @@
         <v>27</v>
       </c>
       <c r="H117" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I117" t="s">
         <v>1325</v>
@@ -12717,7 +12715,7 @@
         <v>1329</v>
       </c>
       <c r="N117" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O117" t="s">
         <v>1330</v>
@@ -12726,7 +12724,7 @@
         <v>1331</v>
       </c>
       <c r="Q117" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R117" t="s">
         <v>1332</v>
@@ -12750,10 +12748,10 @@
         <v>1335</v>
       </c>
       <c r="C118" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D118" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="E118" t="s">
         <v>25</v>
@@ -12762,10 +12760,10 @@
         <v>1324</v>
       </c>
       <c r="G118" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H118" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I118" t="s">
         <v>1336</v>
@@ -12783,7 +12781,7 @@
         <v>1340</v>
       </c>
       <c r="N118" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O118" t="s">
         <v>1341</v>
@@ -12822,16 +12820,16 @@
         <v>350</v>
       </c>
       <c r="E119" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F119" t="s">
         <v>1344</v>
       </c>
       <c r="G119" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H119" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I119" t="s">
         <v>1345</v>
@@ -12858,7 +12856,7 @@
         <v>1351</v>
       </c>
       <c r="Q119" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R119" t="s">
         <v>1181</v>
@@ -12882,13 +12880,13 @@
         <v>1352</v>
       </c>
       <c r="C120" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D120" t="s">
         <v>1353</v>
       </c>
       <c r="E120" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F120" t="s">
         <v>1344</v>
@@ -12897,7 +12895,7 @@
         <v>27</v>
       </c>
       <c r="H120" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I120" t="s">
         <v>1354</v>
@@ -12924,7 +12922,7 @@
         <v>1360</v>
       </c>
       <c r="Q120" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R120" t="s">
         <v>1361</v>
@@ -12948,7 +12946,7 @@
         <v>1364</v>
       </c>
       <c r="C121" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D121" t="s">
         <v>1365</v>
@@ -12963,7 +12961,7 @@
         <v>27</v>
       </c>
       <c r="H121" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I121" t="s">
         <v>1367</v>
@@ -12981,7 +12979,7 @@
         <v>1371</v>
       </c>
       <c r="N121" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O121" t="s">
         <v>1372</v>
@@ -12990,7 +12988,7 @@
         <v>1373</v>
       </c>
       <c r="Q121" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R121" t="s">
         <v>1374</v>
@@ -13014,7 +13012,7 @@
         <v>1377</v>
       </c>
       <c r="C122" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D122" t="s">
         <v>312</v>
@@ -13029,7 +13027,7 @@
         <v>27</v>
       </c>
       <c r="H122" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I122" t="s">
         <v>1378</v>
@@ -13047,7 +13045,7 @@
         <v>1382</v>
       </c>
       <c r="N122" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O122" t="s">
         <v>1383</v>
@@ -13080,13 +13078,13 @@
         <v>1388</v>
       </c>
       <c r="C123" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D123" t="s">
         <v>1353</v>
       </c>
       <c r="E123" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F123" t="s">
         <v>1344</v>
@@ -13095,7 +13093,7 @@
         <v>27</v>
       </c>
       <c r="H123" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I123" t="s">
         <v>1389</v>
@@ -13113,7 +13111,7 @@
         <v>1393</v>
       </c>
       <c r="N123" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O123" t="s">
         <v>1394</v>
@@ -13146,7 +13144,7 @@
         <v>1399</v>
       </c>
       <c r="C124" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D124" t="s">
         <v>1055</v>
@@ -13161,7 +13159,7 @@
         <v>27</v>
       </c>
       <c r="H124" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I124" t="s">
         <v>1400</v>
@@ -13179,7 +13177,7 @@
         <v>1404</v>
       </c>
       <c r="N124" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O124" t="s">
         <v>1405</v>
@@ -13188,7 +13186,7 @@
         <v>1406</v>
       </c>
       <c r="Q124" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R124" t="s">
         <v>1407</v>
@@ -13212,13 +13210,13 @@
         <v>1410</v>
       </c>
       <c r="C125" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D125" t="s">
         <v>1411</v>
       </c>
       <c r="E125" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F125" t="s">
         <v>1412</v>
@@ -13227,7 +13225,7 @@
         <v>27</v>
       </c>
       <c r="H125" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I125" t="s">
         <v>1413</v>
@@ -13245,7 +13243,7 @@
         <v>1417</v>
       </c>
       <c r="N125" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O125" t="s">
         <v>1418</v>
@@ -13254,7 +13252,7 @@
         <v>1419</v>
       </c>
       <c r="Q125" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R125" t="s">
         <v>732</v>
@@ -13278,7 +13276,7 @@
         <v>1420</v>
       </c>
       <c r="C126" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D126" t="s">
         <v>204</v>
@@ -13293,7 +13291,7 @@
         <v>27</v>
       </c>
       <c r="H126" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="I126" t="s">
         <v>1422</v>
@@ -13311,7 +13309,7 @@
         <v>1426</v>
       </c>
       <c r="N126" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O126" t="s">
         <v>1427</v>
@@ -13344,7 +13342,7 @@
         <v>1429</v>
       </c>
       <c r="C127" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D127" t="s">
         <v>1430</v>
@@ -13356,10 +13354,10 @@
         <v>1431</v>
       </c>
       <c r="G127" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H127" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I127" t="s">
         <v>1432</v>
@@ -13377,7 +13375,7 @@
         <v>1436</v>
       </c>
       <c r="N127" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O127" t="s">
         <v>1437</v>
@@ -13422,10 +13420,10 @@
         <v>1441</v>
       </c>
       <c r="G128" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H128" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I128" t="s">
         <v>1442</v>
@@ -13491,7 +13489,7 @@
         <v>27</v>
       </c>
       <c r="H129" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I129" t="s">
         <v>1450</v>
@@ -13507,7 +13505,7 @@
         <v>1453</v>
       </c>
       <c r="N129" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O129" t="s">
         <v>1454</v>
@@ -13516,7 +13514,7 @@
         <v>1455</v>
       </c>
       <c r="Q129" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R129" t="s">
         <v>186</v>
@@ -13555,7 +13553,7 @@
         <v>27</v>
       </c>
       <c r="H130" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I130" t="s">
         <v>1458</v>
@@ -13571,7 +13569,7 @@
         <v>1461</v>
       </c>
       <c r="N130" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O130" t="s">
         <v>1462</v>
@@ -13604,10 +13602,10 @@
         <v>1464</v>
       </c>
       <c r="C131" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D131" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="E131"/>
       <c r="F131" t="s">
@@ -13617,7 +13615,7 @@
         <v>27</v>
       </c>
       <c r="H131" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I131" t="s">
         <v>1466</v>
@@ -13644,7 +13642,7 @@
         <v>1472</v>
       </c>
       <c r="Q131" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R131" t="s">
         <v>1473</v>
@@ -13668,13 +13666,13 @@
         <v>1476</v>
       </c>
       <c r="C132" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D132" t="s">
         <v>771</v>
       </c>
       <c r="E132" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F132" t="s">
         <v>1477</v>
@@ -13683,7 +13681,7 @@
         <v>27</v>
       </c>
       <c r="H132" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I132" t="s">
         <v>1478</v>
@@ -13701,7 +13699,7 @@
         <v>1482</v>
       </c>
       <c r="N132" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O132" t="s">
         <v>1483</v>
@@ -13710,7 +13708,7 @@
         <v>1484</v>
       </c>
       <c r="Q132" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R132" t="s">
         <v>1485</v>
@@ -13734,7 +13732,7 @@
         <v>1488</v>
       </c>
       <c r="C133" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D133" t="s">
         <v>596</v>
@@ -13749,7 +13747,7 @@
         <v>27</v>
       </c>
       <c r="H133" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I133" t="s">
         <v>1489</v>
@@ -13767,7 +13765,7 @@
         <v>1493</v>
       </c>
       <c r="N133" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O133" t="s">
         <v>1494</v>
@@ -13776,7 +13774,7 @@
         <v>1495</v>
       </c>
       <c r="Q133" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R133" t="s">
         <v>1496</v>
@@ -13800,7 +13798,7 @@
         <v>1499</v>
       </c>
       <c r="C134" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D134" t="s">
         <v>1500</v>
@@ -13812,7 +13810,7 @@
         <v>1501</v>
       </c>
       <c r="G134" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H134" t="s">
         <v>747</v>
@@ -13833,7 +13831,7 @@
         <v>1506</v>
       </c>
       <c r="N134" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O134" t="s">
         <v>1507</v>
@@ -13842,7 +13840,7 @@
         <v>1508</v>
       </c>
       <c r="Q134" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R134" t="s">
         <v>1509</v>
@@ -13866,7 +13864,7 @@
         <v>1512</v>
       </c>
       <c r="C135" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D135" t="s">
         <v>901</v>
@@ -13899,7 +13897,7 @@
         <v>1506</v>
       </c>
       <c r="N135" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O135" t="s">
         <v>1513</v>
@@ -13908,7 +13906,7 @@
         <v>1514</v>
       </c>
       <c r="Q135" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R135" t="s">
         <v>1515</v>
@@ -13932,7 +13930,7 @@
         <v>1518</v>
       </c>
       <c r="C136" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D136" t="s">
         <v>1519</v>
@@ -13947,7 +13945,7 @@
         <v>27</v>
       </c>
       <c r="H136" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I136" t="s">
         <v>1521</v>
@@ -13965,7 +13963,7 @@
         <v>1525</v>
       </c>
       <c r="N136" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O136" t="s">
         <v>1526</v>
@@ -13974,7 +13972,7 @@
         <v>1527</v>
       </c>
       <c r="Q136" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R136" t="s">
         <v>526</v>
@@ -13998,22 +13996,22 @@
         <v>1528</v>
       </c>
       <c r="C137" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D137" t="s">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="E137" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F137" t="s">
         <v>1529</v>
       </c>
       <c r="G137" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="H137" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I137" t="s">
         <v>1530</v>
@@ -14031,7 +14029,7 @@
         <v>1534</v>
       </c>
       <c r="N137" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O137" t="s">
         <v>1535</v>
@@ -14064,7 +14062,7 @@
         <v>1540</v>
       </c>
       <c r="C138" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D138" t="s">
         <v>561</v>
@@ -14079,7 +14077,7 @@
         <v>27</v>
       </c>
       <c r="H138" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I138" t="s">
         <v>1542</v>
@@ -14097,7 +14095,7 @@
         <v>1546</v>
       </c>
       <c r="N138" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O138" t="s">
         <v>1547</v>
@@ -14136,7 +14134,7 @@
         <v>1553</v>
       </c>
       <c r="E139" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F139" t="s">
         <v>1541</v>
@@ -14145,7 +14143,7 @@
         <v>27</v>
       </c>
       <c r="H139" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I139" t="s">
         <v>1554</v>
@@ -14161,7 +14159,7 @@
         <v>1557</v>
       </c>
       <c r="N139" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O139" t="s">
         <v>1558</v>
@@ -14170,7 +14168,7 @@
         <v>1559</v>
       </c>
       <c r="Q139" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R139" t="s">
         <v>1549</v>
@@ -14200,7 +14198,7 @@
         <v>1553</v>
       </c>
       <c r="E140" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F140" t="s">
         <v>1541</v>
@@ -14209,7 +14207,7 @@
         <v>27</v>
       </c>
       <c r="H140" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I140" t="s">
         <v>1561</v>
@@ -14225,7 +14223,7 @@
         <v>1564</v>
       </c>
       <c r="N140" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O140" t="s">
         <v>1565</v>
@@ -14234,7 +14232,7 @@
         <v>1566</v>
       </c>
       <c r="Q140" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R140" t="s">
         <v>1549</v>
@@ -14273,7 +14271,7 @@
         <v>27</v>
       </c>
       <c r="H141" t="s">
-        <v>104</v>
+        <v>54</v>
       </c>
       <c r="I141" t="s">
         <v>1570</v>
@@ -14289,7 +14287,7 @@
         <v>1573</v>
       </c>
       <c r="N141" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O141" t="s">
         <v>1574</v>
@@ -14298,7 +14296,7 @@
         <v>1575</v>
       </c>
       <c r="Q141" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="R141" t="s">
         <v>526</v>
@@ -14328,7 +14326,7 @@
         <v>1353</v>
       </c>
       <c r="E142" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="F142" t="s">
         <v>1577</v>
@@ -14337,7 +14335,7 @@
         <v>27</v>
       </c>
       <c r="H142" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="I142" t="s">
         <v>1578</v>
@@ -14353,7 +14351,7 @@
         <v>1581</v>
       </c>
       <c r="N142" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O142" t="s">
         <v>1582</v>
@@ -14362,7 +14360,7 @@
         <v>1583</v>
       </c>
       <c r="Q142" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="R142" t="s">
         <v>1584</v>
@@ -14397,7 +14395,7 @@
       </c>
       <c r="G143"/>
       <c r="H143" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I143" t="s">
         <v>1589</v>
@@ -14415,7 +14413,7 @@
         <v>1593</v>
       </c>
       <c r="N143" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="O143" t="s">
         <v>1594</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-06-15
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -80,6 +80,63 @@
     <t xml:space="preserve">Statut_Change_Date</t>
   </si>
   <si>
+    <t xml:space="preserve">26.7473</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fra.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dobler Loïc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EJPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arbeitsbedingungen beim Staatssekretariat für Migration: Ein Wendepunkt für das Bundespersonal?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conditions d'emploi au SEM : un tournant pour le personnel fédéral ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Selon une communication interne du SEM, une modification réglementaire entrant en vigueur prochainement autoriserait le maintien en CDD jusqu'à six ans d'employés fédéraux, les privant de la protection de l'art. 9 LPers. Alors que le SEM supprime déjà de nombreux postes, cette logique pourrait s'étendre à tout poste sans financement garanti.&amp;nbsp;&lt;br&gt;Le Conseil fédéral confirme-t-il cette modification et quelles garanties prévoit-il pour les employés concernés ?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Laut einer internen Mitteilung des Staatssekretariats für Migration&amp;nbsp;(SEM) soll eine demnächst in Kraft tretende Änderung der rechtlichen Bestimmungen es ermöglichen, Bundesangestellte bis zu sechs Jahre lang in einem befristeten Arbeitsverhältnis zu halten, wodurch ihnen der Schutz von Artikel&amp;nbsp;9 des Bundespersonalgesetzes entzogen würde. Das SEM streicht bereits zahlreiche Stellen. Aufgrund der vorgesehenen Änderung könnten alle Stellen ohne gesicherte Finanzierung gestrichen werden.&amp;nbsp;&lt;br&gt;Bestätigt der Bundesrat diese Änderung und welche Garantien sieht er für die betroffenen Arbeitnehmenden vor?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stellungnahme zum Vorstoss liegt vor / L’avis relatif à l’intervention est disponible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267473</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267473</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Titre uniquement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staatspolitik|Beschäftigung und Arbeit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique d'Etat|Emploi et travail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica nazionale|Occupazione e lavoro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-15</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.3411</t>
   </si>
   <si>
@@ -89,9 +146,6 @@
     <t xml:space="preserve">Crevoisier Crelier Mathilde</t>
   </si>
   <si>
-    <t xml:space="preserve">PS</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-03-20</t>
   </si>
   <si>
@@ -125,9 +179,6 @@
     <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263411</t>
   </si>
   <si>
-    <t xml:space="preserve">Titre uniquement</t>
-  </si>
-  <si>
     <t xml:space="preserve">Wirtschaft|Soziale Fragen|Medien und Kommunikation|Gesundheit</t>
   </si>
   <si>
@@ -210,57 +261,6 @@
   </si>
   <si>
     <t xml:space="preserve">Questioni sociali|Diritto civile|Protezione sociale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.7473</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fra.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dobler Loïc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EJPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arbeitsbedingungen beim Staatssekretariat für Migration: Ein Wendepunkt für das Bundespersonal?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conditions d'emploi au SEM : un tournant pour le personnel fédéral ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Selon une communication interne du SEM, une modification réglementaire entrant en vigueur prochainement autoriserait le maintien en CDD jusqu'à six ans d'employés fédéraux, les privant de la protection de l'art. 9 LPers. Alors que le SEM supprime déjà de nombreux postes, cette logique pourrait s'étendre à tout poste sans financement garanti.&amp;nbsp;&lt;br&gt;Le Conseil fédéral confirme-t-il cette modification et quelles garanties prévoit-il pour les employés concernés ?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Laut einer internen Mitteilung des Staatssekretariats für Migration&amp;nbsp;(SEM) soll eine demnächst in Kraft tretende Änderung der rechtlichen Bestimmungen es ermöglichen, Bundesangestellte bis zu sechs Jahre lang in einem befristeten Arbeitsverhältnis zu halten, wodurch ihnen der Schutz von Artikel&amp;nbsp;9 des Bundespersonalgesetzes entzogen würde. Das SEM streicht bereits zahlreiche Stellen. Aufgrund der vorgesehenen Änderung könnten alle Stellen ohne gesicherte Finanzierung gestrichen werden.&amp;nbsp;&lt;br&gt;Bestätigt der Bundesrat diese Änderung und welche Garantien sieht er für die betroffenen Arbeitnehmenden vor?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stellungnahme zum Vorstoss liegt vor / L’avis relatif à l’intervention est disponible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267473</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267473</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik|Beschäftigung und Arbeit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat|Emploi et travail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale|Occupazione e lavoro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-15</t>
   </si>
   <si>
     <t xml:space="preserve">26.7426</t>
@@ -5418,7 +5418,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>20263411</v>
+        <v>20267473</v>
       </c>
       <c r="B2" t="s">
         <v>22</v>
@@ -5447,230 +5447,228 @@
       <c r="J2" t="s">
         <v>30</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2"/>
+      <c r="L2" t="s">
         <v>31</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>32</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>33</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>34</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>35</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>36</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>37</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>38</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>39</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>40</v>
-      </c>
-      <c r="U2" t="s">
-        <v>41</v>
       </c>
       <c r="V2"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>20263628</v>
+        <v>20263411</v>
       </c>
       <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
         <v>42</v>
-      </c>
-      <c r="C3" t="s">
-        <v>23</v>
       </c>
       <c r="D3" t="s">
         <v>43</v>
       </c>
       <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
         <v>44</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>45</v>
       </c>
-      <c r="G3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3"/>
+      <c r="H3" t="s">
+        <v>46</v>
+      </c>
       <c r="I3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L3" t="s">
-        <v>49</v>
-      </c>
-      <c r="M3"/>
+        <v>50</v>
+      </c>
+      <c r="M3" t="s">
+        <v>51</v>
+      </c>
       <c r="N3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="O3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="P3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Q3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="S3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="T3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="U3" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="V3"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20263597</v>
+        <v>20263628</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="E4" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G4" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H4"/>
       <c r="I4" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="J4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="K4" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="L4" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="M4"/>
       <c r="N4" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="O4" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="P4" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>36</v>
+      </c>
+      <c r="R4" t="s">
+        <v>70</v>
+      </c>
+      <c r="S4" t="s">
+        <v>71</v>
+      </c>
+      <c r="T4" t="s">
+        <v>72</v>
+      </c>
+      <c r="U4" t="s">
         <v>62</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>37</v>
-      </c>
-      <c r="R4" t="s">
-        <v>63</v>
-      </c>
-      <c r="S4" t="s">
-        <v>64</v>
-      </c>
-      <c r="T4" t="s">
-        <v>65</v>
-      </c>
-      <c r="U4" t="s">
-        <v>58</v>
       </c>
       <c r="V4"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20267473</v>
+        <v>20263597</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" t="s">
+        <v>75</v>
+      </c>
+      <c r="G5" t="s">
+        <v>45</v>
+      </c>
+      <c r="H5"/>
+      <c r="I5" t="s">
+        <v>63</v>
+      </c>
+      <c r="J5" t="s">
+        <v>76</v>
+      </c>
+      <c r="K5" t="s">
+        <v>65</v>
+      </c>
+      <c r="L5" t="s">
+        <v>77</v>
+      </c>
+      <c r="M5"/>
+      <c r="N5" t="s">
         <v>67</v>
       </c>
-      <c r="D5" t="s">
-        <v>68</v>
-      </c>
-      <c r="E5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" t="s">
-        <v>69</v>
-      </c>
-      <c r="G5" t="s">
-        <v>70</v>
-      </c>
-      <c r="H5" t="s">
-        <v>71</v>
-      </c>
-      <c r="I5" t="s">
-        <v>72</v>
-      </c>
-      <c r="J5" t="s">
-        <v>73</v>
-      </c>
-      <c r="K5"/>
-      <c r="L5" t="s">
-        <v>74</v>
-      </c>
-      <c r="M5" t="s">
+      <c r="O5" t="s">
+        <v>78</v>
+      </c>
+      <c r="P5" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>36</v>
+      </c>
+      <c r="R5" t="s">
+        <v>80</v>
+      </c>
+      <c r="S5" t="s">
+        <v>81</v>
+      </c>
+      <c r="T5" t="s">
+        <v>82</v>
+      </c>
+      <c r="U5" t="s">
         <v>75</v>
       </c>
-      <c r="N5" t="s">
-        <v>76</v>
-      </c>
-      <c r="O5" t="s">
-        <v>77</v>
-      </c>
-      <c r="P5" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R5" t="s">
-        <v>79</v>
-      </c>
-      <c r="S5" t="s">
-        <v>80</v>
-      </c>
-      <c r="T5" t="s">
-        <v>81</v>
-      </c>
-      <c r="U5" t="s">
-        <v>82</v>
-      </c>
-      <c r="V5" t="s">
-        <v>82</v>
-      </c>
+      <c r="V5"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -5680,10 +5678,10 @@
         <v>83</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="E6" t="s">
         <v>25</v>
@@ -5692,7 +5690,7 @@
         <v>84</v>
       </c>
       <c r="G6" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H6" t="s">
         <v>85</v>
@@ -5720,7 +5718,7 @@
         <v>92</v>
       </c>
       <c r="Q6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R6" t="s">
         <v>93</v>
@@ -5732,7 +5730,7 @@
         <v>95</v>
       </c>
       <c r="U6" t="s">
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="V6"/>
     </row>
@@ -5744,7 +5742,7 @@
         <v>96</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s">
         <v>97</v>
@@ -5756,7 +5754,7 @@
         <v>84</v>
       </c>
       <c r="G7" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H7" t="s">
         <v>85</v>
@@ -5784,7 +5782,7 @@
         <v>104</v>
       </c>
       <c r="Q7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R7" t="s">
         <v>105</v>
@@ -5796,7 +5794,7 @@
         <v>107</v>
       </c>
       <c r="U7" t="s">
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="V7"/>
     </row>
@@ -5820,10 +5818,10 @@
         <v>111</v>
       </c>
       <c r="G8" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H8" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I8" t="s">
         <v>112</v>
@@ -5850,7 +5848,7 @@
         <v>118</v>
       </c>
       <c r="Q8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R8" t="s">
         <v>119</v>
@@ -5877,7 +5875,7 @@
         <v>109</v>
       </c>
       <c r="D9" t="s">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
         <v>25</v>
@@ -5886,24 +5884,24 @@
         <v>124</v>
       </c>
       <c r="G9" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H9"/>
       <c r="I9" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="J9" t="s">
         <v>125</v>
       </c>
       <c r="K9" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="L9" t="s">
         <v>126</v>
       </c>
       <c r="M9"/>
       <c r="N9" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="O9" t="s">
         <v>127</v>
@@ -5912,7 +5910,7 @@
         <v>128</v>
       </c>
       <c r="Q9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R9" t="s">
         <v>129</v>
@@ -5939,7 +5937,7 @@
         <v>109</v>
       </c>
       <c r="D10" t="s">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="E10" t="s">
         <v>25</v>
@@ -5948,7 +5946,7 @@
         <v>124</v>
       </c>
       <c r="G10" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H10"/>
       <c r="I10" t="s">
@@ -5958,14 +5956,14 @@
         <v>134</v>
       </c>
       <c r="K10" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="L10" t="s">
         <v>135</v>
       </c>
       <c r="M10"/>
       <c r="N10" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="O10" t="s">
         <v>136</v>
@@ -5974,7 +5972,7 @@
         <v>137</v>
       </c>
       <c r="Q10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R10" t="s">
         <v>138</v>
@@ -5998,7 +5996,7 @@
         <v>141</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
         <v>142</v>
@@ -6010,7 +6008,7 @@
         <v>124</v>
       </c>
       <c r="G11" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H11"/>
       <c r="I11" t="s">
@@ -6027,7 +6025,7 @@
         <v>145</v>
       </c>
       <c r="N11" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="O11" t="s">
         <v>146</v>
@@ -6063,16 +6061,16 @@
         <v>109</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F12" t="s">
         <v>153</v>
       </c>
       <c r="G12" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H12" t="s">
         <v>154</v>
@@ -6102,7 +6100,7 @@
         <v>161</v>
       </c>
       <c r="Q12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R12" t="s">
         <v>162</v>
@@ -6126,7 +6124,7 @@
         <v>165</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
         <v>166</v>
@@ -6136,7 +6134,7 @@
         <v>167</v>
       </c>
       <c r="G13" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H13" t="s">
         <v>168</v>
@@ -6157,7 +6155,7 @@
         <v>173</v>
       </c>
       <c r="N13" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O13" t="s">
         <v>174</v>
@@ -6202,7 +6200,7 @@
         <v>184</v>
       </c>
       <c r="G14" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H14" t="s">
         <v>85</v>
@@ -6223,7 +6221,7 @@
         <v>189</v>
       </c>
       <c r="N14" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O14" t="s">
         <v>190</v>
@@ -6256,22 +6254,22 @@
         <v>196</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D15" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="E15" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F15" t="s">
         <v>197</v>
       </c>
       <c r="G15" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H15" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I15" t="s">
         <v>198</v>
@@ -6298,7 +6296,7 @@
         <v>205</v>
       </c>
       <c r="Q15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R15" t="s">
         <v>206</v>
@@ -6322,7 +6320,7 @@
         <v>210</v>
       </c>
       <c r="C16" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D16" t="s">
         <v>211</v>
@@ -6331,10 +6329,10 @@
         <v>183</v>
       </c>
       <c r="F16" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="G16" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H16" t="s">
         <v>85</v>
@@ -6355,7 +6353,7 @@
         <v>216</v>
       </c>
       <c r="N16" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O16" t="s">
         <v>217</v>
@@ -6400,7 +6398,7 @@
         <v>184</v>
       </c>
       <c r="G17" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H17" t="s">
         <v>154</v>
@@ -6421,7 +6419,7 @@
         <v>229</v>
       </c>
       <c r="N17" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O17" t="s">
         <v>230</v>
@@ -6454,7 +6452,7 @@
         <v>232</v>
       </c>
       <c r="C18" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D18" t="s">
         <v>233</v>
@@ -6464,10 +6462,10 @@
         <v>153</v>
       </c>
       <c r="G18" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H18" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I18" t="s">
         <v>143</v>
@@ -6485,7 +6483,7 @@
         <v>145</v>
       </c>
       <c r="N18" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O18" t="s">
         <v>237</v>
@@ -6518,17 +6516,17 @@
         <v>239</v>
       </c>
       <c r="C19" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D19" t="s">
         <v>240</v>
       </c>
       <c r="E19"/>
       <c r="F19" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="G19" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H19" t="s">
         <v>168</v>
@@ -6549,7 +6547,7 @@
         <v>245</v>
       </c>
       <c r="N19" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O19" t="s">
         <v>246</v>
@@ -6591,10 +6589,10 @@
         <v>98</v>
       </c>
       <c r="F20" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="G20" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H20" t="s">
         <v>154</v>
@@ -6615,7 +6613,7 @@
         <v>257</v>
       </c>
       <c r="N20" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O20" t="s">
         <v>258</v>
@@ -6624,7 +6622,7 @@
         <v>259</v>
       </c>
       <c r="Q20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R20" t="s">
         <v>260</v>
@@ -6660,7 +6658,7 @@
         <v>265</v>
       </c>
       <c r="G21" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H21" t="s">
         <v>266</v>
@@ -6681,7 +6679,7 @@
         <v>271</v>
       </c>
       <c r="N21" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O21" t="s">
         <v>272</v>
@@ -6714,7 +6712,7 @@
         <v>277</v>
       </c>
       <c r="C22" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D22" t="s">
         <v>278</v>
@@ -6726,10 +6724,10 @@
         <v>153</v>
       </c>
       <c r="G22" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H22" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I22" t="s">
         <v>279</v>
@@ -6747,7 +6745,7 @@
         <v>283</v>
       </c>
       <c r="N22" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O22" t="s">
         <v>284</v>
@@ -6792,7 +6790,7 @@
         <v>292</v>
       </c>
       <c r="G23" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H23" t="s">
         <v>154</v>
@@ -6813,7 +6811,7 @@
         <v>297</v>
       </c>
       <c r="N23" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O23" t="s">
         <v>298</v>
@@ -6846,22 +6844,22 @@
         <v>300</v>
       </c>
       <c r="C24" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D24" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="E24" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F24" t="s">
         <v>301</v>
       </c>
       <c r="G24" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H24" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I24" t="s">
         <v>302</v>
@@ -6879,7 +6877,7 @@
         <v>306</v>
       </c>
       <c r="N24" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="O24" t="s">
         <v>307</v>
@@ -6888,7 +6886,7 @@
         <v>308</v>
       </c>
       <c r="Q24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R24" t="s">
         <v>309</v>
@@ -6912,7 +6910,7 @@
         <v>313</v>
       </c>
       <c r="C25" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D25" t="s">
         <v>110</v>
@@ -6924,7 +6922,7 @@
         <v>314</v>
       </c>
       <c r="G25" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H25" t="s">
         <v>85</v>
@@ -6952,7 +6950,7 @@
         <v>320</v>
       </c>
       <c r="Q25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R25" t="s">
         <v>321</v>
@@ -6976,7 +6974,7 @@
         <v>325</v>
       </c>
       <c r="C26" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D26" t="s">
         <v>326</v>
@@ -6988,10 +6986,10 @@
         <v>292</v>
       </c>
       <c r="G26" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H26" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I26" t="s">
         <v>328</v>
@@ -7049,7 +7047,7 @@
       </c>
       <c r="G27"/>
       <c r="H27" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I27" t="s">
         <v>340</v>
@@ -7072,7 +7070,7 @@
         <v>345</v>
       </c>
       <c r="Q27" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R27" t="s">
         <v>274</v>
@@ -7096,7 +7094,7 @@
         <v>346</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D28" t="s">
         <v>211</v>
@@ -7108,10 +7106,10 @@
         <v>347</v>
       </c>
       <c r="G28" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H28" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I28" t="s">
         <v>348</v>
@@ -7160,7 +7158,7 @@
         <v>357</v>
       </c>
       <c r="C29" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D29" t="s">
         <v>358</v>
@@ -7170,7 +7168,7 @@
         <v>359</v>
       </c>
       <c r="G29" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H29" t="s">
         <v>168</v>
@@ -7236,7 +7234,7 @@
         <v>301</v>
       </c>
       <c r="G30" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H30" t="s">
         <v>168</v>
@@ -7257,7 +7255,7 @@
         <v>377</v>
       </c>
       <c r="N30" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O30" t="s">
         <v>378</v>
@@ -7302,7 +7300,7 @@
         <v>301</v>
       </c>
       <c r="G31" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H31" t="s">
         <v>154</v>
@@ -7323,7 +7321,7 @@
         <v>389</v>
       </c>
       <c r="N31" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O31" t="s">
         <v>390</v>
@@ -7356,19 +7354,19 @@
         <v>395</v>
       </c>
       <c r="C32" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D32" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="E32" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F32" t="s">
         <v>396</v>
       </c>
       <c r="G32" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H32" t="s">
         <v>397</v>
@@ -7398,7 +7396,7 @@
         <v>405</v>
       </c>
       <c r="Q32" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R32" t="s">
         <v>406</v>
@@ -7422,22 +7420,22 @@
         <v>409</v>
       </c>
       <c r="C33" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D33" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="E33" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F33" t="s">
         <v>396</v>
       </c>
       <c r="G33" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H33" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I33" t="s">
         <v>410</v>
@@ -7464,7 +7462,7 @@
         <v>417</v>
       </c>
       <c r="Q33" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R33" t="s">
         <v>418</v>
@@ -7494,13 +7492,13 @@
         <v>422</v>
       </c>
       <c r="E34" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F34" t="s">
         <v>423</v>
       </c>
       <c r="G34" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H34" t="s">
         <v>168</v>
@@ -7554,7 +7552,7 @@
         <v>434</v>
       </c>
       <c r="C35" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D35" t="s">
         <v>278</v>
@@ -7566,7 +7564,7 @@
         <v>111</v>
       </c>
       <c r="G35" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H35" t="s">
         <v>168</v>
@@ -7587,7 +7585,7 @@
         <v>439</v>
       </c>
       <c r="N35" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O35" t="s">
         <v>440</v>
@@ -7620,7 +7618,7 @@
         <v>442</v>
       </c>
       <c r="C36" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D36" t="s">
         <v>443</v>
@@ -7632,7 +7630,7 @@
         <v>444</v>
       </c>
       <c r="G36" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H36" t="s">
         <v>397</v>
@@ -7684,7 +7682,7 @@
         <v>454</v>
       </c>
       <c r="C37" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D37" t="s">
         <v>264</v>
@@ -7696,10 +7694,10 @@
         <v>444</v>
       </c>
       <c r="G37" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H37" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I37" t="s">
         <v>455</v>
@@ -7748,7 +7746,7 @@
         <v>461</v>
       </c>
       <c r="C38" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D38" t="s">
         <v>462</v>
@@ -7758,10 +7756,10 @@
         <v>463</v>
       </c>
       <c r="G38" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H38" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I38" t="s">
         <v>464</v>
@@ -7812,7 +7810,7 @@
         <v>474</v>
       </c>
       <c r="C39" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D39" t="s">
         <v>475</v>
@@ -7824,7 +7822,7 @@
         <v>476</v>
       </c>
       <c r="G39" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H39" t="s">
         <v>168</v>
@@ -7878,7 +7876,7 @@
         <v>487</v>
       </c>
       <c r="C40" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D40" t="s">
         <v>488</v>
@@ -7890,7 +7888,7 @@
         <v>476</v>
       </c>
       <c r="G40" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H40" t="s">
         <v>168</v>
@@ -7911,7 +7909,7 @@
         <v>493</v>
       </c>
       <c r="N40" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O40" t="s">
         <v>494</v>
@@ -7956,7 +7954,7 @@
         <v>476</v>
       </c>
       <c r="G41" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H41" t="s">
         <v>154</v>
@@ -7977,7 +7975,7 @@
         <v>501</v>
       </c>
       <c r="N41" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O41" t="s">
         <v>502</v>
@@ -8010,10 +8008,10 @@
         <v>504</v>
       </c>
       <c r="C42" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D42" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="E42" t="s">
         <v>25</v>
@@ -8022,10 +8020,10 @@
         <v>476</v>
       </c>
       <c r="G42" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H42" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I42" t="s">
         <v>505</v>
@@ -8052,7 +8050,7 @@
         <v>511</v>
       </c>
       <c r="Q42" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R42" t="s">
         <v>512</v>
@@ -8082,13 +8080,13 @@
         <v>516</v>
       </c>
       <c r="E43" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F43" t="s">
         <v>517</v>
       </c>
       <c r="G43" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H43" t="s">
         <v>168</v>
@@ -8145,16 +8143,16 @@
         <v>109</v>
       </c>
       <c r="D44" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="E44" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F44" t="s">
         <v>526</v>
       </c>
       <c r="G44" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H44" t="s">
         <v>85</v>
@@ -8220,7 +8218,7 @@
         <v>526</v>
       </c>
       <c r="G45" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H45" t="s">
         <v>397</v>
@@ -8241,7 +8239,7 @@
         <v>543</v>
       </c>
       <c r="N45" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O45" t="s">
         <v>544</v>
@@ -8280,13 +8278,13 @@
         <v>550</v>
       </c>
       <c r="E46" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F46" t="s">
         <v>551</v>
       </c>
       <c r="G46" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H46" t="s">
         <v>168</v>
@@ -8352,7 +8350,7 @@
         <v>564</v>
       </c>
       <c r="G47" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H47" t="s">
         <v>168</v>
@@ -8382,7 +8380,7 @@
         <v>572</v>
       </c>
       <c r="Q47" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R47" t="s">
         <v>573</v>
@@ -8406,7 +8404,7 @@
         <v>576</v>
       </c>
       <c r="C48" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D48" t="s">
         <v>577</v>
@@ -8418,7 +8416,7 @@
         <v>578</v>
       </c>
       <c r="G48" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H48" t="s">
         <v>154</v>
@@ -8439,7 +8437,7 @@
         <v>583</v>
       </c>
       <c r="N48" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O48" t="s">
         <v>584</v>
@@ -8472,7 +8470,7 @@
         <v>589</v>
       </c>
       <c r="C49" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D49" t="s">
         <v>590</v>
@@ -8484,7 +8482,7 @@
         <v>578</v>
       </c>
       <c r="G49" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H49" t="s">
         <v>168</v>
@@ -8536,19 +8534,19 @@
         <v>598</v>
       </c>
       <c r="C50" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D50" t="s">
         <v>599</v>
       </c>
       <c r="E50" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F50" t="s">
         <v>578</v>
       </c>
       <c r="G50" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H50" t="s">
         <v>85</v>
@@ -8600,7 +8598,7 @@
         <v>609</v>
       </c>
       <c r="C51" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D51" t="s">
         <v>538</v>
@@ -8612,10 +8610,10 @@
         <v>610</v>
       </c>
       <c r="G51" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H51" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I51" t="s">
         <v>611</v>
@@ -8676,7 +8674,7 @@
         <v>622</v>
       </c>
       <c r="G52" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H52" t="s">
         <v>397</v>
@@ -8697,7 +8695,7 @@
         <v>627</v>
       </c>
       <c r="N52" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O52" t="s">
         <v>628</v>
@@ -8730,7 +8728,7 @@
         <v>633</v>
       </c>
       <c r="C53" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D53" t="s">
         <v>621</v>
@@ -8742,7 +8740,7 @@
         <v>622</v>
       </c>
       <c r="G53" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H53" t="s">
         <v>397</v>
@@ -8862,7 +8860,7 @@
         <v>657</v>
       </c>
       <c r="G55" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H55" t="s">
         <v>154</v>
@@ -8883,7 +8881,7 @@
         <v>662</v>
       </c>
       <c r="N55" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O55" t="s">
         <v>663</v>
@@ -8928,7 +8926,7 @@
         <v>657</v>
       </c>
       <c r="G56" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H56" t="s">
         <v>154</v>
@@ -8949,7 +8947,7 @@
         <v>674</v>
       </c>
       <c r="N56" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O56" t="s">
         <v>675</v>
@@ -8982,19 +8980,19 @@
         <v>680</v>
       </c>
       <c r="C57" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D57" t="s">
         <v>681</v>
       </c>
       <c r="E57" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F57" t="s">
         <v>657</v>
       </c>
       <c r="G57" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H57" t="s">
         <v>168</v>
@@ -9048,7 +9046,7 @@
         <v>693</v>
       </c>
       <c r="C58" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D58" t="s">
         <v>240</v>
@@ -9058,7 +9056,7 @@
         <v>694</v>
       </c>
       <c r="G58" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H58" t="s">
         <v>168</v>
@@ -9079,7 +9077,7 @@
         <v>699</v>
       </c>
       <c r="N58" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O58" t="s">
         <v>700</v>
@@ -9124,10 +9122,10 @@
         <v>694</v>
       </c>
       <c r="G59" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H59" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I59" t="s">
         <v>707</v>
@@ -9190,7 +9188,7 @@
         <v>719</v>
       </c>
       <c r="G60" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H60" t="s">
         <v>154</v>
@@ -9244,7 +9242,7 @@
         <v>727</v>
       </c>
       <c r="C61" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D61" t="s">
         <v>728</v>
@@ -9254,7 +9252,7 @@
         <v>719</v>
       </c>
       <c r="G61" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H61" t="s">
         <v>154</v>
@@ -9320,7 +9318,7 @@
         <v>719</v>
       </c>
       <c r="G62" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H62" t="s">
         <v>154</v>
@@ -9341,7 +9339,7 @@
         <v>744</v>
       </c>
       <c r="N62" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O62" t="s">
         <v>745</v>
@@ -9386,7 +9384,7 @@
         <v>752</v>
       </c>
       <c r="G63" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H63" t="s">
         <v>154</v>
@@ -9440,7 +9438,7 @@
         <v>760</v>
       </c>
       <c r="C64" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D64" t="s">
         <v>761</v>
@@ -9452,7 +9450,7 @@
         <v>762</v>
       </c>
       <c r="G64" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H64" t="s">
         <v>154</v>
@@ -9473,7 +9471,7 @@
         <v>767</v>
       </c>
       <c r="N64" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O64" t="s">
         <v>768</v>
@@ -9506,7 +9504,7 @@
         <v>770</v>
       </c>
       <c r="C65" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D65" t="s">
         <v>771</v>
@@ -9518,7 +9516,7 @@
         <v>773</v>
       </c>
       <c r="G65" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H65" t="s">
         <v>168</v>
@@ -9539,7 +9537,7 @@
         <v>778</v>
       </c>
       <c r="N65" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O65" t="s">
         <v>779</v>
@@ -9572,7 +9570,7 @@
         <v>784</v>
       </c>
       <c r="C66" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D66" t="s">
         <v>538</v>
@@ -9584,7 +9582,7 @@
         <v>773</v>
       </c>
       <c r="G66" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H66" t="s">
         <v>168</v>
@@ -9605,7 +9603,7 @@
         <v>789</v>
       </c>
       <c r="N66" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O66" t="s">
         <v>790</v>
@@ -9638,7 +9636,7 @@
         <v>795</v>
       </c>
       <c r="C67" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D67" t="s">
         <v>358</v>
@@ -9648,7 +9646,7 @@
         <v>796</v>
       </c>
       <c r="G67" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H67" t="s">
         <v>168</v>
@@ -9702,19 +9700,19 @@
         <v>804</v>
       </c>
       <c r="C68" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D68" t="s">
         <v>805</v>
       </c>
       <c r="E68" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F68" t="s">
         <v>806</v>
       </c>
       <c r="G68" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H68" t="s">
         <v>807</v>
@@ -9774,16 +9772,16 @@
         <v>819</v>
       </c>
       <c r="E69" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F69" t="s">
         <v>806</v>
       </c>
       <c r="G69" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H69" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I69" t="s">
         <v>820</v>
@@ -9801,7 +9799,7 @@
         <v>824</v>
       </c>
       <c r="N69" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O69" t="s">
         <v>825</v>
@@ -9846,7 +9844,7 @@
         <v>806</v>
       </c>
       <c r="G70" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H70" t="s">
         <v>154</v>
@@ -9867,7 +9865,7 @@
         <v>836</v>
       </c>
       <c r="N70" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O70" t="s">
         <v>837</v>
@@ -9900,22 +9898,22 @@
         <v>839</v>
       </c>
       <c r="C71" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D71" t="s">
         <v>840</v>
       </c>
       <c r="E71" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F71" t="s">
         <v>841</v>
       </c>
       <c r="G71" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H71" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I71" t="s">
         <v>842</v>
@@ -9966,19 +9964,19 @@
         <v>852</v>
       </c>
       <c r="C72" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D72" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="E72" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F72" t="s">
         <v>841</v>
       </c>
       <c r="G72" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H72" t="s">
         <v>168</v>
@@ -10038,13 +10036,13 @@
         <v>422</v>
       </c>
       <c r="E73" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F73" t="s">
         <v>861</v>
       </c>
       <c r="G73" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H73" t="s">
         <v>154</v>
@@ -10110,10 +10108,10 @@
         <v>873</v>
       </c>
       <c r="G74" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H74" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I74" t="s">
         <v>874</v>
@@ -10131,7 +10129,7 @@
         <v>878</v>
       </c>
       <c r="N74" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O74" t="s">
         <v>879</v>
@@ -10193,7 +10191,7 @@
         <v>891</v>
       </c>
       <c r="N75" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="O75" t="s">
         <v>892</v>
@@ -10231,7 +10229,7 @@
       </c>
       <c r="G76"/>
       <c r="H76" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I76" t="s">
         <v>648</v>
@@ -10286,10 +10284,10 @@
         <v>903</v>
       </c>
       <c r="G77" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H77" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I77" t="s">
         <v>904</v>
@@ -10307,7 +10305,7 @@
         <v>908</v>
       </c>
       <c r="N77" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="O77" t="s">
         <v>909</v>
@@ -10352,7 +10350,7 @@
         <v>915</v>
       </c>
       <c r="G78" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H78" t="s">
         <v>154</v>
@@ -10418,7 +10416,7 @@
         <v>915</v>
       </c>
       <c r="G79" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H79" t="s">
         <v>168</v>
@@ -10439,7 +10437,7 @@
         <v>931</v>
       </c>
       <c r="N79" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O79" t="s">
         <v>932</v>
@@ -10478,13 +10476,13 @@
         <v>938</v>
       </c>
       <c r="E80" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F80" t="s">
         <v>915</v>
       </c>
       <c r="G80" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H80" t="s">
         <v>266</v>
@@ -10538,7 +10536,7 @@
         <v>949</v>
       </c>
       <c r="C81" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D81" t="s">
         <v>488</v>
@@ -10550,7 +10548,7 @@
         <v>915</v>
       </c>
       <c r="G81" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H81" t="s">
         <v>168</v>
@@ -10604,7 +10602,7 @@
         <v>960</v>
       </c>
       <c r="C82" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D82" t="s">
         <v>961</v>
@@ -10616,10 +10614,10 @@
         <v>915</v>
       </c>
       <c r="G82" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H82" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I82" t="s">
         <v>962</v>
@@ -10637,7 +10635,7 @@
         <v>966</v>
       </c>
       <c r="N82" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O82" t="s">
         <v>967</v>
@@ -10682,7 +10680,7 @@
         <v>915</v>
       </c>
       <c r="G83" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H83" t="s">
         <v>168</v>
@@ -10703,7 +10701,7 @@
         <v>978</v>
       </c>
       <c r="N83" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O83" t="s">
         <v>979</v>
@@ -10736,19 +10734,19 @@
         <v>984</v>
       </c>
       <c r="C84" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D84" t="s">
         <v>599</v>
       </c>
       <c r="E84" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F84" t="s">
         <v>985</v>
       </c>
       <c r="G84" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H84" t="s">
         <v>154</v>
@@ -10814,7 +10812,7 @@
         <v>985</v>
       </c>
       <c r="G85" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H85" t="s">
         <v>154</v>
@@ -10835,7 +10833,7 @@
         <v>1002</v>
       </c>
       <c r="N85" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O85" t="s">
         <v>1003</v>
@@ -10924,7 +10922,7 @@
         <v>1017</v>
       </c>
       <c r="C87" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D87" t="s">
         <v>97</v>
@@ -10936,7 +10934,7 @@
         <v>1018</v>
       </c>
       <c r="G87" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H87" t="s">
         <v>168</v>
@@ -10990,7 +10988,7 @@
         <v>1025</v>
       </c>
       <c r="C88" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D88" t="s">
         <v>1026</v>
@@ -11002,10 +11000,10 @@
         <v>1027</v>
       </c>
       <c r="G88" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H88" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I88" t="s">
         <v>1028</v>
@@ -11054,7 +11052,7 @@
         <v>1037</v>
       </c>
       <c r="C89" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D89" t="s">
         <v>1038</v>
@@ -11066,7 +11064,7 @@
         <v>1039</v>
       </c>
       <c r="G89" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H89" t="s">
         <v>154</v>
@@ -11127,7 +11125,7 @@
       </c>
       <c r="G90"/>
       <c r="H90" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I90" t="s">
         <v>1048</v>
@@ -11150,7 +11148,7 @@
         <v>1052</v>
       </c>
       <c r="Q90" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R90" t="s">
         <v>1053</v>
@@ -11185,7 +11183,7 @@
       </c>
       <c r="G91"/>
       <c r="H91" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I91" t="s">
         <v>1058</v>
@@ -11203,7 +11201,7 @@
         <v>1062</v>
       </c>
       <c r="N91" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="O91" t="s">
         <v>1063</v>
@@ -11298,7 +11296,7 @@
         <v>1080</v>
       </c>
       <c r="C93" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D93" t="s">
         <v>771</v>
@@ -11310,10 +11308,10 @@
         <v>1081</v>
       </c>
       <c r="G93" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H93" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I93" t="s">
         <v>1082</v>
@@ -11331,7 +11329,7 @@
         <v>1086</v>
       </c>
       <c r="N93" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O93" t="s">
         <v>1087</v>
@@ -11364,19 +11362,19 @@
         <v>1092</v>
       </c>
       <c r="C94" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D94" t="s">
         <v>1093</v>
       </c>
       <c r="E94" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F94" t="s">
         <v>1094</v>
       </c>
       <c r="G94" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H94" t="s">
         <v>85</v>
@@ -11397,7 +11395,7 @@
         <v>1099</v>
       </c>
       <c r="N94" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O94" t="s">
         <v>1100</v>
@@ -11442,7 +11440,7 @@
         <v>1094</v>
       </c>
       <c r="G95" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H95" t="s">
         <v>154</v>
@@ -11496,7 +11494,7 @@
         <v>1114</v>
       </c>
       <c r="C96" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D96" t="s">
         <v>1115</v>
@@ -11508,7 +11506,7 @@
         <v>1094</v>
       </c>
       <c r="G96" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H96" t="s">
         <v>168</v>
@@ -11568,13 +11566,13 @@
         <v>1127</v>
       </c>
       <c r="E97" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F97" t="s">
         <v>1094</v>
       </c>
       <c r="G97" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H97" t="s">
         <v>85</v>
@@ -11595,7 +11593,7 @@
         <v>1132</v>
       </c>
       <c r="N97" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O97" t="s">
         <v>1133</v>
@@ -11628,7 +11626,7 @@
         <v>1135</v>
       </c>
       <c r="C98" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D98" t="s">
         <v>1136</v>
@@ -11640,7 +11638,7 @@
         <v>1137</v>
       </c>
       <c r="G98" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H98" t="s">
         <v>85</v>
@@ -11661,7 +11659,7 @@
         <v>1142</v>
       </c>
       <c r="N98" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O98" t="s">
         <v>1143</v>
@@ -11694,7 +11692,7 @@
         <v>1145</v>
       </c>
       <c r="C99" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D99" t="s">
         <v>538</v>
@@ -11706,10 +11704,10 @@
         <v>1146</v>
       </c>
       <c r="G99" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H99" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I99" t="s">
         <v>1147</v>
@@ -11770,7 +11768,7 @@
         <v>1154</v>
       </c>
       <c r="G100" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H100" t="s">
         <v>154</v>
@@ -11824,19 +11822,19 @@
         <v>1162</v>
       </c>
       <c r="C101" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D101" t="s">
         <v>1127</v>
       </c>
       <c r="E101" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F101" t="s">
         <v>1163</v>
       </c>
       <c r="G101" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H101" t="s">
         <v>154</v>
@@ -11888,7 +11886,7 @@
         <v>1170</v>
       </c>
       <c r="C102" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D102" t="s">
         <v>538</v>
@@ -11900,10 +11898,10 @@
         <v>1163</v>
       </c>
       <c r="G102" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H102" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I102" t="s">
         <v>1171</v>
@@ -11952,7 +11950,7 @@
         <v>1177</v>
       </c>
       <c r="C103" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D103" t="s">
         <v>538</v>
@@ -11964,10 +11962,10 @@
         <v>1163</v>
       </c>
       <c r="G103" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H103" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I103" t="s">
         <v>1171</v>
@@ -12016,7 +12014,7 @@
         <v>1182</v>
       </c>
       <c r="C104" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D104" t="s">
         <v>538</v>
@@ -12028,10 +12026,10 @@
         <v>1163</v>
       </c>
       <c r="G104" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H104" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I104" t="s">
         <v>1171</v>
@@ -12092,10 +12090,10 @@
         <v>1188</v>
       </c>
       <c r="G105" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H105" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I105" t="s">
         <v>1189</v>
@@ -12113,7 +12111,7 @@
         <v>1193</v>
       </c>
       <c r="N105" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O105" t="s">
         <v>1194</v>
@@ -12152,13 +12150,13 @@
         <v>681</v>
       </c>
       <c r="E106" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F106" t="s">
         <v>1200</v>
       </c>
       <c r="G106" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H106" t="s">
         <v>168</v>
@@ -12224,7 +12222,7 @@
         <v>1200</v>
       </c>
       <c r="G107" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H107" t="s">
         <v>154</v>
@@ -12245,7 +12243,7 @@
         <v>1214</v>
       </c>
       <c r="N107" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O107" t="s">
         <v>1215</v>
@@ -12290,7 +12288,7 @@
         <v>1200</v>
       </c>
       <c r="G108" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H108" t="s">
         <v>168</v>
@@ -12311,7 +12309,7 @@
         <v>1226</v>
       </c>
       <c r="N108" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O108" t="s">
         <v>1227</v>
@@ -12373,7 +12371,7 @@
         <v>1238</v>
       </c>
       <c r="N109" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="O109" t="s">
         <v>1239</v>
@@ -12406,19 +12404,19 @@
         <v>1244</v>
       </c>
       <c r="C110" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D110" t="s">
         <v>516</v>
       </c>
       <c r="E110" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F110" t="s">
         <v>1233</v>
       </c>
       <c r="G110" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H110" t="s">
         <v>85</v>
@@ -12439,7 +12437,7 @@
         <v>1249</v>
       </c>
       <c r="N110" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O110" t="s">
         <v>1250</v>
@@ -12472,7 +12470,7 @@
         <v>1255</v>
       </c>
       <c r="C111" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D111" t="s">
         <v>1256</v>
@@ -12484,10 +12482,10 @@
         <v>1233</v>
       </c>
       <c r="G111" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H111" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I111" t="s">
         <v>1257</v>
@@ -12505,7 +12503,7 @@
         <v>1261</v>
       </c>
       <c r="N111" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O111" t="s">
         <v>1262</v>
@@ -12550,10 +12548,10 @@
         <v>1233</v>
       </c>
       <c r="G112" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H112" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I112" t="s">
         <v>1269</v>
@@ -12604,7 +12602,7 @@
         <v>1276</v>
       </c>
       <c r="C113" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D113" t="s">
         <v>669</v>
@@ -12616,7 +12614,7 @@
         <v>1233</v>
       </c>
       <c r="G113" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H113" t="s">
         <v>154</v>
@@ -12637,7 +12635,7 @@
         <v>1281</v>
       </c>
       <c r="N113" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O113" t="s">
         <v>1282</v>
@@ -12670,7 +12668,7 @@
         <v>1287</v>
       </c>
       <c r="C114" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D114" t="s">
         <v>621</v>
@@ -12682,7 +12680,7 @@
         <v>1233</v>
       </c>
       <c r="G114" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H114" t="s">
         <v>168</v>
@@ -12748,7 +12746,7 @@
         <v>1300</v>
       </c>
       <c r="G115" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H115" t="s">
         <v>154</v>
@@ -12802,7 +12800,7 @@
         <v>1308</v>
       </c>
       <c r="C116" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D116" t="s">
         <v>488</v>
@@ -12814,7 +12812,7 @@
         <v>1309</v>
       </c>
       <c r="G116" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H116" t="s">
         <v>168</v>
@@ -12868,7 +12866,7 @@
         <v>1317</v>
       </c>
       <c r="C117" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D117" t="s">
         <v>1318</v>
@@ -12880,7 +12878,7 @@
         <v>1319</v>
       </c>
       <c r="G117" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H117" t="s">
         <v>168</v>
@@ -12932,7 +12930,7 @@
         <v>1326</v>
       </c>
       <c r="C118" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D118" t="s">
         <v>1327</v>
@@ -12944,7 +12942,7 @@
         <v>1319</v>
       </c>
       <c r="G118" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H118" t="s">
         <v>154</v>
@@ -12996,7 +12994,7 @@
         <v>1337</v>
       </c>
       <c r="C119" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D119" t="s">
         <v>224</v>
@@ -13008,7 +13006,7 @@
         <v>1338</v>
       </c>
       <c r="G119" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H119" t="s">
         <v>154</v>
@@ -13029,7 +13027,7 @@
         <v>1343</v>
       </c>
       <c r="N119" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="O119" t="s">
         <v>1344</v>
@@ -13071,7 +13069,7 @@
       </c>
       <c r="G120"/>
       <c r="H120" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I120" t="s">
         <v>1348</v>
@@ -13094,7 +13092,7 @@
         <v>1353</v>
       </c>
       <c r="Q120" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R120" t="s">
         <v>1354</v>
@@ -13129,7 +13127,7 @@
       </c>
       <c r="G121"/>
       <c r="H121" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="I121" t="s">
         <v>1359</v>
@@ -13192,7 +13190,7 @@
         <v>1371</v>
       </c>
       <c r="G122" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H122" t="s">
         <v>154</v>
@@ -13258,10 +13256,10 @@
         <v>1384</v>
       </c>
       <c r="G123" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H123" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I123" t="s">
         <v>1385</v>
@@ -13315,7 +13313,7 @@
         <v>109</v>
       </c>
       <c r="D124" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="E124" t="s">
         <v>25</v>
@@ -13324,7 +13322,7 @@
         <v>1384</v>
       </c>
       <c r="G124" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H124" t="s">
         <v>154</v>
@@ -13378,22 +13376,22 @@
         <v>1403</v>
       </c>
       <c r="C125" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D125" t="s">
         <v>422</v>
       </c>
       <c r="E125" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F125" t="s">
         <v>1404</v>
       </c>
       <c r="G125" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H125" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I125" t="s">
         <v>1405</v>
@@ -13444,19 +13442,19 @@
         <v>1412</v>
       </c>
       <c r="C126" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D126" t="s">
         <v>1413</v>
       </c>
       <c r="E126" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F126" t="s">
         <v>1404</v>
       </c>
       <c r="G126" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H126" t="s">
         <v>154</v>
@@ -13510,7 +13508,7 @@
         <v>1424</v>
       </c>
       <c r="C127" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D127" t="s">
         <v>1425</v>
@@ -13522,7 +13520,7 @@
         <v>1404</v>
       </c>
       <c r="G127" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H127" t="s">
         <v>85</v>
@@ -13588,7 +13586,7 @@
         <v>1404</v>
       </c>
       <c r="G128" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H128" t="s">
         <v>154</v>
@@ -13648,16 +13646,16 @@
         <v>1413</v>
       </c>
       <c r="E129" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F129" t="s">
         <v>1404</v>
       </c>
       <c r="G129" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H129" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I129" t="s">
         <v>1449</v>
@@ -13720,7 +13718,7 @@
         <v>1404</v>
       </c>
       <c r="G130" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H130" t="s">
         <v>168</v>
@@ -13780,13 +13778,13 @@
         <v>1471</v>
       </c>
       <c r="E131" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F131" t="s">
         <v>1472</v>
       </c>
       <c r="G131" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H131" t="s">
         <v>168</v>
@@ -13852,7 +13850,7 @@
         <v>1481</v>
       </c>
       <c r="G132" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H132" t="s">
         <v>168</v>
@@ -13918,10 +13916,10 @@
         <v>1491</v>
       </c>
       <c r="G133" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H133" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I133" t="s">
         <v>1492</v>
@@ -13972,7 +13970,7 @@
         <v>1499</v>
       </c>
       <c r="C134" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D134" t="s">
         <v>1500</v>
@@ -13984,10 +13982,10 @@
         <v>1501</v>
       </c>
       <c r="G134" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H134" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I134" t="s">
         <v>1502</v>
@@ -14038,7 +14036,7 @@
         <v>1509</v>
       </c>
       <c r="C135" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D135" t="s">
         <v>621</v>
@@ -14050,7 +14048,7 @@
         <v>1501</v>
       </c>
       <c r="G135" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H135" t="s">
         <v>154</v>
@@ -14102,7 +14100,7 @@
         <v>1516</v>
       </c>
       <c r="C136" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D136" t="s">
         <v>224</v>
@@ -14114,7 +14112,7 @@
         <v>1517</v>
       </c>
       <c r="G136" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H136" t="s">
         <v>154</v>
@@ -14166,7 +14164,7 @@
         <v>1524</v>
       </c>
       <c r="C137" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D137" t="s">
         <v>166</v>
@@ -14176,10 +14174,10 @@
         <v>1525</v>
       </c>
       <c r="G137" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H137" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I137" t="s">
         <v>1526</v>
@@ -14242,7 +14240,7 @@
         <v>1537</v>
       </c>
       <c r="G138" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H138" t="s">
         <v>154</v>
@@ -14296,7 +14294,7 @@
         <v>1548</v>
       </c>
       <c r="C139" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D139" t="s">
         <v>656</v>
@@ -14308,10 +14306,10 @@
         <v>1537</v>
       </c>
       <c r="G139" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H139" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I139" t="s">
         <v>1549</v>
@@ -14362,7 +14360,7 @@
         <v>1559</v>
       </c>
       <c r="C140" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D140" t="s">
         <v>1560</v>
@@ -14374,7 +14372,7 @@
         <v>1561</v>
       </c>
       <c r="G140" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H140" t="s">
         <v>807</v>
@@ -14428,7 +14426,7 @@
         <v>1572</v>
       </c>
       <c r="C141" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D141" t="s">
         <v>961</v>
@@ -14440,7 +14438,7 @@
         <v>1561</v>
       </c>
       <c r="G141" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H141" t="s">
         <v>807</v>
@@ -14506,7 +14504,7 @@
         <v>1580</v>
       </c>
       <c r="G142" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H142" t="s">
         <v>85</v>
@@ -14563,16 +14561,16 @@
         <v>109</v>
       </c>
       <c r="D143" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="E143" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F143" t="s">
         <v>1589</v>
       </c>
       <c r="G143" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H143" t="s">
         <v>154</v>
@@ -14638,7 +14636,7 @@
         <v>1601</v>
       </c>
       <c r="G144" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H144" t="s">
         <v>154</v>
@@ -14692,7 +14690,7 @@
         <v>1612</v>
       </c>
       <c r="C145" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D145" t="s">
         <v>1613</v>
@@ -14704,7 +14702,7 @@
         <v>1601</v>
       </c>
       <c r="G145" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H145" t="s">
         <v>154</v>
@@ -14756,7 +14754,7 @@
         <v>1620</v>
       </c>
       <c r="C146" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D146" t="s">
         <v>1613</v>
@@ -14768,7 +14766,7 @@
         <v>1601</v>
       </c>
       <c r="G146" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H146" t="s">
         <v>154</v>
@@ -14820,7 +14818,7 @@
         <v>1627</v>
       </c>
       <c r="C147" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D147" t="s">
         <v>1628</v>
@@ -14832,7 +14830,7 @@
         <v>1629</v>
       </c>
       <c r="G147" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H147" t="s">
         <v>154</v>
@@ -14884,22 +14882,22 @@
         <v>1636</v>
       </c>
       <c r="C148" t="s">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D148" t="s">
         <v>1413</v>
       </c>
       <c r="E148" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F148" t="s">
         <v>1637</v>
       </c>
       <c r="G148" t="s">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="H148" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="I148" t="s">
         <v>1638</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-07-01
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -458,10 +458,10 @@
     <t xml:space="preserve">VBS</t>
   </si>
   <si>
-    <t xml:space="preserve">Cybersécurité et souveraineté numérique. Doter la Suisse d’une feuille de route nationale de transition vers la cryptographie post-quantique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cibersicurezza e sovranità digitale: dotare la Svizzera di una tabella di marcia nazionale per la transizione verso la crittografia post-quantistica</t>
+    <t xml:space="preserve">Cybersécurité et souveraineté numérique. Doter la Suisse d'une feuille de route nationale de transition vers la cryptographie post-quantique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cibersicurezza e sovranità digitale. Dotare la Svizzera di una tabella di marcia nazionale per la transizione verso la crittografia post-quantistica</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé d’élaborer, en collaboration avec les cantons, les hautes écoles, les instituts de recherche, les autorités de surveillance sectorielles et le secteur privé, une feuille de route nationale pour la transition de la Suisse vers la cryptographie post-quantique. Cette feuille de route doit garantir la protection durable des données et des communications sensibles, la résilience des infrastructures critiques, la validité à long terme des signatures et des documents électroniques, l’interopérabilité internationale des systèmes suisses et la compétitivité des entreprises actives sur les marchés internationaux. Elle doit en particulier :&lt;/p&gt;&lt;ol style="list-style-type:lower-alpha;"&gt;&lt;li&gt;&lt;strong&gt;établir, d’ici à fin 2027 au plus tard, une stratégie nationale de migration — c’est-à-dire de remplacement progressif des algorithmes vulnérables — fondée sur les risques,&amp;nbsp;&lt;/strong&gt;comprenant un inventaire des usages cryptographiques critiques, une cartographie des dépendances, y compris à l’égard des fournisseurs étrangers, et le lancement de projets pilotes pour les cas d’usage présentant un risque élevé ou une longue durée de confidentialité ;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;fixer des jalons coordonnés avec les calendriers internationaux pertinents,&amp;nbsp;&lt;/strong&gt;notamment la migration prioritaire des cas d’usage à haut risque d’ici à fin 2030 et la transition progressive des autres systèmes critiques ou sensibles d’ici à fin 2035, sous réserve de la maturité des standards, de l’interopérabilité et de la proportionnalité des mesures ;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;désigner les responsabilités de pilotage et de coordination au sein de l’administration fédérale,&amp;nbsp;&lt;/strong&gt;en s’appuyant en particulier sur l’Office fédéral de la cybersécurité (OFCS, anciennement NCSC), l’Office fédéral de l’informatique et de la télécommunication (OFIT) et les autorités sectorielles compétentes, sans créer de structures redondantes, et présenter au Parlement un rapport biennal sur l’état d’avancement ;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;définir les exigences minimales applicables aux infrastructures critiques, aux systèmes d’information de la Confédération et aux fournisseurs de prestations numériques critiques,&amp;nbsp;&lt;/strong&gt;notamment en matière d’inventaire cryptographique standardisé et interopérable — fondé, lorsque cela est approprié, sur des formats reconnus tels que le Cryptographic Bill of Materials (CBOM) —, de crypto-agilité, de capacité de mise à jour et de gestion sécurisée des dépendances fournisseurs, ces inventaires étant traités comme des informations sensibles de sécurité à accès restreint et non destinées à publication détaillée ;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;intégrer des exigences de préparation à la cryptographie post-quantique dans les marchés publics fédéraux et dans les contrats fournisseurs&amp;nbsp;&lt;/strong&gt;pour les produits et services numériques dont la durée de vie, la criticité ou la durée de confidentialité attendue dépasse 2030 ;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;garantir la résilience quantique de la signature électronique et de l’archivage à long terme,&amp;nbsp;&lt;/strong&gt;afin de préserver la validité durable des signatures, certificats, horodatages, actes authentiques, dossiers médicaux, registres publics et archives, en cohérence avec les travaux de la Swiss Government PKI ;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;assurer la cohérence avec les cadres internationaux applicables,&amp;nbsp;&lt;/strong&gt;en particulier la feuille de route coordonnée adoptée par le NIS Cooperation Group de l’Union européenne le 11 juin 2025, ainsi que les exigences du Cyber Resilience Act applicables dès le 11 décembre 2027 aux produits placés sur le marché européen ;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;examiner les adaptations légales ou réglementaires nécessaires,&amp;nbsp;&lt;/strong&gt;notamment dans le cadre de la législation sur la sécurité de l’information, de l’ordonnance sur la cybersécurité, des prescriptions de marchés publics et des réglementations sectorielles applicables ;&lt;/li&gt;&lt;li&gt;&lt;strong&gt;prévoir des mesures de soutien proportionnées pour les cantons, les PME, les hautes écoles et les entreprises suisses,&amp;nbsp;&lt;/strong&gt;notamment par des lignes directrices, des modèles d’inventaire, des projets pilotes, des tests d’interopérabilité et la mobilisation des compétences nationales, dans une logique de souveraineté technologique cohérente avec l’objectif de la motion 24.3209.&lt;/li&gt;&lt;/ol&gt;&lt;p&gt;La feuille de route respecte les principes de neutralité technologique, d’ouverture des standards, de sécurité par conception et de proportionnalité économique — les obligations étant graduées selon le risque, la criticité, la durée de confidentialité des données et la durée de vie des systèmes. Conformément à la tradition suisse de conditions-cadres favorables plutôt que de politique industrielle sélective, elle ne vise pas à privilégier un fournisseur ou une technologie, mais à fixer les exigences de sécurité applicables aux infrastructures de l’État. Les informations sensibles contenues dans les inventaires cryptographiques sont protégées.&lt;/p&gt;</t>
@@ -668,10 +668,10 @@
     <t xml:space="preserve">26.3564</t>
   </si>
   <si>
-    <t xml:space="preserve">Arztzeugnisse für Kurzabwesenheiten: unnötige Kosten für die obligatorische Krankenversicherung?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Certificats médicaux pour courtes absences : un coût inutile pour la LAMal ?</t>
+    <t xml:space="preserve">Arztzeugnisse für Kurzabwesenheiten. Unnötige Kosten für die obligatorische Krankenversicherung?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Certificats médicaux pour courtes absences. Un coût inutile pour la LAMal ?</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;De nombreux employeurs exigent un certificat médical dès le premier ou le deuxième jour d'absence de leurs employées et employés, y compris pour des maladies bénignes de courte durée. Cette pratique contraint les salarié·e·s à consulter un médecin ou une médecin non pas pour des raisons thérapeutiques, mais pour satisfaire une exigence administrative. Ces consultations sont remboursées par la LAMal, après déduction de la franchise et de la quote-part. Elles génèrent donc des coûts réels pour les salarié·e·s et pour le système de santé, sans aucune valeur médicale ajoutée.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Le Code des obligations ne fixe aucun délai minimal avant qu'un employeur puisse exiger un tel certificat, laissant une liberté totale sur ce point. Certaines conventions collectives de travail prévoient des règles plus protectrices, mais elles ne couvrent pas l'ensemble des travailleuses et travailleurs.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Si un employeur juge nécessaire d'exiger une attestation médicale avant tout délai raisonnable, il est logique que les frais qui en découlent lui incombent. Il n'appartient pas à l'assurance obligatoire des soins, financée par l'ensemble des assuré·e·s, de couvrir des dépenses qui résultent d'une exigence administrative privée. De leur côté, les salarié·e·s concerné·e·s contribuent financièrement au travers de leur franchise et quote-part. À l'heure où la maîtrise des coûts de la santé est une priorité politique affichée, cette source de dépenses évitable mérite d'être examinée.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Je pose les questions suivantes au Conseil fédéral :&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;ol&gt;&lt;li&gt;Dispose-t-il de données sur le nombre de consultations médicales annuelles dont le seul motif est la délivrance d'un certificat exigé par un employeur ou une employeuse pour une courte absence ?&lt;/li&gt;&lt;li&gt;Quel est le coût estimé de ces consultations pour la LAMal ?&lt;/li&gt;&lt;li&gt;Est-il prêt à examiner une réglementation fixant un délai minimal avant qu'un employeur puisse exiger un certificat médical ?&lt;/li&gt;&lt;li&gt;Est-il prêt à examiner une modification légale permettant de mettre les frais de ces consultations à la charge de l'employeur ou de l'employeuse qui les exige, plutôt qu'à celle de l'assurance obligatoire des soins ?&lt;/li&gt;&lt;/ol&gt;</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-07-13
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -212,13 +212,13 @@
     <t xml:space="preserve">2026-06-19</t>
   </si>
   <si>
-    <t xml:space="preserve">Für eine neue Finanzierungsquelle für grosse öffentliche Ausgabenposten: eine befristete Solidaritätsabgabe auf den Zahlungsverkehr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pour une nouvelle source de financement des grands dossiers en charge des collectivités publiques: une contribution de solidarité temporaire prélevée sur les mouvements financiers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Una nuova fonte di finanziamento per i grandi progetti a carico delle collettività pubbliche: un contributo di solidarietà temporaneo prelevato sui movimenti finanziari</t>
+    <t xml:space="preserve">Für eine neue Finanzierungsquelle für grosse öffentliche Ausgabenposten. Eine befristete Solidaritätsabgabe auf den Zahlungsverkehr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pour une nouvelle source de financement des grands dossiers en charge des collectivités publiques. Une contribution de solidarité temporaire prélevée sur les mouvements financiers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una nuova fonte di finanziamento per i grandi progetti a carico delle collettività pubbliche. Un contributo di solidarietà temporaneo prelevato sui movimenti finanziari</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;La Confédération doit faire face à des défis financiers importants que les sources de financements actuelles n'arriveront sans doute pas à financer. Il y a les impôts, les taxes, la TVA notamment; mais celles-ci ne suffisent plus à financer des grands projets dont le pays a besoin. Il s'agit notamment de l'AVS, des infrastructures de transport, de la sécurité du pays (armée notamment), la prévention des dangers naturels liés au changement climatique (tâche partagée avec les cantons et les communes). Mes questions portent sur la création temporaire (10 ans) d'une forme de contribution de solidarité pour les "grands travaux" des 3 niveaux politiques suisses.&amp;nbsp;&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Je demande au Conseil fédéral de bien vouloir répondre aux questions suivantes:&lt;/p&gt;&lt;p&gt;1. Le Conseil fédéral a-t-il déjà mené des réflexions quant à la mise en œuvre de nouvelles sources de financement, si oui lesquelles?&lt;/p&gt;&lt;p&gt;2. Sachant que le nombre annuel des mouvements financiers ( et non les transactions financières) s'élève à environ 5560 mio pour un volume financier d'environ CHF 17'530 milliards ( pour 2025), le prélèvement de 1 pour-mille sur ces transactions pourrait rapporter environ CHF 17,5 milliards/an, que ces montants pourraient être versés dans 3 fonds spécifiques (prévoyance sociale, sécurité, dangers naturels) gérés par la Confédération ou la BNS, le Conseil fédéral est-il prêt à examiner rapidement cette nouvelle source de financement et, cas échéant de proposer un projet au Parlement?&lt;/p&gt;</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-07-31
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -7468,7 +7468,9 @@
         <v>391</v>
       </c>
       <c r="D31"/>
-      <c r="E31"/>
+      <c r="E31" t="s">
+        <v>25</v>
+      </c>
       <c r="F31" t="s">
         <v>392</v>
       </c>
@@ -9250,7 +9252,7 @@
         <v>697</v>
       </c>
       <c r="N58" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="O58" t="s">
         <v>698</v>
@@ -11548,7 +11550,9 @@
         <v>391</v>
       </c>
       <c r="D94"/>
-      <c r="E94"/>
+      <c r="E94" t="s">
+        <v>25</v>
+      </c>
       <c r="F94" t="s">
         <v>1093</v>
       </c>
@@ -13492,7 +13496,9 @@
         <v>391</v>
       </c>
       <c r="D124"/>
-      <c r="E124"/>
+      <c r="E124" t="s">
+        <v>25</v>
+      </c>
       <c r="F124" t="s">
         <v>1393</v>
       </c>

</xml_diff>

<commit_message>
Update parliament data - 2026-09-01
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -5672,9 +5672,7 @@
       <c r="U2" t="s">
         <v>41</v>
       </c>
-      <c r="V2" t="s">
-        <v>41</v>
-      </c>
+      <c r="V2"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -5740,9 +5738,7 @@
       <c r="U3" t="s">
         <v>41</v>
       </c>
-      <c r="V3" t="s">
-        <v>41</v>
-      </c>
+      <c r="V3"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -5808,9 +5804,7 @@
       <c r="U4" t="s">
         <v>41</v>
       </c>
-      <c r="V4" t="s">
-        <v>41</v>
-      </c>
+      <c r="V4"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -5876,9 +5870,7 @@
       <c r="U5" t="s">
         <v>41</v>
       </c>
-      <c r="V5" t="s">
-        <v>41</v>
-      </c>
+      <c r="V5"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -7593,7 +7585,9 @@
         <v>407</v>
       </c>
       <c r="D32"/>
-      <c r="E32"/>
+      <c r="E32" t="s">
+        <v>153</v>
+      </c>
       <c r="F32" t="s">
         <v>408</v>
       </c>
@@ -11673,7 +11667,9 @@
         <v>407</v>
       </c>
       <c r="D95"/>
-      <c r="E95"/>
+      <c r="E95" t="s">
+        <v>153</v>
+      </c>
       <c r="F95" t="s">
         <v>1110</v>
       </c>
@@ -13617,7 +13613,9 @@
         <v>407</v>
       </c>
       <c r="D125"/>
-      <c r="E125"/>
+      <c r="E125" t="s">
+        <v>153</v>
+      </c>
       <c r="F125" t="s">
         <v>1410</v>
       </c>

</xml_diff>

<commit_message>
Update parliament data - 2026-09-03
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_Jura.xlsx
+++ b/Objets_parlementaires_Jura.xlsx
@@ -797,9 +797,6 @@
     <t xml:space="preserve">&lt;p&gt;Viele Arbeitgeber verlangen von ihren Angestellten bei Krankheit bereits ab dem ersten oder zweiten Abwesenheitstag ein Arztzeugnis, auch bei leichter, kurzer Krankheit. Diese Praxis zwingt die Arbeitnehmerinnen und Arbeitnehmer dazu, einen Arzt oder eine Ärztin nicht wegen eines medizinischen Problems aufzusuchen, sondern um einer administrativen Vorgabe des Arbeitgebers nachzukommen. Diese Konsultationen werden nach Abzug der Franchise und des Selbstbehalts von der obligatorischen Krankenversicherung vergütet. Sie generieren somit tatsächliche Kosten für die Arbeitnehmerinnen und Arbeitnehmer sowie für das Gesundheitssystem, ohne dass sie einen medizinischen Mehrwert bieten.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Das Obligationenrecht legt keine Mindestfrist fest, nach deren Ablauf ein Arbeitgeber ein Arztzeugnis verlangen kann – diesbezüglich herrscht völlige Freiheit. Einige Gesamtarbeitsverträge sehen strengere Vorschriften zum Schutz der Arbeitnehmerinnen und Arbeitnehmer vor, doch diese gelten nicht für die Gesamtheit der Arbeitnehmerinnen und Arbeitnehmer.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Wenn ein Arbeitgeber es für notwendig erachtet, bereits vor Ablauf einer angemessenen Frist ein Arztzeugnis zu verlangen, wäre es nur folgerichtig, wenn die damit verbundenen Kosten zu seinen Lasten gingen. Es ist nicht Aufgabe der obligatorischen Krankenpflegeversicherung, die von allen Versicherten finanziert wird, Kosten zu übernehmen, die sich aus einer privaten administrativen Forderung ergeben. Die betroffenen Arbeitnehmerinnen und Arbeitnehmer leisten ihrerseits einen finanziellen Beitrag in Form ihrer Franchise und ihres Selbstbehalts. In einer Zeit, in der die Kostendämpfung im Gesundheitswesen eine erklärte politische Priorität ist, sollte dieser vermeidbare Kostenfaktor genauer unter die Lupe genommen werden.&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;p&gt;Ich bitte den Bundesrat, folgende Fragen zu beantworten:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;ol&gt;&lt;li&gt;Verfügt der Bundesrat über Daten zur Anzahl der jährlichen Arztbesuche, deren einziger Grund die Ausstellung eines Arztzeugnisses ist, die ein Arbeitgeber für eine Kurzabwesenheit verlangt?&lt;/li&gt;&lt;li&gt;Wie hoch werden die Kosten dieser Konsultationen für die obligatorische Krankenversicherung geschätzt?&lt;/li&gt;&lt;li&gt;Ist der Bundesrat bereit, eine Regelung zu prüfen, die eine Mindestfrist festlegt, bevor ein Arbeitgeber ein Arztzeugnis verlangen darf?&lt;/li&gt;&lt;li&gt;Ist der Bundesrat bereit, eine Gesetzesänderung zu prüfen, die es ermöglicht, die Kosten für diese Konsultationen dem entsprechenden Arbeitgeber anzulasten, anstatt der obligatorischen Krankenversicherung?&lt;/li&gt;&lt;/ol&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">Eingereicht / Déposé</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263564</t>
   </si>
   <si>
@@ -813,6 +810,9 @@
   </si>
   <si>
     <t xml:space="preserve">Occupazione e lavoro|Diritto civile|Salute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-03</t>
   </si>
   <si>
     <t xml:space="preserve">26.3121</t>
@@ -6765,30 +6765,32 @@
         <v>260</v>
       </c>
       <c r="N19" t="s">
+        <v>53</v>
+      </c>
+      <c r="O19" t="s">
         <v>261</v>
       </c>
-      <c r="O19" t="s">
+      <c r="P19" t="s">
         <v>262</v>
-      </c>
-      <c r="P19" t="s">
-        <v>263</v>
       </c>
       <c r="Q19" t="s">
         <v>56</v>
       </c>
       <c r="R19" t="s">
+        <v>263</v>
+      </c>
+      <c r="S19" t="s">
         <v>264</v>
       </c>
-      <c r="S19" t="s">
+      <c r="T19" t="s">
         <v>265</v>
       </c>
-      <c r="T19" t="s">
+      <c r="U19" t="s">
         <v>266</v>
       </c>
-      <c r="U19" t="s">
-        <v>115</v>
-      </c>
-      <c r="V19"/>
+      <c r="V19" t="s">
+        <v>266</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">

</xml_diff>